<commit_message>
benchmarks: update results, sync report docx, and mirror READMEs
</commit_message>
<xml_diff>
--- a/Programming_Benchmark_Report.xlsx
+++ b/Programming_Benchmark_Report.xlsx
@@ -6642,26 +6642,26 @@
         </is>
       </c>
       <c r="E20" s="11" t="n">
-        <v>7045.07</v>
+        <v>9324.9</v>
       </c>
       <c r="F20" s="11" t="n">
-        <v>4028.49</v>
-      </c>
-      <c r="G20" s="12">
+        <v>10087.07</v>
+      </c>
+      <c r="G20" s="17">
         <f>IF(E20&gt;0, (F20-E20)/E20, 0)</f>
         <v/>
       </c>
       <c r="H20" s="11" t="n">
-        <v>14.41</v>
+        <v>2.31</v>
       </c>
       <c r="I20" s="11" t="n">
-        <v>5.03</v>
+        <v>2.42</v>
       </c>
       <c r="J20" s="11" t="n">
-        <v>0</v>
+        <v>4.11</v>
       </c>
       <c r="K20" s="11" t="n">
-        <v>6.93</v>
+        <v>3.4</v>
       </c>
       <c r="L20" s="13" t="n">
         <v>0</v>
@@ -6692,26 +6692,26 @@
         </is>
       </c>
       <c r="E21" s="16" t="n">
-        <v>7297.44</v>
+        <v>10604.52</v>
       </c>
       <c r="F21" s="16" t="n">
-        <v>4605.9</v>
-      </c>
-      <c r="G21" s="12">
+        <v>14308.05</v>
+      </c>
+      <c r="G21" s="17">
         <f>IF(E21&gt;0, (F21-E21)/E21, 0)</f>
         <v/>
       </c>
       <c r="H21" s="16" t="n">
-        <v>13.94</v>
+        <v>2.07</v>
       </c>
       <c r="I21" s="16" t="n">
-        <v>4.36</v>
+        <v>1.65</v>
       </c>
       <c r="J21" s="16" t="n">
-        <v>0</v>
+        <v>3.83</v>
       </c>
       <c r="K21" s="16" t="n">
-        <v>6.36</v>
+        <v>2.83</v>
       </c>
       <c r="L21" s="18" t="n">
         <v>0</v>
@@ -6742,26 +6742,26 @@
         </is>
       </c>
       <c r="E22" s="11" t="n">
-        <v>4506.78</v>
+        <v>12581.47</v>
       </c>
       <c r="F22" s="11" t="n">
-        <v>3599.8</v>
-      </c>
-      <c r="G22" s="12">
+        <v>18730.75</v>
+      </c>
+      <c r="G22" s="17">
         <f>IF(E22&gt;0, (F22-E22)/E22, 0)</f>
         <v/>
       </c>
       <c r="H22" s="11" t="n">
-        <v>23.91</v>
+        <v>2.27</v>
       </c>
       <c r="I22" s="11" t="n">
-        <v>5.89</v>
+        <v>1.41</v>
       </c>
       <c r="J22" s="11" t="n">
-        <v>0</v>
+        <v>4.5</v>
       </c>
       <c r="K22" s="11" t="n">
-        <v>13.05</v>
+        <v>3.34</v>
       </c>
       <c r="L22" s="13" t="n">
         <v>0</v>
@@ -6792,26 +6792,26 @@
         </is>
       </c>
       <c r="E23" s="16" t="n">
-        <v>7123.85</v>
+        <v>9833.5</v>
       </c>
       <c r="F23" s="16" t="n">
-        <v>5057.31</v>
-      </c>
-      <c r="G23" s="12">
+        <v>12905.17</v>
+      </c>
+      <c r="G23" s="17">
         <f>IF(E23&gt;0, (F23-E23)/E23, 0)</f>
         <v/>
       </c>
       <c r="H23" s="16" t="n">
-        <v>14.05</v>
+        <v>2.81</v>
       </c>
       <c r="I23" s="16" t="n">
-        <v>3.97</v>
+        <v>1.74</v>
       </c>
       <c r="J23" s="16" t="n">
-        <v>0</v>
+        <v>4.21</v>
       </c>
       <c r="K23" s="16" t="n">
-        <v>5.25</v>
+        <v>3.29</v>
       </c>
       <c r="L23" s="18" t="n">
         <v>0</v>
@@ -6842,26 +6842,26 @@
         </is>
       </c>
       <c r="E24" s="11" t="n">
-        <v>5708.88</v>
+        <v>9774.09</v>
       </c>
       <c r="F24" s="11" t="n">
-        <v>4642.41</v>
-      </c>
-      <c r="G24" s="12">
+        <v>12851.51</v>
+      </c>
+      <c r="G24" s="17">
         <f>IF(E24&gt;0, (F24-E24)/E24, 0)</f>
         <v/>
       </c>
       <c r="H24" s="11" t="n">
-        <v>17.63</v>
+        <v>2.21</v>
       </c>
       <c r="I24" s="11" t="n">
-        <v>4.34</v>
+        <v>1.79</v>
       </c>
       <c r="J24" s="11" t="n">
-        <v>0</v>
+        <v>4.14</v>
       </c>
       <c r="K24" s="11" t="n">
-        <v>6.44</v>
+        <v>3.49</v>
       </c>
       <c r="L24" s="13" t="n">
         <v>0</v>
@@ -6899,7 +6899,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L85"/>
+  <dimension ref="A1:L97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="112" customWidth="1" min="1" max="1"/>
@@ -8969,12 +8969,12 @@
     <row r="78" ht="20" customHeight="1">
       <c r="A78" s="9" t="inlineStr">
         <is>
-          <t>Min</t>
+          <t>POC</t>
         </is>
       </c>
       <c r="B78" s="9" t="inlineStr">
         <is>
-          <t>100 conn (2 threads)</t>
+          <t>20 conn (2 threads)</t>
         </is>
       </c>
       <c r="C78" s="19" t="inlineStr">
@@ -8983,26 +8983,26 @@
         </is>
       </c>
       <c r="D78" s="11" t="n">
-        <v>7045.07</v>
+        <v>9324.9</v>
       </c>
       <c r="E78" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="F78" s="12">
+        <v>10087.07</v>
+      </c>
+      <c r="F78" s="17">
         <f>IF(D78&gt;0, (E78-D78)/D78, 0)</f>
         <v/>
       </c>
       <c r="G78" s="11" t="n">
-        <v>14.41</v>
+        <v>2.31</v>
       </c>
       <c r="H78" s="11" t="n">
-        <v>0</v>
+        <v>2.42</v>
       </c>
       <c r="I78" s="11" t="n">
-        <v>0</v>
+        <v>4.11</v>
       </c>
       <c r="J78" s="11" t="n">
-        <v>0</v>
+        <v>3.4</v>
       </c>
       <c r="K78" s="13" t="n">
         <v>0</v>
@@ -9014,12 +9014,12 @@
     <row r="79" ht="20" customHeight="1">
       <c r="A79" s="14" t="inlineStr">
         <is>
-          <t>Min</t>
+          <t>POC</t>
         </is>
       </c>
       <c r="B79" s="14" t="inlineStr">
         <is>
-          <t>100 conn (2 threads)</t>
+          <t>20 conn (2 threads)</t>
         </is>
       </c>
       <c r="C79" s="20" t="inlineStr">
@@ -9028,26 +9028,26 @@
         </is>
       </c>
       <c r="D79" s="16" t="n">
-        <v>4836.32</v>
+        <v>5274.29</v>
       </c>
       <c r="E79" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="F79" s="12">
+        <v>5556.55</v>
+      </c>
+      <c r="F79" s="17">
         <f>IF(D79&gt;0, (E79-D79)/D79, 0)</f>
         <v/>
       </c>
       <c r="G79" s="16" t="n">
-        <v>20.87</v>
+        <v>3.97</v>
       </c>
       <c r="H79" s="16" t="n">
-        <v>0</v>
+        <v>3.85</v>
       </c>
       <c r="I79" s="16" t="n">
-        <v>0</v>
+        <v>6.42</v>
       </c>
       <c r="J79" s="16" t="n">
-        <v>0</v>
+        <v>5.75</v>
       </c>
       <c r="K79" s="18" t="n">
         <v>0</v>
@@ -9059,12 +9059,12 @@
     <row r="80" ht="20" customHeight="1">
       <c r="A80" s="9" t="inlineStr">
         <is>
-          <t>Min</t>
+          <t>POC</t>
         </is>
       </c>
       <c r="B80" s="9" t="inlineStr">
         <is>
-          <t>100 conn (2 threads)</t>
+          <t>20 conn (2 threads)</t>
         </is>
       </c>
       <c r="C80" s="19" t="inlineStr">
@@ -9073,26 +9073,26 @@
         </is>
       </c>
       <c r="D80" s="11" t="n">
-        <v>4395.94</v>
+        <v>4457.83</v>
       </c>
       <c r="E80" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="F80" s="12">
+        <v>4852.79</v>
+      </c>
+      <c r="F80" s="17">
         <f>IF(D80&gt;0, (E80-D80)/D80, 0)</f>
         <v/>
       </c>
       <c r="G80" s="11" t="n">
-        <v>22.75</v>
+        <v>4.66</v>
       </c>
       <c r="H80" s="11" t="n">
-        <v>0</v>
+        <v>4.31</v>
       </c>
       <c r="I80" s="11" t="n">
-        <v>0</v>
+        <v>7.44</v>
       </c>
       <c r="J80" s="11" t="n">
-        <v>0</v>
+        <v>6.31</v>
       </c>
       <c r="K80" s="13" t="n">
         <v>0</v>
@@ -9104,12 +9104,12 @@
     <row r="81" ht="20" customHeight="1">
       <c r="A81" s="14" t="inlineStr">
         <is>
-          <t>Min</t>
+          <t>POC</t>
         </is>
       </c>
       <c r="B81" s="14" t="inlineStr">
         <is>
-          <t>100 conn (2 threads)</t>
+          <t>20 conn (2 threads)</t>
         </is>
       </c>
       <c r="C81" s="20" t="inlineStr">
@@ -9118,26 +9118,26 @@
         </is>
       </c>
       <c r="D81" s="16" t="n">
-        <v>3684.23</v>
+        <v>3360.52</v>
       </c>
       <c r="E81" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="F81" s="12">
+        <v>3651.39</v>
+      </c>
+      <c r="F81" s="17">
         <f>IF(D81&gt;0, (E81-D81)/D81, 0)</f>
         <v/>
       </c>
       <c r="G81" s="16" t="n">
-        <v>27.18</v>
+        <v>6.45</v>
       </c>
       <c r="H81" s="16" t="n">
-        <v>0</v>
+        <v>5.65</v>
       </c>
       <c r="I81" s="16" t="n">
-        <v>0</v>
+        <v>9.93</v>
       </c>
       <c r="J81" s="16" t="n">
-        <v>0</v>
+        <v>8.33</v>
       </c>
       <c r="K81" s="18" t="n">
         <v>0</v>
@@ -9149,12 +9149,12 @@
     <row r="82" ht="20" customHeight="1">
       <c r="A82" s="9" t="inlineStr">
         <is>
-          <t>POC</t>
+          <t>Small</t>
         </is>
       </c>
       <c r="B82" s="9" t="inlineStr">
         <is>
-          <t>20 conn (2 threads)</t>
+          <t>100 conn (4 threads)</t>
         </is>
       </c>
       <c r="C82" s="19" t="inlineStr">
@@ -9163,26 +9163,26 @@
         </is>
       </c>
       <c r="D82" s="11" t="n">
-        <v>0</v>
+        <v>8698.629999999999</v>
       </c>
       <c r="E82" s="11" t="n">
-        <v>4028.49</v>
-      </c>
-      <c r="F82" s="21">
+        <v>13839.32</v>
+      </c>
+      <c r="F82" s="17">
         <f>IF(D82&gt;0, (E82-D82)/D82, 0)</f>
         <v/>
       </c>
       <c r="G82" s="11" t="n">
-        <v>0</v>
+        <v>22.51</v>
       </c>
       <c r="H82" s="11" t="n">
-        <v>5.03</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="I82" s="11" t="n">
-        <v>0</v>
+        <v>96.52</v>
       </c>
       <c r="J82" s="11" t="n">
-        <v>6.93</v>
+        <v>20.59</v>
       </c>
       <c r="K82" s="13" t="n">
         <v>0</v>
@@ -9194,12 +9194,12 @@
     <row r="83" ht="20" customHeight="1">
       <c r="A83" s="14" t="inlineStr">
         <is>
-          <t>POC</t>
+          <t>Small</t>
         </is>
       </c>
       <c r="B83" s="14" t="inlineStr">
         <is>
-          <t>20 conn (2 threads)</t>
+          <t>100 conn (4 threads)</t>
         </is>
       </c>
       <c r="C83" s="20" t="inlineStr">
@@ -9208,26 +9208,26 @@
         </is>
       </c>
       <c r="D83" s="16" t="n">
-        <v>0</v>
+        <v>6258.85</v>
       </c>
       <c r="E83" s="16" t="n">
-        <v>3065.06</v>
-      </c>
-      <c r="F83" s="22">
+        <v>7563.67</v>
+      </c>
+      <c r="F83" s="17">
         <f>IF(D83&gt;0, (E83-D83)/D83, 0)</f>
         <v/>
       </c>
       <c r="G83" s="16" t="n">
-        <v>0</v>
+        <v>18.06</v>
       </c>
       <c r="H83" s="16" t="n">
-        <v>6.56</v>
+        <v>14.51</v>
       </c>
       <c r="I83" s="16" t="n">
-        <v>0</v>
+        <v>44.39</v>
       </c>
       <c r="J83" s="16" t="n">
-        <v>9.029999999999999</v>
+        <v>32.41</v>
       </c>
       <c r="K83" s="18" t="n">
         <v>0</v>
@@ -9239,12 +9239,12 @@
     <row r="84" ht="20" customHeight="1">
       <c r="A84" s="9" t="inlineStr">
         <is>
-          <t>POC</t>
+          <t>Small</t>
         </is>
       </c>
       <c r="B84" s="9" t="inlineStr">
         <is>
-          <t>20 conn (2 threads)</t>
+          <t>100 conn (4 threads)</t>
         </is>
       </c>
       <c r="C84" s="19" t="inlineStr">
@@ -9253,26 +9253,26 @@
         </is>
       </c>
       <c r="D84" s="11" t="n">
-        <v>0</v>
+        <v>5410.04</v>
       </c>
       <c r="E84" s="11" t="n">
-        <v>2754.16</v>
-      </c>
-      <c r="F84" s="21">
+        <v>6236.25</v>
+      </c>
+      <c r="F84" s="17">
         <f>IF(D84&gt;0, (E84-D84)/D84, 0)</f>
         <v/>
       </c>
       <c r="G84" s="11" t="n">
-        <v>0</v>
+        <v>20.07</v>
       </c>
       <c r="H84" s="11" t="n">
-        <v>7.37</v>
+        <v>17.41</v>
       </c>
       <c r="I84" s="11" t="n">
-        <v>0</v>
+        <v>44.97</v>
       </c>
       <c r="J84" s="11" t="n">
-        <v>9.99</v>
+        <v>38.3</v>
       </c>
       <c r="K84" s="13" t="n">
         <v>0</v>
@@ -9284,12 +9284,12 @@
     <row r="85" ht="20" customHeight="1">
       <c r="A85" s="14" t="inlineStr">
         <is>
-          <t>POC</t>
+          <t>Small</t>
         </is>
       </c>
       <c r="B85" s="14" t="inlineStr">
         <is>
-          <t>20 conn (2 threads)</t>
+          <t>100 conn (4 threads)</t>
         </is>
       </c>
       <c r="C85" s="20" t="inlineStr">
@@ -9298,32 +9298,572 @@
         </is>
       </c>
       <c r="D85" s="16" t="n">
-        <v>0</v>
+        <v>3927</v>
       </c>
       <c r="E85" s="16" t="n">
-        <v>2367.66</v>
-      </c>
-      <c r="F85" s="22">
+        <v>4299.57</v>
+      </c>
+      <c r="F85" s="17">
         <f>IF(D85&gt;0, (E85-D85)/D85, 0)</f>
         <v/>
       </c>
       <c r="G85" s="16" t="n">
-        <v>0</v>
+        <v>27.07</v>
       </c>
       <c r="H85" s="16" t="n">
-        <v>8.49</v>
+        <v>24.83</v>
       </c>
       <c r="I85" s="16" t="n">
-        <v>0</v>
+        <v>58.67</v>
       </c>
       <c r="J85" s="16" t="n">
-        <v>11.24</v>
+        <v>54.7</v>
       </c>
       <c r="K85" s="18" t="n">
         <v>0</v>
       </c>
       <c r="L85" s="18" t="n">
         <v>0</v>
+      </c>
+    </row>
+    <row r="86" ht="20" customHeight="1">
+      <c r="A86" s="9" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="B86" s="9" t="inlineStr">
+        <is>
+          <t>500 conn (8 threads)</t>
+        </is>
+      </c>
+      <c r="C86" s="19" t="inlineStr">
+        <is>
+          <t>1table</t>
+        </is>
+      </c>
+      <c r="D86" s="11" t="n">
+        <v>7384.74</v>
+      </c>
+      <c r="E86" s="11" t="n">
+        <v>8950.27</v>
+      </c>
+      <c r="F86" s="17">
+        <f>IF(D86&gt;0, (E86-D86)/D86, 0)</f>
+        <v/>
+      </c>
+      <c r="G86" s="11" t="n">
+        <v>202.47</v>
+      </c>
+      <c r="H86" s="11" t="n">
+        <v>171.07</v>
+      </c>
+      <c r="I86" s="11" t="n">
+        <v>925.89</v>
+      </c>
+      <c r="J86" s="11" t="n">
+        <v>771.48</v>
+      </c>
+      <c r="K86" s="23" t="n">
+        <v>14776</v>
+      </c>
+      <c r="L86" s="23" t="n">
+        <v>4819</v>
+      </c>
+    </row>
+    <row r="87" ht="20" customHeight="1">
+      <c r="A87" s="14" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="B87" s="14" t="inlineStr">
+        <is>
+          <t>500 conn (8 threads)</t>
+        </is>
+      </c>
+      <c r="C87" s="20" t="inlineStr">
+        <is>
+          <t>2table</t>
+        </is>
+      </c>
+      <c r="D87" s="16" t="n">
+        <v>4952.12</v>
+      </c>
+      <c r="E87" s="16" t="n">
+        <v>5612.02</v>
+      </c>
+      <c r="F87" s="17">
+        <f>IF(D87&gt;0, (E87-D87)/D87, 0)</f>
+        <v/>
+      </c>
+      <c r="G87" s="16" t="n">
+        <v>196.89</v>
+      </c>
+      <c r="H87" s="16" t="n">
+        <v>164.66</v>
+      </c>
+      <c r="I87" s="16" t="n">
+        <v>837.21</v>
+      </c>
+      <c r="J87" s="16" t="n">
+        <v>676.5599999999999</v>
+      </c>
+      <c r="K87" s="23" t="n">
+        <v>7519</v>
+      </c>
+      <c r="L87" s="23" t="n">
+        <v>2012</v>
+      </c>
+    </row>
+    <row r="88" ht="20" customHeight="1">
+      <c r="A88" s="9" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="B88" s="9" t="inlineStr">
+        <is>
+          <t>500 conn (8 threads)</t>
+        </is>
+      </c>
+      <c r="C88" s="19" t="inlineStr">
+        <is>
+          <t>3table</t>
+        </is>
+      </c>
+      <c r="D88" s="11" t="n">
+        <v>4263.4</v>
+      </c>
+      <c r="E88" s="11" t="n">
+        <v>4655.97</v>
+      </c>
+      <c r="F88" s="17">
+        <f>IF(D88&gt;0, (E88-D88)/D88, 0)</f>
+        <v/>
+      </c>
+      <c r="G88" s="11" t="n">
+        <v>194</v>
+      </c>
+      <c r="H88" s="11" t="n">
+        <v>163.46</v>
+      </c>
+      <c r="I88" s="11" t="n">
+        <v>774.13</v>
+      </c>
+      <c r="J88" s="11" t="n">
+        <v>607.6799999999999</v>
+      </c>
+      <c r="K88" s="23" t="n">
+        <v>5172</v>
+      </c>
+      <c r="L88" s="23" t="n">
+        <v>1203</v>
+      </c>
+    </row>
+    <row r="89" ht="20" customHeight="1">
+      <c r="A89" s="14" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="B89" s="14" t="inlineStr">
+        <is>
+          <t>500 conn (8 threads)</t>
+        </is>
+      </c>
+      <c r="C89" s="20" t="inlineStr">
+        <is>
+          <t>4table</t>
+        </is>
+      </c>
+      <c r="D89" s="16" t="n">
+        <v>2932.88</v>
+      </c>
+      <c r="E89" s="16" t="n">
+        <v>3155.03</v>
+      </c>
+      <c r="F89" s="17">
+        <f>IF(D89&gt;0, (E89-D89)/D89, 0)</f>
+        <v/>
+      </c>
+      <c r="G89" s="16" t="n">
+        <v>255.98</v>
+      </c>
+      <c r="H89" s="16" t="n">
+        <v>239.71</v>
+      </c>
+      <c r="I89" s="16" t="n">
+        <v>1035.98</v>
+      </c>
+      <c r="J89" s="16" t="n">
+        <v>935.54</v>
+      </c>
+      <c r="K89" s="23" t="n">
+        <v>23500</v>
+      </c>
+      <c r="L89" s="23" t="n">
+        <v>12612</v>
+      </c>
+    </row>
+    <row r="90" ht="20" customHeight="1">
+      <c r="A90" s="9" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="B90" s="9" t="inlineStr">
+        <is>
+          <t>2,000 conn (8 threads)</t>
+        </is>
+      </c>
+      <c r="C90" s="19" t="inlineStr">
+        <is>
+          <t>1table</t>
+        </is>
+      </c>
+      <c r="D90" s="11" t="n">
+        <v>7091.58</v>
+      </c>
+      <c r="E90" s="11" t="n">
+        <v>8728.6</v>
+      </c>
+      <c r="F90" s="17">
+        <f>IF(D90&gt;0, (E90-D90)/D90, 0)</f>
+        <v/>
+      </c>
+      <c r="G90" s="11" t="n">
+        <v>325.16</v>
+      </c>
+      <c r="H90" s="11" t="n">
+        <v>277.94</v>
+      </c>
+      <c r="I90" s="11" t="n">
+        <v>945.62</v>
+      </c>
+      <c r="J90" s="11" t="n">
+        <v>821.12</v>
+      </c>
+      <c r="K90" s="23" t="n">
+        <v>65027</v>
+      </c>
+      <c r="L90" s="23" t="n">
+        <v>21979</v>
+      </c>
+    </row>
+    <row r="91" ht="20" customHeight="1">
+      <c r="A91" s="14" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="B91" s="14" t="inlineStr">
+        <is>
+          <t>2,000 conn (8 threads)</t>
+        </is>
+      </c>
+      <c r="C91" s="20" t="inlineStr">
+        <is>
+          <t>2table</t>
+        </is>
+      </c>
+      <c r="D91" s="16" t="n">
+        <v>4826.72</v>
+      </c>
+      <c r="E91" s="16" t="n">
+        <v>5453.79</v>
+      </c>
+      <c r="F91" s="17">
+        <f>IF(D91&gt;0, (E91-D91)/D91, 0)</f>
+        <v/>
+      </c>
+      <c r="G91" s="16" t="n">
+        <v>440.95</v>
+      </c>
+      <c r="H91" s="16" t="n">
+        <v>399.35</v>
+      </c>
+      <c r="I91" s="16" t="n">
+        <v>1122.96</v>
+      </c>
+      <c r="J91" s="16" t="n">
+        <v>1022.8</v>
+      </c>
+      <c r="K91" s="23" t="n">
+        <v>64129</v>
+      </c>
+      <c r="L91" s="23" t="n">
+        <v>28847</v>
+      </c>
+    </row>
+    <row r="92" ht="20" customHeight="1">
+      <c r="A92" s="9" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="B92" s="9" t="inlineStr">
+        <is>
+          <t>2,000 conn (8 threads)</t>
+        </is>
+      </c>
+      <c r="C92" s="19" t="inlineStr">
+        <is>
+          <t>3table</t>
+        </is>
+      </c>
+      <c r="D92" s="11" t="n">
+        <v>4170.34</v>
+      </c>
+      <c r="E92" s="11" t="n">
+        <v>4548.17</v>
+      </c>
+      <c r="F92" s="17">
+        <f>IF(D92&gt;0, (E92-D92)/D92, 0)</f>
+        <v/>
+      </c>
+      <c r="G92" s="11" t="n">
+        <v>496.05</v>
+      </c>
+      <c r="H92" s="11" t="n">
+        <v>463.02</v>
+      </c>
+      <c r="I92" s="11" t="n">
+        <v>1211.24</v>
+      </c>
+      <c r="J92" s="11" t="n">
+        <v>1122.53</v>
+      </c>
+      <c r="K92" s="23" t="n">
+        <v>76588</v>
+      </c>
+      <c r="L92" s="23" t="n">
+        <v>39318</v>
+      </c>
+    </row>
+    <row r="93" ht="20" customHeight="1">
+      <c r="A93" s="14" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="B93" s="14" t="inlineStr">
+        <is>
+          <t>2,000 conn (8 threads)</t>
+        </is>
+      </c>
+      <c r="C93" s="20" t="inlineStr">
+        <is>
+          <t>4table</t>
+        </is>
+      </c>
+      <c r="D93" s="16" t="n">
+        <v>2896.76</v>
+      </c>
+      <c r="E93" s="16" t="n">
+        <v>3068.06</v>
+      </c>
+      <c r="F93" s="17">
+        <f>IF(D93&gt;0, (E93-D93)/D93, 0)</f>
+        <v/>
+      </c>
+      <c r="G93" s="16" t="n">
+        <v>646.6</v>
+      </c>
+      <c r="H93" s="16" t="n">
+        <v>628</v>
+      </c>
+      <c r="I93" s="16" t="n">
+        <v>1451.61</v>
+      </c>
+      <c r="J93" s="16" t="n">
+        <v>1389.48</v>
+      </c>
+      <c r="K93" s="23" t="n">
+        <v>207120</v>
+      </c>
+      <c r="L93" s="23" t="n">
+        <v>157846</v>
+      </c>
+    </row>
+    <row r="94" ht="20" customHeight="1">
+      <c r="A94" s="9" t="inlineStr">
+        <is>
+          <t>Stress</t>
+        </is>
+      </c>
+      <c r="B94" s="9" t="inlineStr">
+        <is>
+          <t>10,000 conn (16 threads)</t>
+        </is>
+      </c>
+      <c r="C94" s="19" t="inlineStr">
+        <is>
+          <t>1table</t>
+        </is>
+      </c>
+      <c r="D94" s="11" t="n">
+        <v>6759.35</v>
+      </c>
+      <c r="E94" s="11" t="n">
+        <v>8641.09</v>
+      </c>
+      <c r="F94" s="17">
+        <f>IF(D94&gt;0, (E94-D94)/D94, 0)</f>
+        <v/>
+      </c>
+      <c r="G94" s="11" t="n">
+        <v>812.0700000000001</v>
+      </c>
+      <c r="H94" s="11" t="n">
+        <v>540.45</v>
+      </c>
+      <c r="I94" s="11" t="n">
+        <v>1777.54</v>
+      </c>
+      <c r="J94" s="11" t="n">
+        <v>1544.14</v>
+      </c>
+      <c r="K94" s="23" t="n">
+        <v>9930089</v>
+      </c>
+      <c r="L94" s="23" t="n">
+        <v>11396035</v>
+      </c>
+    </row>
+    <row r="95" ht="20" customHeight="1">
+      <c r="A95" s="14" t="inlineStr">
+        <is>
+          <t>Stress</t>
+        </is>
+      </c>
+      <c r="B95" s="14" t="inlineStr">
+        <is>
+          <t>10,000 conn (16 threads)</t>
+        </is>
+      </c>
+      <c r="C95" s="20" t="inlineStr">
+        <is>
+          <t>2table</t>
+        </is>
+      </c>
+      <c r="D95" s="16" t="n">
+        <v>4730.62</v>
+      </c>
+      <c r="E95" s="16" t="n">
+        <v>5488.15</v>
+      </c>
+      <c r="F95" s="17">
+        <f>IF(D95&gt;0, (E95-D95)/D95, 0)</f>
+        <v/>
+      </c>
+      <c r="G95" s="16" t="n">
+        <v>667.74</v>
+      </c>
+      <c r="H95" s="16" t="n">
+        <v>768.85</v>
+      </c>
+      <c r="I95" s="16" t="n">
+        <v>1940.59</v>
+      </c>
+      <c r="J95" s="16" t="n">
+        <v>1915.8</v>
+      </c>
+      <c r="K95" s="23" t="n">
+        <v>13844249</v>
+      </c>
+      <c r="L95" s="23" t="n">
+        <v>11436935</v>
+      </c>
+    </row>
+    <row r="96" ht="20" customHeight="1">
+      <c r="A96" s="9" t="inlineStr">
+        <is>
+          <t>Stress</t>
+        </is>
+      </c>
+      <c r="B96" s="9" t="inlineStr">
+        <is>
+          <t>10,000 conn (16 threads)</t>
+        </is>
+      </c>
+      <c r="C96" s="19" t="inlineStr">
+        <is>
+          <t>3table</t>
+        </is>
+      </c>
+      <c r="D96" s="11" t="n">
+        <v>4106.6</v>
+      </c>
+      <c r="E96" s="11" t="n">
+        <v>4571.22</v>
+      </c>
+      <c r="F96" s="17">
+        <f>IF(D96&gt;0, (E96-D96)/D96, 0)</f>
+        <v/>
+      </c>
+      <c r="G96" s="11" t="n">
+        <v>402.45</v>
+      </c>
+      <c r="H96" s="11" t="n">
+        <v>534.55</v>
+      </c>
+      <c r="I96" s="11" t="n">
+        <v>1895.41</v>
+      </c>
+      <c r="J96" s="11" t="n">
+        <v>1956.34</v>
+      </c>
+      <c r="K96" s="23" t="n">
+        <v>15235684</v>
+      </c>
+      <c r="L96" s="23" t="n">
+        <v>15212131</v>
+      </c>
+    </row>
+    <row r="97" ht="20" customHeight="1">
+      <c r="A97" s="14" t="inlineStr">
+        <is>
+          <t>Stress</t>
+        </is>
+      </c>
+      <c r="B97" s="14" t="inlineStr">
+        <is>
+          <t>10,000 conn (16 threads)</t>
+        </is>
+      </c>
+      <c r="C97" s="20" t="inlineStr">
+        <is>
+          <t>4table</t>
+        </is>
+      </c>
+      <c r="D97" s="16" t="n">
+        <v>2874.17</v>
+      </c>
+      <c r="E97" s="16" t="n">
+        <v>3053.83</v>
+      </c>
+      <c r="F97" s="17">
+        <f>IF(D97&gt;0, (E97-D97)/D97, 0)</f>
+        <v/>
+      </c>
+      <c r="G97" s="16" t="n">
+        <v>150.05</v>
+      </c>
+      <c r="H97" s="16" t="n">
+        <v>142.18</v>
+      </c>
+      <c r="I97" s="16" t="n">
+        <v>716.75</v>
+      </c>
+      <c r="J97" s="16" t="n">
+        <v>633</v>
+      </c>
+      <c r="K97" s="23" t="n">
+        <v>13106737</v>
+      </c>
+      <c r="L97" s="23" t="n">
+        <v>13761138</v>
       </c>
     </row>
   </sheetData>
@@ -9345,7 +9885,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L85"/>
+  <dimension ref="A1:L97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="109" customWidth="1" min="1" max="1"/>
@@ -11415,12 +11955,12 @@
     <row r="78" ht="20" customHeight="1">
       <c r="A78" s="9" t="inlineStr">
         <is>
-          <t>Min</t>
+          <t>POC</t>
         </is>
       </c>
       <c r="B78" s="9" t="inlineStr">
         <is>
-          <t>100 conn (2 threads)</t>
+          <t>20 conn (2 threads)</t>
         </is>
       </c>
       <c r="C78" s="19" t="inlineStr">
@@ -11429,26 +11969,26 @@
         </is>
       </c>
       <c r="D78" s="11" t="n">
-        <v>7297.44</v>
+        <v>10604.52</v>
       </c>
       <c r="E78" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="F78" s="12">
+        <v>14308.05</v>
+      </c>
+      <c r="F78" s="17">
         <f>IF(D78&gt;0, (E78-D78)/D78, 0)</f>
         <v/>
       </c>
       <c r="G78" s="11" t="n">
-        <v>13.94</v>
+        <v>2.07</v>
       </c>
       <c r="H78" s="11" t="n">
-        <v>0</v>
+        <v>1.65</v>
       </c>
       <c r="I78" s="11" t="n">
-        <v>0</v>
+        <v>3.83</v>
       </c>
       <c r="J78" s="11" t="n">
-        <v>0</v>
+        <v>2.83</v>
       </c>
       <c r="K78" s="13" t="n">
         <v>0</v>
@@ -11460,12 +12000,12 @@
     <row r="79" ht="20" customHeight="1">
       <c r="A79" s="14" t="inlineStr">
         <is>
-          <t>Min</t>
+          <t>POC</t>
         </is>
       </c>
       <c r="B79" s="14" t="inlineStr">
         <is>
-          <t>100 conn (2 threads)</t>
+          <t>20 conn (2 threads)</t>
         </is>
       </c>
       <c r="C79" s="20" t="inlineStr">
@@ -11474,26 +12014,26 @@
         </is>
       </c>
       <c r="D79" s="16" t="n">
-        <v>4327.39</v>
+        <v>4672.64</v>
       </c>
       <c r="E79" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="F79" s="12">
+        <v>5908.4</v>
+      </c>
+      <c r="F79" s="17">
         <f>IF(D79&gt;0, (E79-D79)/D79, 0)</f>
         <v/>
       </c>
       <c r="G79" s="16" t="n">
-        <v>23.2</v>
+        <v>4.42</v>
       </c>
       <c r="H79" s="16" t="n">
-        <v>0</v>
+        <v>3.81</v>
       </c>
       <c r="I79" s="16" t="n">
-        <v>0</v>
+        <v>7.13</v>
       </c>
       <c r="J79" s="16" t="n">
-        <v>0</v>
+        <v>5.45</v>
       </c>
       <c r="K79" s="18" t="n">
         <v>0</v>
@@ -11505,12 +12045,12 @@
     <row r="80" ht="20" customHeight="1">
       <c r="A80" s="9" t="inlineStr">
         <is>
-          <t>Min</t>
+          <t>POC</t>
         </is>
       </c>
       <c r="B80" s="9" t="inlineStr">
         <is>
-          <t>100 conn (2 threads)</t>
+          <t>20 conn (2 threads)</t>
         </is>
       </c>
       <c r="C80" s="19" t="inlineStr">
@@ -11519,26 +12059,26 @@
         </is>
       </c>
       <c r="D80" s="11" t="n">
-        <v>3830.39</v>
+        <v>3861.93</v>
       </c>
       <c r="E80" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="F80" s="12">
+        <v>4863.33</v>
+      </c>
+      <c r="F80" s="17">
         <f>IF(D80&gt;0, (E80-D80)/D80, 0)</f>
         <v/>
       </c>
       <c r="G80" s="11" t="n">
-        <v>26.06</v>
+        <v>5.31</v>
       </c>
       <c r="H80" s="11" t="n">
-        <v>0</v>
+        <v>4.28</v>
       </c>
       <c r="I80" s="11" t="n">
-        <v>0</v>
+        <v>8.43</v>
       </c>
       <c r="J80" s="11" t="n">
-        <v>0</v>
+        <v>6.43</v>
       </c>
       <c r="K80" s="13" t="n">
         <v>0</v>
@@ -11550,12 +12090,12 @@
     <row r="81" ht="20" customHeight="1">
       <c r="A81" s="14" t="inlineStr">
         <is>
-          <t>Min</t>
+          <t>POC</t>
         </is>
       </c>
       <c r="B81" s="14" t="inlineStr">
         <is>
-          <t>100 conn (2 threads)</t>
+          <t>20 conn (2 threads)</t>
         </is>
       </c>
       <c r="C81" s="20" t="inlineStr">
@@ -11564,26 +12104,26 @@
         </is>
       </c>
       <c r="D81" s="16" t="n">
-        <v>2907.82</v>
+        <v>2885.08</v>
       </c>
       <c r="E81" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="F81" s="12">
+        <v>3625.69</v>
+      </c>
+      <c r="F81" s="17">
         <f>IF(D81&gt;0, (E81-D81)/D81, 0)</f>
         <v/>
       </c>
       <c r="G81" s="16" t="n">
-        <v>34.41</v>
+        <v>7.09</v>
       </c>
       <c r="H81" s="16" t="n">
-        <v>0</v>
+        <v>5.7</v>
       </c>
       <c r="I81" s="16" t="n">
-        <v>0</v>
+        <v>11.4</v>
       </c>
       <c r="J81" s="16" t="n">
-        <v>0</v>
+        <v>8.539999999999999</v>
       </c>
       <c r="K81" s="18" t="n">
         <v>0</v>
@@ -11595,12 +12135,12 @@
     <row r="82" ht="20" customHeight="1">
       <c r="A82" s="9" t="inlineStr">
         <is>
-          <t>POC</t>
+          <t>Small</t>
         </is>
       </c>
       <c r="B82" s="9" t="inlineStr">
         <is>
-          <t>20 conn (2 threads)</t>
+          <t>100 conn (4 threads)</t>
         </is>
       </c>
       <c r="C82" s="19" t="inlineStr">
@@ -11609,26 +12149,26 @@
         </is>
       </c>
       <c r="D82" s="11" t="n">
-        <v>0</v>
+        <v>9095.809999999999</v>
       </c>
       <c r="E82" s="11" t="n">
-        <v>4605.9</v>
-      </c>
-      <c r="F82" s="21">
+        <v>14305.56</v>
+      </c>
+      <c r="F82" s="17">
         <f>IF(D82&gt;0, (E82-D82)/D82, 0)</f>
         <v/>
       </c>
       <c r="G82" s="11" t="n">
-        <v>0</v>
+        <v>21.29</v>
       </c>
       <c r="H82" s="11" t="n">
-        <v>4.36</v>
+        <v>9.16</v>
       </c>
       <c r="I82" s="11" t="n">
-        <v>0</v>
+        <v>91.61</v>
       </c>
       <c r="J82" s="11" t="n">
-        <v>6.36</v>
+        <v>25.71</v>
       </c>
       <c r="K82" s="13" t="n">
         <v>0</v>
@@ -11640,12 +12180,12 @@
     <row r="83" ht="20" customHeight="1">
       <c r="A83" s="14" t="inlineStr">
         <is>
-          <t>POC</t>
+          <t>Small</t>
         </is>
       </c>
       <c r="B83" s="14" t="inlineStr">
         <is>
-          <t>20 conn (2 threads)</t>
+          <t>100 conn (4 threads)</t>
         </is>
       </c>
       <c r="C83" s="20" t="inlineStr">
@@ -11654,26 +12194,26 @@
         </is>
       </c>
       <c r="D83" s="16" t="n">
-        <v>0</v>
+        <v>5005.85</v>
       </c>
       <c r="E83" s="16" t="n">
-        <v>3273.11</v>
-      </c>
-      <c r="F83" s="22">
+        <v>6300.88</v>
+      </c>
+      <c r="F83" s="17">
         <f>IF(D83&gt;0, (E83-D83)/D83, 0)</f>
         <v/>
       </c>
       <c r="G83" s="16" t="n">
-        <v>0</v>
+        <v>20.24</v>
       </c>
       <c r="H83" s="16" t="n">
-        <v>6.19</v>
+        <v>16.36</v>
       </c>
       <c r="I83" s="16" t="n">
-        <v>0</v>
+        <v>30.51</v>
       </c>
       <c r="J83" s="16" t="n">
-        <v>8.91</v>
+        <v>23.54</v>
       </c>
       <c r="K83" s="18" t="n">
         <v>0</v>
@@ -11685,12 +12225,12 @@
     <row r="84" ht="20" customHeight="1">
       <c r="A84" s="9" t="inlineStr">
         <is>
-          <t>POC</t>
+          <t>Small</t>
         </is>
       </c>
       <c r="B84" s="9" t="inlineStr">
         <is>
-          <t>20 conn (2 threads)</t>
+          <t>100 conn (4 threads)</t>
         </is>
       </c>
       <c r="C84" s="19" t="inlineStr">
@@ -11699,26 +12239,26 @@
         </is>
       </c>
       <c r="D84" s="11" t="n">
-        <v>0</v>
+        <v>4180.3</v>
       </c>
       <c r="E84" s="11" t="n">
-        <v>3035.43</v>
-      </c>
-      <c r="F84" s="21">
+        <v>5220.53</v>
+      </c>
+      <c r="F84" s="17">
         <f>IF(D84&gt;0, (E84-D84)/D84, 0)</f>
         <v/>
       </c>
       <c r="G84" s="11" t="n">
-        <v>0</v>
+        <v>24.08</v>
       </c>
       <c r="H84" s="11" t="n">
-        <v>6.7</v>
+        <v>19.65</v>
       </c>
       <c r="I84" s="11" t="n">
-        <v>0</v>
+        <v>35.6</v>
       </c>
       <c r="J84" s="11" t="n">
-        <v>9.42</v>
+        <v>28.24</v>
       </c>
       <c r="K84" s="13" t="n">
         <v>0</v>
@@ -11730,12 +12270,12 @@
     <row r="85" ht="20" customHeight="1">
       <c r="A85" s="14" t="inlineStr">
         <is>
-          <t>POC</t>
+          <t>Small</t>
         </is>
       </c>
       <c r="B85" s="14" t="inlineStr">
         <is>
-          <t>20 conn (2 threads)</t>
+          <t>100 conn (4 threads)</t>
         </is>
       </c>
       <c r="C85" s="20" t="inlineStr">
@@ -11744,32 +12284,572 @@
         </is>
       </c>
       <c r="D85" s="16" t="n">
-        <v>0</v>
+        <v>3115.32</v>
       </c>
       <c r="E85" s="16" t="n">
-        <v>2446.43</v>
-      </c>
-      <c r="F85" s="22">
+        <v>3822.98</v>
+      </c>
+      <c r="F85" s="17">
         <f>IF(D85&gt;0, (E85-D85)/D85, 0)</f>
         <v/>
       </c>
       <c r="G85" s="16" t="n">
-        <v>0</v>
+        <v>32.23</v>
       </c>
       <c r="H85" s="16" t="n">
-        <v>8.369999999999999</v>
+        <v>26.47</v>
       </c>
       <c r="I85" s="16" t="n">
-        <v>0</v>
+        <v>46.84</v>
       </c>
       <c r="J85" s="16" t="n">
-        <v>11.56</v>
+        <v>39.84</v>
       </c>
       <c r="K85" s="18" t="n">
         <v>0</v>
       </c>
       <c r="L85" s="18" t="n">
         <v>0</v>
+      </c>
+    </row>
+    <row r="86" ht="20" customHeight="1">
+      <c r="A86" s="9" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="B86" s="9" t="inlineStr">
+        <is>
+          <t>500 conn (8 threads)</t>
+        </is>
+      </c>
+      <c r="C86" s="19" t="inlineStr">
+        <is>
+          <t>1table</t>
+        </is>
+      </c>
+      <c r="D86" s="11" t="n">
+        <v>7311.04</v>
+      </c>
+      <c r="E86" s="11" t="n">
+        <v>9339.360000000001</v>
+      </c>
+      <c r="F86" s="17">
+        <f>IF(D86&gt;0, (E86-D86)/D86, 0)</f>
+        <v/>
+      </c>
+      <c r="G86" s="11" t="n">
+        <v>205.22</v>
+      </c>
+      <c r="H86" s="11" t="n">
+        <v>169.69</v>
+      </c>
+      <c r="I86" s="11" t="n">
+        <v>938.87</v>
+      </c>
+      <c r="J86" s="11" t="n">
+        <v>765.92</v>
+      </c>
+      <c r="K86" s="23" t="n">
+        <v>16045</v>
+      </c>
+      <c r="L86" s="23" t="n">
+        <v>4658</v>
+      </c>
+    </row>
+    <row r="87" ht="20" customHeight="1">
+      <c r="A87" s="14" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="B87" s="14" t="inlineStr">
+        <is>
+          <t>500 conn (8 threads)</t>
+        </is>
+      </c>
+      <c r="C87" s="20" t="inlineStr">
+        <is>
+          <t>2table</t>
+        </is>
+      </c>
+      <c r="D87" s="16" t="n">
+        <v>4718.4</v>
+      </c>
+      <c r="E87" s="16" t="n">
+        <v>5874.18</v>
+      </c>
+      <c r="F87" s="17">
+        <f>IF(D87&gt;0, (E87-D87)/D87, 0)</f>
+        <v/>
+      </c>
+      <c r="G87" s="16" t="n">
+        <v>108.29</v>
+      </c>
+      <c r="H87" s="16" t="n">
+        <v>87.58</v>
+      </c>
+      <c r="I87" s="16" t="n">
+        <v>192.58</v>
+      </c>
+      <c r="J87" s="16" t="n">
+        <v>158.97</v>
+      </c>
+      <c r="K87" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="L87" s="18" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="88" ht="20" customHeight="1">
+      <c r="A88" s="9" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="B88" s="9" t="inlineStr">
+        <is>
+          <t>500 conn (8 threads)</t>
+        </is>
+      </c>
+      <c r="C88" s="19" t="inlineStr">
+        <is>
+          <t>3table</t>
+        </is>
+      </c>
+      <c r="D88" s="11" t="n">
+        <v>3979.22</v>
+      </c>
+      <c r="E88" s="11" t="n">
+        <v>4887.96</v>
+      </c>
+      <c r="F88" s="17">
+        <f>IF(D88&gt;0, (E88-D88)/D88, 0)</f>
+        <v/>
+      </c>
+      <c r="G88" s="11" t="n">
+        <v>125.76</v>
+      </c>
+      <c r="H88" s="11" t="n">
+        <v>103.36</v>
+      </c>
+      <c r="I88" s="11" t="n">
+        <v>190.09</v>
+      </c>
+      <c r="J88" s="11" t="n">
+        <v>173.81</v>
+      </c>
+      <c r="K88" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="L88" s="13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="89" ht="20" customHeight="1">
+      <c r="A89" s="14" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="B89" s="14" t="inlineStr">
+        <is>
+          <t>500 conn (8 threads)</t>
+        </is>
+      </c>
+      <c r="C89" s="20" t="inlineStr">
+        <is>
+          <t>4table</t>
+        </is>
+      </c>
+      <c r="D89" s="16" t="n">
+        <v>2910.63</v>
+      </c>
+      <c r="E89" s="16" t="n">
+        <v>3509.02</v>
+      </c>
+      <c r="F89" s="17">
+        <f>IF(D89&gt;0, (E89-D89)/D89, 0)</f>
+        <v/>
+      </c>
+      <c r="G89" s="16" t="n">
+        <v>171.42</v>
+      </c>
+      <c r="H89" s="16" t="n">
+        <v>144.71</v>
+      </c>
+      <c r="I89" s="16" t="n">
+        <v>275.11</v>
+      </c>
+      <c r="J89" s="16" t="n">
+        <v>267.66</v>
+      </c>
+      <c r="K89" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="L89" s="18" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="90" ht="20" customHeight="1">
+      <c r="A90" s="9" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="B90" s="9" t="inlineStr">
+        <is>
+          <t>2,000 conn (8 threads)</t>
+        </is>
+      </c>
+      <c r="C90" s="19" t="inlineStr">
+        <is>
+          <t>1table</t>
+        </is>
+      </c>
+      <c r="D90" s="11" t="n">
+        <v>7053.23</v>
+      </c>
+      <c r="E90" s="11" t="n">
+        <v>9202.110000000001</v>
+      </c>
+      <c r="F90" s="17">
+        <f>IF(D90&gt;0, (E90-D90)/D90, 0)</f>
+        <v/>
+      </c>
+      <c r="G90" s="11" t="n">
+        <v>309.52</v>
+      </c>
+      <c r="H90" s="11" t="n">
+        <v>245.9</v>
+      </c>
+      <c r="I90" s="11" t="n">
+        <v>808.7</v>
+      </c>
+      <c r="J90" s="11" t="n">
+        <v>658.72</v>
+      </c>
+      <c r="K90" s="23" t="n">
+        <v>53763</v>
+      </c>
+      <c r="L90" s="23" t="n">
+        <v>16108</v>
+      </c>
+    </row>
+    <row r="91" ht="20" customHeight="1">
+      <c r="A91" s="14" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="B91" s="14" t="inlineStr">
+        <is>
+          <t>2,000 conn (8 threads)</t>
+        </is>
+      </c>
+      <c r="C91" s="20" t="inlineStr">
+        <is>
+          <t>2table</t>
+        </is>
+      </c>
+      <c r="D91" s="16" t="n">
+        <v>4490.31</v>
+      </c>
+      <c r="E91" s="16" t="n">
+        <v>5707.67</v>
+      </c>
+      <c r="F91" s="17">
+        <f>IF(D91&gt;0, (E91-D91)/D91, 0)</f>
+        <v/>
+      </c>
+      <c r="G91" s="16" t="n">
+        <v>441.61</v>
+      </c>
+      <c r="H91" s="16" t="n">
+        <v>348.83</v>
+      </c>
+      <c r="I91" s="16" t="n">
+        <v>545.87</v>
+      </c>
+      <c r="J91" s="16" t="n">
+        <v>442.06</v>
+      </c>
+      <c r="K91" s="23" t="n">
+        <v>14975</v>
+      </c>
+      <c r="L91" s="23" t="n">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="92" ht="20" customHeight="1">
+      <c r="A92" s="9" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="B92" s="9" t="inlineStr">
+        <is>
+          <t>2,000 conn (8 threads)</t>
+        </is>
+      </c>
+      <c r="C92" s="19" t="inlineStr">
+        <is>
+          <t>3table</t>
+        </is>
+      </c>
+      <c r="D92" s="11" t="n">
+        <v>3774.47</v>
+      </c>
+      <c r="E92" s="11" t="n">
+        <v>4737.78</v>
+      </c>
+      <c r="F92" s="17">
+        <f>IF(D92&gt;0, (E92-D92)/D92, 0)</f>
+        <v/>
+      </c>
+      <c r="G92" s="11" t="n">
+        <v>523.96</v>
+      </c>
+      <c r="H92" s="11" t="n">
+        <v>420.02</v>
+      </c>
+      <c r="I92" s="11" t="n">
+        <v>633.91</v>
+      </c>
+      <c r="J92" s="11" t="n">
+        <v>522.04</v>
+      </c>
+      <c r="K92" s="23" t="n">
+        <v>17374</v>
+      </c>
+      <c r="L92" s="23" t="n">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="93" ht="20" customHeight="1">
+      <c r="A93" s="14" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="B93" s="14" t="inlineStr">
+        <is>
+          <t>2,000 conn (8 threads)</t>
+        </is>
+      </c>
+      <c r="C93" s="20" t="inlineStr">
+        <is>
+          <t>4table</t>
+        </is>
+      </c>
+      <c r="D93" s="16" t="n">
+        <v>2774.78</v>
+      </c>
+      <c r="E93" s="16" t="n">
+        <v>3373.84</v>
+      </c>
+      <c r="F93" s="17">
+        <f>IF(D93&gt;0, (E93-D93)/D93, 0)</f>
+        <v/>
+      </c>
+      <c r="G93" s="16" t="n">
+        <v>712.86</v>
+      </c>
+      <c r="H93" s="16" t="n">
+        <v>588.73</v>
+      </c>
+      <c r="I93" s="16" t="n">
+        <v>853.89</v>
+      </c>
+      <c r="J93" s="16" t="n">
+        <v>733.77</v>
+      </c>
+      <c r="K93" s="23" t="n">
+        <v>15849</v>
+      </c>
+      <c r="L93" s="23" t="n">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="94" ht="20" customHeight="1">
+      <c r="A94" s="9" t="inlineStr">
+        <is>
+          <t>Stress</t>
+        </is>
+      </c>
+      <c r="B94" s="9" t="inlineStr">
+        <is>
+          <t>10,000 conn (16 threads)</t>
+        </is>
+      </c>
+      <c r="C94" s="19" t="inlineStr">
+        <is>
+          <t>1table</t>
+        </is>
+      </c>
+      <c r="D94" s="11" t="n">
+        <v>6746.36</v>
+      </c>
+      <c r="E94" s="11" t="n">
+        <v>8814.200000000001</v>
+      </c>
+      <c r="F94" s="17">
+        <f>IF(D94&gt;0, (E94-D94)/D94, 0)</f>
+        <v/>
+      </c>
+      <c r="G94" s="11" t="n">
+        <v>1422.01</v>
+      </c>
+      <c r="H94" s="11" t="n">
+        <v>1113.09</v>
+      </c>
+      <c r="I94" s="11" t="n">
+        <v>1815.18</v>
+      </c>
+      <c r="J94" s="11" t="n">
+        <v>1438.92</v>
+      </c>
+      <c r="K94" s="23" t="n">
+        <v>1922657</v>
+      </c>
+      <c r="L94" s="23" t="n">
+        <v>647782</v>
+      </c>
+    </row>
+    <row r="95" ht="20" customHeight="1">
+      <c r="A95" s="14" t="inlineStr">
+        <is>
+          <t>Stress</t>
+        </is>
+      </c>
+      <c r="B95" s="14" t="inlineStr">
+        <is>
+          <t>10,000 conn (16 threads)</t>
+        </is>
+      </c>
+      <c r="C95" s="20" t="inlineStr">
+        <is>
+          <t>2table</t>
+        </is>
+      </c>
+      <c r="D95" s="16" t="n">
+        <v>4357.52</v>
+      </c>
+      <c r="E95" s="16" t="n">
+        <v>5688.49</v>
+      </c>
+      <c r="F95" s="17">
+        <f>IF(D95&gt;0, (E95-D95)/D95, 0)</f>
+        <v/>
+      </c>
+      <c r="G95" s="16" t="n">
+        <v>1269.13</v>
+      </c>
+      <c r="H95" s="16" t="n">
+        <v>1700.84</v>
+      </c>
+      <c r="I95" s="16" t="n">
+        <v>1980.26</v>
+      </c>
+      <c r="J95" s="16" t="n">
+        <v>1933.6</v>
+      </c>
+      <c r="K95" s="23" t="n">
+        <v>24203173</v>
+      </c>
+      <c r="L95" s="23" t="n">
+        <v>1579467</v>
+      </c>
+    </row>
+    <row r="96" ht="20" customHeight="1">
+      <c r="A96" s="9" t="inlineStr">
+        <is>
+          <t>Stress</t>
+        </is>
+      </c>
+      <c r="B96" s="9" t="inlineStr">
+        <is>
+          <t>10,000 conn (16 threads)</t>
+        </is>
+      </c>
+      <c r="C96" s="19" t="inlineStr">
+        <is>
+          <t>3table</t>
+        </is>
+      </c>
+      <c r="D96" s="11" t="n">
+        <v>3671.77</v>
+      </c>
+      <c r="E96" s="11" t="n">
+        <v>4698.1</v>
+      </c>
+      <c r="F96" s="17">
+        <f>IF(D96&gt;0, (E96-D96)/D96, 0)</f>
+        <v/>
+      </c>
+      <c r="G96" s="11" t="n">
+        <v>1096.34</v>
+      </c>
+      <c r="H96" s="11" t="n">
+        <v>1752.84</v>
+      </c>
+      <c r="I96" s="11" t="n">
+        <v>1907.62</v>
+      </c>
+      <c r="J96" s="11" t="n">
+        <v>1994.1</v>
+      </c>
+      <c r="K96" s="23" t="n">
+        <v>21001257</v>
+      </c>
+      <c r="L96" s="23" t="n">
+        <v>21745607</v>
+      </c>
+    </row>
+    <row r="97" ht="20" customHeight="1">
+      <c r="A97" s="14" t="inlineStr">
+        <is>
+          <t>Stress</t>
+        </is>
+      </c>
+      <c r="B97" s="14" t="inlineStr">
+        <is>
+          <t>10,000 conn (16 threads)</t>
+        </is>
+      </c>
+      <c r="C97" s="20" t="inlineStr">
+        <is>
+          <t>4table</t>
+        </is>
+      </c>
+      <c r="D97" s="16" t="n">
+        <v>2699.97</v>
+      </c>
+      <c r="E97" s="16" t="n">
+        <v>3359.24</v>
+      </c>
+      <c r="F97" s="17">
+        <f>IF(D97&gt;0, (E97-D97)/D97, 0)</f>
+        <v/>
+      </c>
+      <c r="G97" s="16" t="n">
+        <v>1211.06</v>
+      </c>
+      <c r="H97" s="16" t="n">
+        <v>1268.17</v>
+      </c>
+      <c r="I97" s="16" t="n">
+        <v>1909.21</v>
+      </c>
+      <c r="J97" s="16" t="n">
+        <v>1925.28</v>
+      </c>
+      <c r="K97" s="23" t="n">
+        <v>15815786</v>
+      </c>
+      <c r="L97" s="23" t="n">
+        <v>19774430</v>
       </c>
     </row>
   </sheetData>
@@ -11791,7 +12871,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L85"/>
+  <dimension ref="A1:L97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -13861,12 +14941,12 @@
     <row r="78" ht="20" customHeight="1">
       <c r="A78" s="9" t="inlineStr">
         <is>
-          <t>Min</t>
+          <t>POC</t>
         </is>
       </c>
       <c r="B78" s="9" t="inlineStr">
         <is>
-          <t>100 conn (2 threads)</t>
+          <t>20 conn (2 threads)</t>
         </is>
       </c>
       <c r="C78" s="19" t="inlineStr">
@@ -13875,26 +14955,26 @@
         </is>
       </c>
       <c r="D78" s="11" t="n">
-        <v>4506.78</v>
+        <v>12581.47</v>
       </c>
       <c r="E78" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="F78" s="12">
+        <v>18730.75</v>
+      </c>
+      <c r="F78" s="17">
         <f>IF(D78&gt;0, (E78-D78)/D78, 0)</f>
         <v/>
       </c>
       <c r="G78" s="11" t="n">
-        <v>23.91</v>
+        <v>2.27</v>
       </c>
       <c r="H78" s="11" t="n">
-        <v>0</v>
+        <v>1.41</v>
       </c>
       <c r="I78" s="11" t="n">
-        <v>0</v>
+        <v>4.5</v>
       </c>
       <c r="J78" s="11" t="n">
-        <v>0</v>
+        <v>3.34</v>
       </c>
       <c r="K78" s="13" t="n">
         <v>0</v>
@@ -13906,12 +14986,12 @@
     <row r="79" ht="20" customHeight="1">
       <c r="A79" s="14" t="inlineStr">
         <is>
-          <t>Min</t>
+          <t>POC</t>
         </is>
       </c>
       <c r="B79" s="14" t="inlineStr">
         <is>
-          <t>100 conn (2 threads)</t>
+          <t>20 conn (2 threads)</t>
         </is>
       </c>
       <c r="C79" s="20" t="inlineStr">
@@ -13920,26 +15000,26 @@
         </is>
       </c>
       <c r="D79" s="16" t="n">
-        <v>3375.61</v>
+        <v>6640.47</v>
       </c>
       <c r="E79" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="F79" s="12">
+        <v>7659.67</v>
+      </c>
+      <c r="F79" s="17">
         <f>IF(D79&gt;0, (E79-D79)/D79, 0)</f>
         <v/>
       </c>
       <c r="G79" s="16" t="n">
-        <v>37.14</v>
+        <v>3.34</v>
       </c>
       <c r="H79" s="16" t="n">
-        <v>0</v>
+        <v>3.06</v>
       </c>
       <c r="I79" s="16" t="n">
-        <v>0</v>
+        <v>7.57</v>
       </c>
       <c r="J79" s="16" t="n">
-        <v>0</v>
+        <v>7.79</v>
       </c>
       <c r="K79" s="18" t="n">
         <v>0</v>
@@ -13951,12 +15031,12 @@
     <row r="80" ht="20" customHeight="1">
       <c r="A80" s="9" t="inlineStr">
         <is>
-          <t>Min</t>
+          <t>POC</t>
         </is>
       </c>
       <c r="B80" s="9" t="inlineStr">
         <is>
-          <t>100 conn (2 threads)</t>
+          <t>20 conn (2 threads)</t>
         </is>
       </c>
       <c r="C80" s="19" t="inlineStr">
@@ -13965,26 +15045,26 @@
         </is>
       </c>
       <c r="D80" s="11" t="n">
-        <v>2520.47</v>
+        <v>5452.02</v>
       </c>
       <c r="E80" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="F80" s="12">
+        <v>6304.13</v>
+      </c>
+      <c r="F80" s="17">
         <f>IF(D80&gt;0, (E80-D80)/D80, 0)</f>
         <v/>
       </c>
       <c r="G80" s="11" t="n">
-        <v>44.71</v>
+        <v>4.08</v>
       </c>
       <c r="H80" s="11" t="n">
-        <v>0</v>
+        <v>3.77</v>
       </c>
       <c r="I80" s="11" t="n">
-        <v>0</v>
+        <v>9.640000000000001</v>
       </c>
       <c r="J80" s="11" t="n">
-        <v>0</v>
+        <v>9.390000000000001</v>
       </c>
       <c r="K80" s="13" t="n">
         <v>0</v>
@@ -13996,12 +15076,12 @@
     <row r="81" ht="20" customHeight="1">
       <c r="A81" s="14" t="inlineStr">
         <is>
-          <t>Min</t>
+          <t>POC</t>
         </is>
       </c>
       <c r="B81" s="14" t="inlineStr">
         <is>
-          <t>100 conn (2 threads)</t>
+          <t>20 conn (2 threads)</t>
         </is>
       </c>
       <c r="C81" s="20" t="inlineStr">
@@ -14010,26 +15090,26 @@
         </is>
       </c>
       <c r="D81" s="16" t="n">
-        <v>2484.42</v>
+        <v>4091.48</v>
       </c>
       <c r="E81" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="F81" s="12">
+        <v>4390.46</v>
+      </c>
+      <c r="F81" s="17">
         <f>IF(D81&gt;0, (E81-D81)/D81, 0)</f>
         <v/>
       </c>
       <c r="G81" s="16" t="n">
-        <v>48.57</v>
+        <v>5.37</v>
       </c>
       <c r="H81" s="16" t="n">
-        <v>0</v>
+        <v>5.24</v>
       </c>
       <c r="I81" s="16" t="n">
-        <v>0</v>
+        <v>12.32</v>
       </c>
       <c r="J81" s="16" t="n">
-        <v>0</v>
+        <v>12.78</v>
       </c>
       <c r="K81" s="18" t="n">
         <v>0</v>
@@ -14041,12 +15121,12 @@
     <row r="82" ht="20" customHeight="1">
       <c r="A82" s="9" t="inlineStr">
         <is>
-          <t>POC</t>
+          <t>Small</t>
         </is>
       </c>
       <c r="B82" s="9" t="inlineStr">
         <is>
-          <t>20 conn (2 threads)</t>
+          <t>100 conn (4 threads)</t>
         </is>
       </c>
       <c r="C82" s="19" t="inlineStr">
@@ -14055,26 +15135,26 @@
         </is>
       </c>
       <c r="D82" s="11" t="n">
-        <v>0</v>
+        <v>12991.53</v>
       </c>
       <c r="E82" s="11" t="n">
-        <v>3599.8</v>
-      </c>
-      <c r="F82" s="21">
+        <v>16223.81</v>
+      </c>
+      <c r="F82" s="17">
         <f>IF(D82&gt;0, (E82-D82)/D82, 0)</f>
         <v/>
       </c>
       <c r="G82" s="11" t="n">
-        <v>0</v>
+        <v>9.25</v>
       </c>
       <c r="H82" s="11" t="n">
-        <v>5.89</v>
+        <v>7.35</v>
       </c>
       <c r="I82" s="11" t="n">
-        <v>0</v>
+        <v>26.37</v>
       </c>
       <c r="J82" s="11" t="n">
-        <v>13.05</v>
+        <v>20.15</v>
       </c>
       <c r="K82" s="13" t="n">
         <v>0</v>
@@ -14086,12 +15166,12 @@
     <row r="83" ht="20" customHeight="1">
       <c r="A83" s="14" t="inlineStr">
         <is>
-          <t>POC</t>
+          <t>Small</t>
         </is>
       </c>
       <c r="B83" s="14" t="inlineStr">
         <is>
-          <t>20 conn (2 threads)</t>
+          <t>100 conn (4 threads)</t>
         </is>
       </c>
       <c r="C83" s="20" t="inlineStr">
@@ -14100,26 +15180,26 @@
         </is>
       </c>
       <c r="D83" s="16" t="n">
-        <v>0</v>
+        <v>7940.02</v>
       </c>
       <c r="E83" s="16" t="n">
-        <v>928.6</v>
-      </c>
-      <c r="F83" s="22">
+        <v>9946.59</v>
+      </c>
+      <c r="F83" s="17">
         <f>IF(D83&gt;0, (E83-D83)/D83, 0)</f>
         <v/>
       </c>
       <c r="G83" s="16" t="n">
-        <v>0</v>
+        <v>14.38</v>
       </c>
       <c r="H83" s="16" t="n">
-        <v>22.04</v>
+        <v>11.53</v>
       </c>
       <c r="I83" s="16" t="n">
-        <v>0</v>
+        <v>38.16</v>
       </c>
       <c r="J83" s="16" t="n">
-        <v>37.71</v>
+        <v>30.16</v>
       </c>
       <c r="K83" s="18" t="n">
         <v>0</v>
@@ -14131,12 +15211,12 @@
     <row r="84" ht="20" customHeight="1">
       <c r="A84" s="9" t="inlineStr">
         <is>
-          <t>POC</t>
+          <t>Small</t>
         </is>
       </c>
       <c r="B84" s="9" t="inlineStr">
         <is>
-          <t>20 conn (2 threads)</t>
+          <t>100 conn (4 threads)</t>
         </is>
       </c>
       <c r="C84" s="19" t="inlineStr">
@@ -14145,26 +15225,26 @@
         </is>
       </c>
       <c r="D84" s="11" t="n">
-        <v>0</v>
+        <v>6644.96</v>
       </c>
       <c r="E84" s="11" t="n">
-        <v>2730.57</v>
-      </c>
-      <c r="F84" s="21">
+        <v>8090.44</v>
+      </c>
+      <c r="F84" s="17">
         <f>IF(D84&gt;0, (E84-D84)/D84, 0)</f>
         <v/>
       </c>
       <c r="G84" s="11" t="n">
-        <v>0</v>
+        <v>17.27</v>
       </c>
       <c r="H84" s="11" t="n">
-        <v>7.49</v>
+        <v>14.58</v>
       </c>
       <c r="I84" s="11" t="n">
-        <v>0</v>
+        <v>45.57</v>
       </c>
       <c r="J84" s="11" t="n">
-        <v>14.34</v>
+        <v>39.91</v>
       </c>
       <c r="K84" s="13" t="n">
         <v>0</v>
@@ -14176,12 +15256,12 @@
     <row r="85" ht="20" customHeight="1">
       <c r="A85" s="14" t="inlineStr">
         <is>
-          <t>POC</t>
+          <t>Small</t>
         </is>
       </c>
       <c r="B85" s="14" t="inlineStr">
         <is>
-          <t>20 conn (2 threads)</t>
+          <t>100 conn (4 threads)</t>
         </is>
       </c>
       <c r="C85" s="20" t="inlineStr">
@@ -14190,32 +15270,572 @@
         </is>
       </c>
       <c r="D85" s="16" t="n">
-        <v>0</v>
+        <v>4886.8</v>
       </c>
       <c r="E85" s="16" t="n">
-        <v>1714.31</v>
-      </c>
-      <c r="F85" s="22">
+        <v>5673.3</v>
+      </c>
+      <c r="F85" s="17">
         <f>IF(D85&gt;0, (E85-D85)/D85, 0)</f>
         <v/>
       </c>
       <c r="G85" s="16" t="n">
-        <v>0</v>
+        <v>24.8</v>
       </c>
       <c r="H85" s="16" t="n">
-        <v>14.15</v>
+        <v>20.05</v>
       </c>
       <c r="I85" s="16" t="n">
-        <v>0</v>
+        <v>72.48999999999999</v>
       </c>
       <c r="J85" s="16" t="n">
-        <v>38.23</v>
+        <v>52.46</v>
       </c>
       <c r="K85" s="18" t="n">
         <v>0</v>
       </c>
       <c r="L85" s="18" t="n">
         <v>0</v>
+      </c>
+    </row>
+    <row r="86" ht="20" customHeight="1">
+      <c r="A86" s="9" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="B86" s="9" t="inlineStr">
+        <is>
+          <t>500 conn (8 threads)</t>
+        </is>
+      </c>
+      <c r="C86" s="19" t="inlineStr">
+        <is>
+          <t>1table</t>
+        </is>
+      </c>
+      <c r="D86" s="11" t="n">
+        <v>12337.62</v>
+      </c>
+      <c r="E86" s="11" t="n">
+        <v>15039.32</v>
+      </c>
+      <c r="F86" s="17">
+        <f>IF(D86&gt;0, (E86-D86)/D86, 0)</f>
+        <v/>
+      </c>
+      <c r="G86" s="11" t="n">
+        <v>44.58</v>
+      </c>
+      <c r="H86" s="11" t="n">
+        <v>34.36</v>
+      </c>
+      <c r="I86" s="11" t="n">
+        <v>114.27</v>
+      </c>
+      <c r="J86" s="11" t="n">
+        <v>73.95</v>
+      </c>
+      <c r="K86" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="L86" s="13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="87" ht="20" customHeight="1">
+      <c r="A87" s="14" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="B87" s="14" t="inlineStr">
+        <is>
+          <t>500 conn (8 threads)</t>
+        </is>
+      </c>
+      <c r="C87" s="20" t="inlineStr">
+        <is>
+          <t>2table</t>
+        </is>
+      </c>
+      <c r="D87" s="16" t="n">
+        <v>7837.77</v>
+      </c>
+      <c r="E87" s="16" t="n">
+        <v>9655.32</v>
+      </c>
+      <c r="F87" s="17">
+        <f>IF(D87&gt;0, (E87-D87)/D87, 0)</f>
+        <v/>
+      </c>
+      <c r="G87" s="16" t="n">
+        <v>73.29000000000001</v>
+      </c>
+      <c r="H87" s="16" t="n">
+        <v>53.01</v>
+      </c>
+      <c r="I87" s="16" t="n">
+        <v>204.06</v>
+      </c>
+      <c r="J87" s="16" t="n">
+        <v>110.14</v>
+      </c>
+      <c r="K87" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="L87" s="18" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="88" ht="20" customHeight="1">
+      <c r="A88" s="9" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="B88" s="9" t="inlineStr">
+        <is>
+          <t>500 conn (8 threads)</t>
+        </is>
+      </c>
+      <c r="C88" s="19" t="inlineStr">
+        <is>
+          <t>3table</t>
+        </is>
+      </c>
+      <c r="D88" s="11" t="n">
+        <v>6595.58</v>
+      </c>
+      <c r="E88" s="11" t="n">
+        <v>7891.13</v>
+      </c>
+      <c r="F88" s="17">
+        <f>IF(D88&gt;0, (E88-D88)/D88, 0)</f>
+        <v/>
+      </c>
+      <c r="G88" s="11" t="n">
+        <v>84.16</v>
+      </c>
+      <c r="H88" s="11" t="n">
+        <v>65.34999999999999</v>
+      </c>
+      <c r="I88" s="11" t="n">
+        <v>220.65</v>
+      </c>
+      <c r="J88" s="11" t="n">
+        <v>138.86</v>
+      </c>
+      <c r="K88" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="L88" s="13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="89" ht="20" customHeight="1">
+      <c r="A89" s="14" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="B89" s="14" t="inlineStr">
+        <is>
+          <t>500 conn (8 threads)</t>
+        </is>
+      </c>
+      <c r="C89" s="20" t="inlineStr">
+        <is>
+          <t>4table</t>
+        </is>
+      </c>
+      <c r="D89" s="16" t="n">
+        <v>4839.8</v>
+      </c>
+      <c r="E89" s="16" t="n">
+        <v>5522.55</v>
+      </c>
+      <c r="F89" s="17">
+        <f>IF(D89&gt;0, (E89-D89)/D89, 0)</f>
+        <v/>
+      </c>
+      <c r="G89" s="16" t="n">
+        <v>120.17</v>
+      </c>
+      <c r="H89" s="16" t="n">
+        <v>92.31</v>
+      </c>
+      <c r="I89" s="16" t="n">
+        <v>335.52</v>
+      </c>
+      <c r="J89" s="16" t="n">
+        <v>188.89</v>
+      </c>
+      <c r="K89" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="L89" s="18" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="90" ht="20" customHeight="1">
+      <c r="A90" s="9" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="B90" s="9" t="inlineStr">
+        <is>
+          <t>2,000 conn (8 threads)</t>
+        </is>
+      </c>
+      <c r="C90" s="19" t="inlineStr">
+        <is>
+          <t>1table</t>
+        </is>
+      </c>
+      <c r="D90" s="11" t="n">
+        <v>12115.97</v>
+      </c>
+      <c r="E90" s="11" t="n">
+        <v>15198.4</v>
+      </c>
+      <c r="F90" s="17">
+        <f>IF(D90&gt;0, (E90-D90)/D90, 0)</f>
+        <v/>
+      </c>
+      <c r="G90" s="11" t="n">
+        <v>167.56</v>
+      </c>
+      <c r="H90" s="11" t="n">
+        <v>131.98</v>
+      </c>
+      <c r="I90" s="11" t="n">
+        <v>327.38</v>
+      </c>
+      <c r="J90" s="11" t="n">
+        <v>217.8</v>
+      </c>
+      <c r="K90" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="L90" s="13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="91" ht="20" customHeight="1">
+      <c r="A91" s="14" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="B91" s="14" t="inlineStr">
+        <is>
+          <t>2,000 conn (8 threads)</t>
+        </is>
+      </c>
+      <c r="C91" s="20" t="inlineStr">
+        <is>
+          <t>2table</t>
+        </is>
+      </c>
+      <c r="D91" s="16" t="n">
+        <v>7718.06</v>
+      </c>
+      <c r="E91" s="16" t="n">
+        <v>9623.299999999999</v>
+      </c>
+      <c r="F91" s="17">
+        <f>IF(D91&gt;0, (E91-D91)/D91, 0)</f>
+        <v/>
+      </c>
+      <c r="G91" s="16" t="n">
+        <v>262.92</v>
+      </c>
+      <c r="H91" s="16" t="n">
+        <v>208.16</v>
+      </c>
+      <c r="I91" s="16" t="n">
+        <v>518.8</v>
+      </c>
+      <c r="J91" s="16" t="n">
+        <v>347.05</v>
+      </c>
+      <c r="K91" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="L91" s="18" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="92" ht="20" customHeight="1">
+      <c r="A92" s="9" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="B92" s="9" t="inlineStr">
+        <is>
+          <t>2,000 conn (8 threads)</t>
+        </is>
+      </c>
+      <c r="C92" s="19" t="inlineStr">
+        <is>
+          <t>3table</t>
+        </is>
+      </c>
+      <c r="D92" s="11" t="n">
+        <v>6492.29</v>
+      </c>
+      <c r="E92" s="11" t="n">
+        <v>7846.1</v>
+      </c>
+      <c r="F92" s="17">
+        <f>IF(D92&gt;0, (E92-D92)/D92, 0)</f>
+        <v/>
+      </c>
+      <c r="G92" s="11" t="n">
+        <v>312.14</v>
+      </c>
+      <c r="H92" s="11" t="n">
+        <v>255.54</v>
+      </c>
+      <c r="I92" s="11" t="n">
+        <v>602.03</v>
+      </c>
+      <c r="J92" s="11" t="n">
+        <v>420.46</v>
+      </c>
+      <c r="K92" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="L92" s="13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="93" ht="20" customHeight="1">
+      <c r="A93" s="14" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="B93" s="14" t="inlineStr">
+        <is>
+          <t>2,000 conn (8 threads)</t>
+        </is>
+      </c>
+      <c r="C93" s="20" t="inlineStr">
+        <is>
+          <t>4table</t>
+        </is>
+      </c>
+      <c r="D93" s="16" t="n">
+        <v>4791.45</v>
+      </c>
+      <c r="E93" s="16" t="n">
+        <v>5514.66</v>
+      </c>
+      <c r="F93" s="17">
+        <f>IF(D93&gt;0, (E93-D93)/D93, 0)</f>
+        <v/>
+      </c>
+      <c r="G93" s="16" t="n">
+        <v>420.86</v>
+      </c>
+      <c r="H93" s="16" t="n">
+        <v>363.19</v>
+      </c>
+      <c r="I93" s="16" t="n">
+        <v>792.87</v>
+      </c>
+      <c r="J93" s="16" t="n">
+        <v>589.5700000000001</v>
+      </c>
+      <c r="K93" s="23" t="n">
+        <v>352</v>
+      </c>
+      <c r="L93" s="23" t="n">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="94" ht="20" customHeight="1">
+      <c r="A94" s="9" t="inlineStr">
+        <is>
+          <t>Stress</t>
+        </is>
+      </c>
+      <c r="B94" s="9" t="inlineStr">
+        <is>
+          <t>10,000 conn (16 threads)</t>
+        </is>
+      </c>
+      <c r="C94" s="19" t="inlineStr">
+        <is>
+          <t>1table</t>
+        </is>
+      </c>
+      <c r="D94" s="11" t="n">
+        <v>11841.08</v>
+      </c>
+      <c r="E94" s="11" t="n">
+        <v>14907.18</v>
+      </c>
+      <c r="F94" s="17">
+        <f>IF(D94&gt;0, (E94-D94)/D94, 0)</f>
+        <v/>
+      </c>
+      <c r="G94" s="11" t="n">
+        <v>838.95</v>
+      </c>
+      <c r="H94" s="11" t="n">
+        <v>669.76</v>
+      </c>
+      <c r="I94" s="11" t="n">
+        <v>1226.74</v>
+      </c>
+      <c r="J94" s="11" t="n">
+        <v>946.48</v>
+      </c>
+      <c r="K94" s="23" t="n">
+        <v>116310</v>
+      </c>
+      <c r="L94" s="23" t="n">
+        <v>688</v>
+      </c>
+    </row>
+    <row r="95" ht="20" customHeight="1">
+      <c r="A95" s="14" t="inlineStr">
+        <is>
+          <t>Stress</t>
+        </is>
+      </c>
+      <c r="B95" s="14" t="inlineStr">
+        <is>
+          <t>10,000 conn (16 threads)</t>
+        </is>
+      </c>
+      <c r="C95" s="20" t="inlineStr">
+        <is>
+          <t>2table</t>
+        </is>
+      </c>
+      <c r="D95" s="16" t="n">
+        <v>7614.33</v>
+      </c>
+      <c r="E95" s="16" t="n">
+        <v>9532.92</v>
+      </c>
+      <c r="F95" s="17">
+        <f>IF(D95&gt;0, (E95-D95)/D95, 0)</f>
+        <v/>
+      </c>
+      <c r="G95" s="16" t="n">
+        <v>1298.96</v>
+      </c>
+      <c r="H95" s="16" t="n">
+        <v>1042.03</v>
+      </c>
+      <c r="I95" s="16" t="n">
+        <v>1658.4</v>
+      </c>
+      <c r="J95" s="16" t="n">
+        <v>1541.74</v>
+      </c>
+      <c r="K95" s="23" t="n">
+        <v>261650</v>
+      </c>
+      <c r="L95" s="23" t="n">
+        <v>199775</v>
+      </c>
+    </row>
+    <row r="96" ht="20" customHeight="1">
+      <c r="A96" s="9" t="inlineStr">
+        <is>
+          <t>Stress</t>
+        </is>
+      </c>
+      <c r="B96" s="9" t="inlineStr">
+        <is>
+          <t>10,000 conn (16 threads)</t>
+        </is>
+      </c>
+      <c r="C96" s="19" t="inlineStr">
+        <is>
+          <t>3table</t>
+        </is>
+      </c>
+      <c r="D96" s="11" t="n">
+        <v>6494.12</v>
+      </c>
+      <c r="E96" s="11" t="n">
+        <v>7800.7</v>
+      </c>
+      <c r="F96" s="17">
+        <f>IF(D96&gt;0, (E96-D96)/D96, 0)</f>
+        <v/>
+      </c>
+      <c r="G96" s="11" t="n">
+        <v>1483.81</v>
+      </c>
+      <c r="H96" s="11" t="n">
+        <v>1202.15</v>
+      </c>
+      <c r="I96" s="11" t="n">
+        <v>1874.12</v>
+      </c>
+      <c r="J96" s="11" t="n">
+        <v>1815.01</v>
+      </c>
+      <c r="K96" s="23" t="n">
+        <v>1963204</v>
+      </c>
+      <c r="L96" s="23" t="n">
+        <v>3082224</v>
+      </c>
+    </row>
+    <row r="97" ht="20" customHeight="1">
+      <c r="A97" s="14" t="inlineStr">
+        <is>
+          <t>Stress</t>
+        </is>
+      </c>
+      <c r="B97" s="14" t="inlineStr">
+        <is>
+          <t>10,000 conn (16 threads)</t>
+        </is>
+      </c>
+      <c r="C97" s="20" t="inlineStr">
+        <is>
+          <t>4table</t>
+        </is>
+      </c>
+      <c r="D97" s="16" t="n">
+        <v>4772.92</v>
+      </c>
+      <c r="E97" s="16" t="n">
+        <v>5542.99</v>
+      </c>
+      <c r="F97" s="17">
+        <f>IF(D97&gt;0, (E97-D97)/D97, 0)</f>
+        <v/>
+      </c>
+      <c r="G97" s="16" t="n">
+        <v>1598.88</v>
+      </c>
+      <c r="H97" s="16" t="n">
+        <v>1261.41</v>
+      </c>
+      <c r="I97" s="16" t="n">
+        <v>1950.49</v>
+      </c>
+      <c r="J97" s="16" t="n">
+        <v>1876.15</v>
+      </c>
+      <c r="K97" s="23" t="n">
+        <v>12683295</v>
+      </c>
+      <c r="L97" s="23" t="n">
+        <v>10699464</v>
       </c>
     </row>
   </sheetData>
@@ -14237,7 +15857,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L85"/>
+  <dimension ref="A1:L97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="113" customWidth="1" min="1" max="1"/>
@@ -16307,12 +17927,12 @@
     <row r="78" ht="20" customHeight="1">
       <c r="A78" s="9" t="inlineStr">
         <is>
-          <t>Min</t>
+          <t>POC</t>
         </is>
       </c>
       <c r="B78" s="9" t="inlineStr">
         <is>
-          <t>100 conn (2 threads)</t>
+          <t>20 conn (2 threads)</t>
         </is>
       </c>
       <c r="C78" s="19" t="inlineStr">
@@ -16321,26 +17941,26 @@
         </is>
       </c>
       <c r="D78" s="11" t="n">
-        <v>7123.85</v>
+        <v>9833.5</v>
       </c>
       <c r="E78" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="F78" s="12">
+        <v>12905.17</v>
+      </c>
+      <c r="F78" s="17">
         <f>IF(D78&gt;0, (E78-D78)/D78, 0)</f>
         <v/>
       </c>
       <c r="G78" s="11" t="n">
-        <v>14.05</v>
+        <v>2.81</v>
       </c>
       <c r="H78" s="11" t="n">
-        <v>0</v>
+        <v>1.74</v>
       </c>
       <c r="I78" s="11" t="n">
-        <v>0</v>
+        <v>4.21</v>
       </c>
       <c r="J78" s="11" t="n">
-        <v>0</v>
+        <v>3.29</v>
       </c>
       <c r="K78" s="13" t="n">
         <v>0</v>
@@ -16352,12 +17972,12 @@
     <row r="79" ht="20" customHeight="1">
       <c r="A79" s="14" t="inlineStr">
         <is>
-          <t>Min</t>
+          <t>POC</t>
         </is>
       </c>
       <c r="B79" s="14" t="inlineStr">
         <is>
-          <t>100 conn (2 threads)</t>
+          <t>20 conn (2 threads)</t>
         </is>
       </c>
       <c r="C79" s="20" t="inlineStr">
@@ -16366,26 +17986,26 @@
         </is>
       </c>
       <c r="D79" s="16" t="n">
-        <v>4962.62</v>
+        <v>5134.47</v>
       </c>
       <c r="E79" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="F79" s="12">
+        <v>6051.09</v>
+      </c>
+      <c r="F79" s="17">
         <f>IF(D79&gt;0, (E79-D79)/D79, 0)</f>
         <v/>
       </c>
       <c r="G79" s="16" t="n">
-        <v>20.38</v>
+        <v>4.04</v>
       </c>
       <c r="H79" s="16" t="n">
-        <v>0</v>
+        <v>3.46</v>
       </c>
       <c r="I79" s="16" t="n">
-        <v>0</v>
+        <v>6.68</v>
       </c>
       <c r="J79" s="16" t="n">
-        <v>0</v>
+        <v>5.43</v>
       </c>
       <c r="K79" s="18" t="n">
         <v>0</v>
@@ -16397,12 +18017,12 @@
     <row r="80" ht="20" customHeight="1">
       <c r="A80" s="9" t="inlineStr">
         <is>
-          <t>Min</t>
+          <t>POC</t>
         </is>
       </c>
       <c r="B80" s="9" t="inlineStr">
         <is>
-          <t>100 conn (2 threads)</t>
+          <t>20 conn (2 threads)</t>
         </is>
       </c>
       <c r="C80" s="19" t="inlineStr">
@@ -16411,26 +18031,26 @@
         </is>
       </c>
       <c r="D80" s="11" t="n">
-        <v>4008.93</v>
+        <v>4010.5</v>
       </c>
       <c r="E80" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="F80" s="12">
+        <v>4555.75</v>
+      </c>
+      <c r="F80" s="17">
         <f>IF(D80&gt;0, (E80-D80)/D80, 0)</f>
         <v/>
       </c>
       <c r="G80" s="11" t="n">
-        <v>25.09</v>
+        <v>5.13</v>
       </c>
       <c r="H80" s="11" t="n">
-        <v>0</v>
+        <v>4.97</v>
       </c>
       <c r="I80" s="11" t="n">
-        <v>0</v>
+        <v>8.119999999999999</v>
       </c>
       <c r="J80" s="11" t="n">
-        <v>0</v>
+        <v>7.04</v>
       </c>
       <c r="K80" s="13" t="n">
         <v>0</v>
@@ -16442,12 +18062,12 @@
     <row r="81" ht="20" customHeight="1">
       <c r="A81" s="14" t="inlineStr">
         <is>
-          <t>Min</t>
+          <t>POC</t>
         </is>
       </c>
       <c r="B81" s="14" t="inlineStr">
         <is>
-          <t>100 conn (2 threads)</t>
+          <t>20 conn (2 threads)</t>
         </is>
       </c>
       <c r="C81" s="20" t="inlineStr">
@@ -16456,26 +18076,26 @@
         </is>
       </c>
       <c r="D81" s="16" t="n">
-        <v>2818.92</v>
+        <v>2767.17</v>
       </c>
       <c r="E81" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="F81" s="12">
+        <v>3019.23</v>
+      </c>
+      <c r="F81" s="17">
         <f>IF(D81&gt;0, (E81-D81)/D81, 0)</f>
         <v/>
       </c>
       <c r="G81" s="16" t="n">
-        <v>35.83</v>
+        <v>7.38</v>
       </c>
       <c r="H81" s="16" t="n">
-        <v>0</v>
+        <v>6.8</v>
       </c>
       <c r="I81" s="16" t="n">
-        <v>0</v>
+        <v>11.11</v>
       </c>
       <c r="J81" s="16" t="n">
-        <v>0</v>
+        <v>10.17</v>
       </c>
       <c r="K81" s="18" t="n">
         <v>0</v>
@@ -16487,12 +18107,12 @@
     <row r="82" ht="20" customHeight="1">
       <c r="A82" s="9" t="inlineStr">
         <is>
-          <t>POC</t>
+          <t>Small</t>
         </is>
       </c>
       <c r="B82" s="9" t="inlineStr">
         <is>
-          <t>20 conn (2 threads)</t>
+          <t>100 conn (4 threads)</t>
         </is>
       </c>
       <c r="C82" s="19" t="inlineStr">
@@ -16501,26 +18121,26 @@
         </is>
       </c>
       <c r="D82" s="11" t="n">
-        <v>0</v>
+        <v>8021.8</v>
       </c>
       <c r="E82" s="11" t="n">
-        <v>5057.31</v>
-      </c>
-      <c r="F82" s="21">
+        <v>9174.700000000001</v>
+      </c>
+      <c r="F82" s="17">
         <f>IF(D82&gt;0, (E82-D82)/D82, 0)</f>
         <v/>
       </c>
       <c r="G82" s="11" t="n">
-        <v>0</v>
+        <v>35.71</v>
       </c>
       <c r="H82" s="11" t="n">
-        <v>3.97</v>
+        <v>36.19</v>
       </c>
       <c r="I82" s="11" t="n">
-        <v>0</v>
+        <v>161.61</v>
       </c>
       <c r="J82" s="11" t="n">
-        <v>5.25</v>
+        <v>165.33</v>
       </c>
       <c r="K82" s="13" t="n">
         <v>0</v>
@@ -16532,12 +18152,12 @@
     <row r="83" ht="20" customHeight="1">
       <c r="A83" s="14" t="inlineStr">
         <is>
-          <t>POC</t>
+          <t>Small</t>
         </is>
       </c>
       <c r="B83" s="14" t="inlineStr">
         <is>
-          <t>20 conn (2 threads)</t>
+          <t>100 conn (4 threads)</t>
         </is>
       </c>
       <c r="C83" s="20" t="inlineStr">
@@ -16546,26 +18166,26 @@
         </is>
       </c>
       <c r="D83" s="16" t="n">
-        <v>0</v>
+        <v>5094.64</v>
       </c>
       <c r="E83" s="16" t="n">
-        <v>3715.69</v>
-      </c>
-      <c r="F83" s="22">
+        <v>5548.59</v>
+      </c>
+      <c r="F83" s="17">
         <f>IF(D83&gt;0, (E83-D83)/D83, 0)</f>
         <v/>
       </c>
       <c r="G83" s="16" t="n">
-        <v>0</v>
+        <v>29.08</v>
       </c>
       <c r="H83" s="16" t="n">
-        <v>5.43</v>
+        <v>29.09</v>
       </c>
       <c r="I83" s="16" t="n">
-        <v>0</v>
+        <v>105.09</v>
       </c>
       <c r="J83" s="16" t="n">
-        <v>7.29</v>
+        <v>110.96</v>
       </c>
       <c r="K83" s="18" t="n">
         <v>0</v>
@@ -16577,12 +18197,12 @@
     <row r="84" ht="20" customHeight="1">
       <c r="A84" s="9" t="inlineStr">
         <is>
-          <t>POC</t>
+          <t>Small</t>
         </is>
       </c>
       <c r="B84" s="9" t="inlineStr">
         <is>
-          <t>20 conn (2 threads)</t>
+          <t>100 conn (4 threads)</t>
         </is>
       </c>
       <c r="C84" s="19" t="inlineStr">
@@ -16591,26 +18211,26 @@
         </is>
       </c>
       <c r="D84" s="11" t="n">
-        <v>0</v>
+        <v>4174.7</v>
       </c>
       <c r="E84" s="11" t="n">
-        <v>3114.51</v>
-      </c>
-      <c r="F84" s="21">
+        <v>4450.67</v>
+      </c>
+      <c r="F84" s="17">
         <f>IF(D84&gt;0, (E84-D84)/D84, 0)</f>
         <v/>
       </c>
       <c r="G84" s="11" t="n">
-        <v>0</v>
+        <v>29.86</v>
       </c>
       <c r="H84" s="11" t="n">
-        <v>6.54</v>
+        <v>29.71</v>
       </c>
       <c r="I84" s="11" t="n">
-        <v>0</v>
+        <v>88.54000000000001</v>
       </c>
       <c r="J84" s="11" t="n">
-        <v>8.619999999999999</v>
+        <v>94.8</v>
       </c>
       <c r="K84" s="13" t="n">
         <v>0</v>
@@ -16622,12 +18242,12 @@
     <row r="85" ht="20" customHeight="1">
       <c r="A85" s="14" t="inlineStr">
         <is>
-          <t>POC</t>
+          <t>Small</t>
         </is>
       </c>
       <c r="B85" s="14" t="inlineStr">
         <is>
-          <t>20 conn (2 threads)</t>
+          <t>100 conn (4 threads)</t>
         </is>
       </c>
       <c r="C85" s="20" t="inlineStr">
@@ -16636,32 +18256,572 @@
         </is>
       </c>
       <c r="D85" s="16" t="n">
-        <v>0</v>
+        <v>2819.71</v>
       </c>
       <c r="E85" s="16" t="n">
-        <v>2335.17</v>
-      </c>
-      <c r="F85" s="22">
+        <v>2926.63</v>
+      </c>
+      <c r="F85" s="17">
         <f>IF(D85&gt;0, (E85-D85)/D85, 0)</f>
         <v/>
       </c>
       <c r="G85" s="16" t="n">
-        <v>0</v>
+        <v>39.13</v>
       </c>
       <c r="H85" s="16" t="n">
-        <v>8.58</v>
+        <v>38.59</v>
       </c>
       <c r="I85" s="16" t="n">
-        <v>0</v>
+        <v>93.86</v>
       </c>
       <c r="J85" s="16" t="n">
-        <v>11.35</v>
+        <v>97.75</v>
       </c>
       <c r="K85" s="18" t="n">
         <v>0</v>
       </c>
       <c r="L85" s="18" t="n">
         <v>0</v>
+      </c>
+    </row>
+    <row r="86" ht="20" customHeight="1">
+      <c r="A86" s="9" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="B86" s="9" t="inlineStr">
+        <is>
+          <t>500 conn (8 threads)</t>
+        </is>
+      </c>
+      <c r="C86" s="19" t="inlineStr">
+        <is>
+          <t>1table</t>
+        </is>
+      </c>
+      <c r="D86" s="11" t="n">
+        <v>7863.88</v>
+      </c>
+      <c r="E86" s="11" t="n">
+        <v>9055.059999999999</v>
+      </c>
+      <c r="F86" s="17">
+        <f>IF(D86&gt;0, (E86-D86)/D86, 0)</f>
+        <v/>
+      </c>
+      <c r="G86" s="11" t="n">
+        <v>123.6</v>
+      </c>
+      <c r="H86" s="11" t="n">
+        <v>65.36</v>
+      </c>
+      <c r="I86" s="11" t="n">
+        <v>524.22</v>
+      </c>
+      <c r="J86" s="11" t="n">
+        <v>184.13</v>
+      </c>
+      <c r="K86" s="23" t="n">
+        <v>2728</v>
+      </c>
+      <c r="L86" s="13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="87" ht="20" customHeight="1">
+      <c r="A87" s="14" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="B87" s="14" t="inlineStr">
+        <is>
+          <t>500 conn (8 threads)</t>
+        </is>
+      </c>
+      <c r="C87" s="20" t="inlineStr">
+        <is>
+          <t>2table</t>
+        </is>
+      </c>
+      <c r="D87" s="16" t="n">
+        <v>5006.91</v>
+      </c>
+      <c r="E87" s="16" t="n">
+        <v>5461.98</v>
+      </c>
+      <c r="F87" s="17">
+        <f>IF(D87&gt;0, (E87-D87)/D87, 0)</f>
+        <v/>
+      </c>
+      <c r="G87" s="16" t="n">
+        <v>161.72</v>
+      </c>
+      <c r="H87" s="16" t="n">
+        <v>101.1</v>
+      </c>
+      <c r="I87" s="16" t="n">
+        <v>662.75</v>
+      </c>
+      <c r="J87" s="16" t="n">
+        <v>259.71</v>
+      </c>
+      <c r="K87" s="23" t="n">
+        <v>10939</v>
+      </c>
+      <c r="L87" s="18" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="88" ht="20" customHeight="1">
+      <c r="A88" s="9" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="B88" s="9" t="inlineStr">
+        <is>
+          <t>500 conn (8 threads)</t>
+        </is>
+      </c>
+      <c r="C88" s="19" t="inlineStr">
+        <is>
+          <t>3table</t>
+        </is>
+      </c>
+      <c r="D88" s="11" t="n">
+        <v>4097.01</v>
+      </c>
+      <c r="E88" s="11" t="n">
+        <v>4379.97</v>
+      </c>
+      <c r="F88" s="17">
+        <f>IF(D88&gt;0, (E88-D88)/D88, 0)</f>
+        <v/>
+      </c>
+      <c r="G88" s="11" t="n">
+        <v>179.32</v>
+      </c>
+      <c r="H88" s="11" t="n">
+        <v>125.06</v>
+      </c>
+      <c r="I88" s="11" t="n">
+        <v>703.75</v>
+      </c>
+      <c r="J88" s="11" t="n">
+        <v>316.69</v>
+      </c>
+      <c r="K88" s="23" t="n">
+        <v>15303</v>
+      </c>
+      <c r="L88" s="13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="89" ht="20" customHeight="1">
+      <c r="A89" s="14" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="B89" s="14" t="inlineStr">
+        <is>
+          <t>500 conn (8 threads)</t>
+        </is>
+      </c>
+      <c r="C89" s="20" t="inlineStr">
+        <is>
+          <t>4table</t>
+        </is>
+      </c>
+      <c r="D89" s="16" t="n">
+        <v>2801.2</v>
+      </c>
+      <c r="E89" s="16" t="n">
+        <v>2887.66</v>
+      </c>
+      <c r="F89" s="17">
+        <f>IF(D89&gt;0, (E89-D89)/D89, 0)</f>
+        <v/>
+      </c>
+      <c r="G89" s="16" t="n">
+        <v>214.1</v>
+      </c>
+      <c r="H89" s="16" t="n">
+        <v>188.81</v>
+      </c>
+      <c r="I89" s="16" t="n">
+        <v>771.0700000000001</v>
+      </c>
+      <c r="J89" s="16" t="n">
+        <v>474.44</v>
+      </c>
+      <c r="K89" s="23" t="n">
+        <v>24329</v>
+      </c>
+      <c r="L89" s="23" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="90" ht="20" customHeight="1">
+      <c r="A90" s="9" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="B90" s="9" t="inlineStr">
+        <is>
+          <t>2,000 conn (8 threads)</t>
+        </is>
+      </c>
+      <c r="C90" s="19" t="inlineStr">
+        <is>
+          <t>1table</t>
+        </is>
+      </c>
+      <c r="D90" s="11" t="n">
+        <v>7817.09</v>
+      </c>
+      <c r="E90" s="11" t="n">
+        <v>8987.5</v>
+      </c>
+      <c r="F90" s="17">
+        <f>IF(D90&gt;0, (E90-D90)/D90, 0)</f>
+        <v/>
+      </c>
+      <c r="G90" s="11" t="n">
+        <v>240.46</v>
+      </c>
+      <c r="H90" s="11" t="n">
+        <v>256.57</v>
+      </c>
+      <c r="I90" s="11" t="n">
+        <v>903.79</v>
+      </c>
+      <c r="J90" s="11" t="n">
+        <v>697.41</v>
+      </c>
+      <c r="K90" s="23" t="n">
+        <v>321629</v>
+      </c>
+      <c r="L90" s="23" t="n">
+        <v>1794</v>
+      </c>
+    </row>
+    <row r="91" ht="20" customHeight="1">
+      <c r="A91" s="14" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="B91" s="14" t="inlineStr">
+        <is>
+          <t>2,000 conn (8 threads)</t>
+        </is>
+      </c>
+      <c r="C91" s="20" t="inlineStr">
+        <is>
+          <t>2table</t>
+        </is>
+      </c>
+      <c r="D91" s="16" t="n">
+        <v>4966.76</v>
+      </c>
+      <c r="E91" s="16" t="n">
+        <v>5420.53</v>
+      </c>
+      <c r="F91" s="17">
+        <f>IF(D91&gt;0, (E91-D91)/D91, 0)</f>
+        <v/>
+      </c>
+      <c r="G91" s="16" t="n">
+        <v>306.27</v>
+      </c>
+      <c r="H91" s="16" t="n">
+        <v>406.82</v>
+      </c>
+      <c r="I91" s="16" t="n">
+        <v>1088.88</v>
+      </c>
+      <c r="J91" s="16" t="n">
+        <v>1085.96</v>
+      </c>
+      <c r="K91" s="23" t="n">
+        <v>344562</v>
+      </c>
+      <c r="L91" s="23" t="n">
+        <v>44483</v>
+      </c>
+    </row>
+    <row r="92" ht="20" customHeight="1">
+      <c r="A92" s="9" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="B92" s="9" t="inlineStr">
+        <is>
+          <t>2,000 conn (8 threads)</t>
+        </is>
+      </c>
+      <c r="C92" s="19" t="inlineStr">
+        <is>
+          <t>3table</t>
+        </is>
+      </c>
+      <c r="D92" s="11" t="n">
+        <v>4073.84</v>
+      </c>
+      <c r="E92" s="11" t="n">
+        <v>4365.94</v>
+      </c>
+      <c r="F92" s="17">
+        <f>IF(D92&gt;0, (E92-D92)/D92, 0)</f>
+        <v/>
+      </c>
+      <c r="G92" s="11" t="n">
+        <v>340.02</v>
+      </c>
+      <c r="H92" s="11" t="n">
+        <v>479.93</v>
+      </c>
+      <c r="I92" s="11" t="n">
+        <v>1182.01</v>
+      </c>
+      <c r="J92" s="11" t="n">
+        <v>1256.59</v>
+      </c>
+      <c r="K92" s="23" t="n">
+        <v>372325</v>
+      </c>
+      <c r="L92" s="23" t="n">
+        <v>108868</v>
+      </c>
+    </row>
+    <row r="93" ht="20" customHeight="1">
+      <c r="A93" s="14" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="B93" s="14" t="inlineStr">
+        <is>
+          <t>2,000 conn (8 threads)</t>
+        </is>
+      </c>
+      <c r="C93" s="20" t="inlineStr">
+        <is>
+          <t>4table</t>
+        </is>
+      </c>
+      <c r="D93" s="16" t="n">
+        <v>2780.53</v>
+      </c>
+      <c r="E93" s="16" t="n">
+        <v>2879.32</v>
+      </c>
+      <c r="F93" s="17">
+        <f>IF(D93&gt;0, (E93-D93)/D93, 0)</f>
+        <v/>
+      </c>
+      <c r="G93" s="16" t="n">
+        <v>401.59</v>
+      </c>
+      <c r="H93" s="16" t="n">
+        <v>613.77</v>
+      </c>
+      <c r="I93" s="16" t="n">
+        <v>1317.18</v>
+      </c>
+      <c r="J93" s="16" t="n">
+        <v>1536.28</v>
+      </c>
+      <c r="K93" s="23" t="n">
+        <v>433562</v>
+      </c>
+      <c r="L93" s="23" t="n">
+        <v>346282</v>
+      </c>
+    </row>
+    <row r="94" ht="20" customHeight="1">
+      <c r="A94" s="9" t="inlineStr">
+        <is>
+          <t>Stress</t>
+        </is>
+      </c>
+      <c r="B94" s="9" t="inlineStr">
+        <is>
+          <t>10,000 conn (16 threads)</t>
+        </is>
+      </c>
+      <c r="C94" s="19" t="inlineStr">
+        <is>
+          <t>1table</t>
+        </is>
+      </c>
+      <c r="D94" s="11" t="n">
+        <v>7751.62</v>
+      </c>
+      <c r="E94" s="11" t="n">
+        <v>8868.889999999999</v>
+      </c>
+      <c r="F94" s="17">
+        <f>IF(D94&gt;0, (E94-D94)/D94, 0)</f>
+        <v/>
+      </c>
+      <c r="G94" s="11" t="n">
+        <v>454.37</v>
+      </c>
+      <c r="H94" s="11" t="n">
+        <v>722.99</v>
+      </c>
+      <c r="I94" s="11" t="n">
+        <v>1523.2</v>
+      </c>
+      <c r="J94" s="11" t="n">
+        <v>1752.74</v>
+      </c>
+      <c r="K94" s="23" t="n">
+        <v>5944646</v>
+      </c>
+      <c r="L94" s="23" t="n">
+        <v>8887305</v>
+      </c>
+    </row>
+    <row r="95" ht="20" customHeight="1">
+      <c r="A95" s="14" t="inlineStr">
+        <is>
+          <t>Stress</t>
+        </is>
+      </c>
+      <c r="B95" s="14" t="inlineStr">
+        <is>
+          <t>10,000 conn (16 threads)</t>
+        </is>
+      </c>
+      <c r="C95" s="20" t="inlineStr">
+        <is>
+          <t>2table</t>
+        </is>
+      </c>
+      <c r="D95" s="16" t="n">
+        <v>4903.47</v>
+      </c>
+      <c r="E95" s="16" t="n">
+        <v>5333.35</v>
+      </c>
+      <c r="F95" s="17">
+        <f>IF(D95&gt;0, (E95-D95)/D95, 0)</f>
+        <v/>
+      </c>
+      <c r="G95" s="16" t="n">
+        <v>553.92</v>
+      </c>
+      <c r="H95" s="16" t="n">
+        <v>834.35</v>
+      </c>
+      <c r="I95" s="16" t="n">
+        <v>1653.43</v>
+      </c>
+      <c r="J95" s="16" t="n">
+        <v>1830.25</v>
+      </c>
+      <c r="K95" s="23" t="n">
+        <v>6644766</v>
+      </c>
+      <c r="L95" s="23" t="n">
+        <v>10919810</v>
+      </c>
+    </row>
+    <row r="96" ht="20" customHeight="1">
+      <c r="A96" s="9" t="inlineStr">
+        <is>
+          <t>Stress</t>
+        </is>
+      </c>
+      <c r="B96" s="9" t="inlineStr">
+        <is>
+          <t>10,000 conn (16 threads)</t>
+        </is>
+      </c>
+      <c r="C96" s="19" t="inlineStr">
+        <is>
+          <t>3table</t>
+        </is>
+      </c>
+      <c r="D96" s="11" t="n">
+        <v>3984.6</v>
+      </c>
+      <c r="E96" s="11" t="n">
+        <v>4287.1</v>
+      </c>
+      <c r="F96" s="17">
+        <f>IF(D96&gt;0, (E96-D96)/D96, 0)</f>
+        <v/>
+      </c>
+      <c r="G96" s="11" t="n">
+        <v>592.88</v>
+      </c>
+      <c r="H96" s="11" t="n">
+        <v>870.89</v>
+      </c>
+      <c r="I96" s="11" t="n">
+        <v>1691.32</v>
+      </c>
+      <c r="J96" s="11" t="n">
+        <v>1848.52</v>
+      </c>
+      <c r="K96" s="23" t="n">
+        <v>6434479</v>
+      </c>
+      <c r="L96" s="23" t="n">
+        <v>10843807</v>
+      </c>
+    </row>
+    <row r="97" ht="20" customHeight="1">
+      <c r="A97" s="14" t="inlineStr">
+        <is>
+          <t>Stress</t>
+        </is>
+      </c>
+      <c r="B97" s="14" t="inlineStr">
+        <is>
+          <t>10,000 conn (16 threads)</t>
+        </is>
+      </c>
+      <c r="C97" s="20" t="inlineStr">
+        <is>
+          <t>4table</t>
+        </is>
+      </c>
+      <c r="D97" s="16" t="n">
+        <v>2713.64</v>
+      </c>
+      <c r="E97" s="16" t="n">
+        <v>2825.3</v>
+      </c>
+      <c r="F97" s="17">
+        <f>IF(D97&gt;0, (E97-D97)/D97, 0)</f>
+        <v/>
+      </c>
+      <c r="G97" s="16" t="n">
+        <v>650</v>
+      </c>
+      <c r="H97" s="16" t="n">
+        <v>924.86</v>
+      </c>
+      <c r="I97" s="16" t="n">
+        <v>1738.33</v>
+      </c>
+      <c r="J97" s="16" t="n">
+        <v>1870.71</v>
+      </c>
+      <c r="K97" s="23" t="n">
+        <v>5668213</v>
+      </c>
+      <c r="L97" s="23" t="n">
+        <v>9616149</v>
       </c>
     </row>
   </sheetData>
@@ -16683,7 +18843,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L85"/>
+  <dimension ref="A1:L97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="105" customWidth="1" min="1" max="1"/>
@@ -18753,12 +20913,12 @@
     <row r="78" ht="20" customHeight="1">
       <c r="A78" s="9" t="inlineStr">
         <is>
-          <t>Min</t>
+          <t>POC</t>
         </is>
       </c>
       <c r="B78" s="9" t="inlineStr">
         <is>
-          <t>100 conn (2 threads)</t>
+          <t>20 conn (2 threads)</t>
         </is>
       </c>
       <c r="C78" s="19" t="inlineStr">
@@ -18767,26 +20927,26 @@
         </is>
       </c>
       <c r="D78" s="11" t="n">
-        <v>5708.88</v>
+        <v>9774.09</v>
       </c>
       <c r="E78" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="F78" s="12">
+        <v>12851.51</v>
+      </c>
+      <c r="F78" s="17">
         <f>IF(D78&gt;0, (E78-D78)/D78, 0)</f>
         <v/>
       </c>
       <c r="G78" s="11" t="n">
-        <v>17.63</v>
+        <v>2.21</v>
       </c>
       <c r="H78" s="11" t="n">
-        <v>0</v>
+        <v>1.79</v>
       </c>
       <c r="I78" s="11" t="n">
-        <v>0</v>
+        <v>4.14</v>
       </c>
       <c r="J78" s="11" t="n">
-        <v>0</v>
+        <v>3.49</v>
       </c>
       <c r="K78" s="13" t="n">
         <v>0</v>
@@ -18798,12 +20958,12 @@
     <row r="79" ht="20" customHeight="1">
       <c r="A79" s="14" t="inlineStr">
         <is>
-          <t>Min</t>
+          <t>POC</t>
         </is>
       </c>
       <c r="B79" s="14" t="inlineStr">
         <is>
-          <t>100 conn (2 threads)</t>
+          <t>20 conn (2 threads)</t>
         </is>
       </c>
       <c r="C79" s="20" t="inlineStr">
@@ -18812,26 +20972,26 @@
         </is>
       </c>
       <c r="D79" s="16" t="n">
-        <v>4539.56</v>
+        <v>5122.51</v>
       </c>
       <c r="E79" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="F79" s="12">
+        <v>5946.41</v>
+      </c>
+      <c r="F79" s="17">
         <f>IF(D79&gt;0, (E79-D79)/D79, 0)</f>
         <v/>
       </c>
       <c r="G79" s="16" t="n">
-        <v>22.01</v>
+        <v>4.04</v>
       </c>
       <c r="H79" s="16" t="n">
-        <v>0</v>
+        <v>4.18</v>
       </c>
       <c r="I79" s="16" t="n">
-        <v>0</v>
+        <v>6.51</v>
       </c>
       <c r="J79" s="16" t="n">
-        <v>0</v>
+        <v>5.63</v>
       </c>
       <c r="K79" s="18" t="n">
         <v>0</v>
@@ -18843,12 +21003,12 @@
     <row r="80" ht="20" customHeight="1">
       <c r="A80" s="9" t="inlineStr">
         <is>
-          <t>Min</t>
+          <t>POC</t>
         </is>
       </c>
       <c r="B80" s="9" t="inlineStr">
         <is>
-          <t>100 conn (2 threads)</t>
+          <t>20 conn (2 threads)</t>
         </is>
       </c>
       <c r="C80" s="19" t="inlineStr">
@@ -18857,26 +21017,26 @@
         </is>
       </c>
       <c r="D80" s="11" t="n">
-        <v>3896.54</v>
+        <v>4378.74</v>
       </c>
       <c r="E80" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="F80" s="12">
+        <v>5049.73</v>
+      </c>
+      <c r="F80" s="17">
         <f>IF(D80&gt;0, (E80-D80)/D80, 0)</f>
         <v/>
       </c>
       <c r="G80" s="11" t="n">
-        <v>25.85</v>
+        <v>4.95</v>
       </c>
       <c r="H80" s="11" t="n">
-        <v>0</v>
+        <v>4.12</v>
       </c>
       <c r="I80" s="11" t="n">
-        <v>0</v>
+        <v>7.68</v>
       </c>
       <c r="J80" s="11" t="n">
-        <v>0</v>
+        <v>6.51</v>
       </c>
       <c r="K80" s="13" t="n">
         <v>0</v>
@@ -18888,12 +21048,12 @@
     <row r="81" ht="20" customHeight="1">
       <c r="A81" s="14" t="inlineStr">
         <is>
-          <t>Min</t>
+          <t>POC</t>
         </is>
       </c>
       <c r="B81" s="14" t="inlineStr">
         <is>
-          <t>100 conn (2 threads)</t>
+          <t>20 conn (2 threads)</t>
         </is>
       </c>
       <c r="C81" s="20" t="inlineStr">
@@ -18902,26 +21062,26 @@
         </is>
       </c>
       <c r="D81" s="16" t="n">
-        <v>3256.14</v>
+        <v>3393.85</v>
       </c>
       <c r="E81" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="F81" s="12">
+        <v>3820.8</v>
+      </c>
+      <c r="F81" s="17">
         <f>IF(D81&gt;0, (E81-D81)/D81, 0)</f>
         <v/>
       </c>
       <c r="G81" s="16" t="n">
-        <v>30.69</v>
+        <v>6.07</v>
       </c>
       <c r="H81" s="16" t="n">
-        <v>0</v>
+        <v>5.41</v>
       </c>
       <c r="I81" s="16" t="n">
-        <v>0</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="J81" s="16" t="n">
-        <v>0</v>
+        <v>8.390000000000001</v>
       </c>
       <c r="K81" s="18" t="n">
         <v>0</v>
@@ -18933,12 +21093,12 @@
     <row r="82" ht="20" customHeight="1">
       <c r="A82" s="9" t="inlineStr">
         <is>
-          <t>POC</t>
+          <t>Small</t>
         </is>
       </c>
       <c r="B82" s="9" t="inlineStr">
         <is>
-          <t>20 conn (2 threads)</t>
+          <t>100 conn (4 threads)</t>
         </is>
       </c>
       <c r="C82" s="19" t="inlineStr">
@@ -18947,26 +21107,26 @@
         </is>
       </c>
       <c r="D82" s="11" t="n">
-        <v>0</v>
+        <v>8307.32</v>
       </c>
       <c r="E82" s="11" t="n">
-        <v>4642.41</v>
-      </c>
-      <c r="F82" s="21">
+        <v>9971.76</v>
+      </c>
+      <c r="F82" s="17">
         <f>IF(D82&gt;0, (E82-D82)/D82, 0)</f>
         <v/>
       </c>
       <c r="G82" s="11" t="n">
-        <v>0</v>
+        <v>29.64</v>
       </c>
       <c r="H82" s="11" t="n">
-        <v>4.34</v>
+        <v>25.37</v>
       </c>
       <c r="I82" s="11" t="n">
-        <v>0</v>
+        <v>132.48</v>
       </c>
       <c r="J82" s="11" t="n">
-        <v>6.44</v>
+        <v>115.24</v>
       </c>
       <c r="K82" s="13" t="n">
         <v>0</v>
@@ -18978,12 +21138,12 @@
     <row r="83" ht="20" customHeight="1">
       <c r="A83" s="14" t="inlineStr">
         <is>
-          <t>POC</t>
+          <t>Small</t>
         </is>
       </c>
       <c r="B83" s="14" t="inlineStr">
         <is>
-          <t>20 conn (2 threads)</t>
+          <t>100 conn (4 threads)</t>
         </is>
       </c>
       <c r="C83" s="20" t="inlineStr">
@@ -18992,26 +21152,26 @@
         </is>
       </c>
       <c r="D83" s="16" t="n">
-        <v>0</v>
+        <v>5009.29</v>
       </c>
       <c r="E83" s="16" t="n">
-        <v>3581.48</v>
-      </c>
-      <c r="F83" s="22">
+        <v>5674.41</v>
+      </c>
+      <c r="F83" s="17">
         <f>IF(D83&gt;0, (E83-D83)/D83, 0)</f>
         <v/>
       </c>
       <c r="G83" s="16" t="n">
-        <v>0</v>
+        <v>26.07</v>
       </c>
       <c r="H83" s="16" t="n">
-        <v>5.67</v>
+        <v>24.21</v>
       </c>
       <c r="I83" s="16" t="n">
-        <v>0</v>
+        <v>82.34</v>
       </c>
       <c r="J83" s="16" t="n">
-        <v>7.58</v>
+        <v>80.81</v>
       </c>
       <c r="K83" s="18" t="n">
         <v>0</v>
@@ -19023,12 +21183,12 @@
     <row r="84" ht="20" customHeight="1">
       <c r="A84" s="9" t="inlineStr">
         <is>
-          <t>POC</t>
+          <t>Small</t>
         </is>
       </c>
       <c r="B84" s="9" t="inlineStr">
         <is>
-          <t>20 conn (2 threads)</t>
+          <t>100 conn (4 threads)</t>
         </is>
       </c>
       <c r="C84" s="19" t="inlineStr">
@@ -19037,26 +21197,26 @@
         </is>
       </c>
       <c r="D84" s="11" t="n">
-        <v>0</v>
+        <v>4433.42</v>
       </c>
       <c r="E84" s="11" t="n">
-        <v>3233.34</v>
-      </c>
-      <c r="F84" s="21">
+        <v>4926.66</v>
+      </c>
+      <c r="F84" s="17">
         <f>IF(D84&gt;0, (E84-D84)/D84, 0)</f>
         <v/>
       </c>
       <c r="G84" s="11" t="n">
-        <v>0</v>
+        <v>26.02</v>
       </c>
       <c r="H84" s="11" t="n">
-        <v>6.22</v>
+        <v>24.98</v>
       </c>
       <c r="I84" s="11" t="n">
-        <v>0</v>
+        <v>67.86</v>
       </c>
       <c r="J84" s="11" t="n">
-        <v>8.43</v>
+        <v>72.84</v>
       </c>
       <c r="K84" s="13" t="n">
         <v>0</v>
@@ -19068,12 +21228,12 @@
     <row r="85" ht="20" customHeight="1">
       <c r="A85" s="14" t="inlineStr">
         <is>
-          <t>POC</t>
+          <t>Small</t>
         </is>
       </c>
       <c r="B85" s="14" t="inlineStr">
         <is>
-          <t>20 conn (2 threads)</t>
+          <t>100 conn (4 threads)</t>
         </is>
       </c>
       <c r="C85" s="20" t="inlineStr">
@@ -19082,32 +21242,572 @@
         </is>
       </c>
       <c r="D85" s="16" t="n">
-        <v>0</v>
+        <v>3260.17</v>
       </c>
       <c r="E85" s="16" t="n">
-        <v>2663.06</v>
-      </c>
-      <c r="F85" s="22">
+        <v>3498.43</v>
+      </c>
+      <c r="F85" s="17">
         <f>IF(D85&gt;0, (E85-D85)/D85, 0)</f>
         <v/>
       </c>
       <c r="G85" s="16" t="n">
-        <v>0</v>
+        <v>34.79</v>
       </c>
       <c r="H85" s="16" t="n">
-        <v>7.55</v>
+        <v>33.3</v>
       </c>
       <c r="I85" s="16" t="n">
-        <v>0</v>
+        <v>88.53</v>
       </c>
       <c r="J85" s="16" t="n">
-        <v>10.07</v>
+        <v>88.59</v>
       </c>
       <c r="K85" s="18" t="n">
         <v>0</v>
       </c>
       <c r="L85" s="18" t="n">
         <v>0</v>
+      </c>
+    </row>
+    <row r="86" ht="20" customHeight="1">
+      <c r="A86" s="9" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="B86" s="9" t="inlineStr">
+        <is>
+          <t>500 conn (8 threads)</t>
+        </is>
+      </c>
+      <c r="C86" s="19" t="inlineStr">
+        <is>
+          <t>1table</t>
+        </is>
+      </c>
+      <c r="D86" s="11" t="n">
+        <v>7835.42</v>
+      </c>
+      <c r="E86" s="11" t="n">
+        <v>9423.450000000001</v>
+      </c>
+      <c r="F86" s="17">
+        <f>IF(D86&gt;0, (E86-D86)/D86, 0)</f>
+        <v/>
+      </c>
+      <c r="G86" s="11" t="n">
+        <v>71.06999999999999</v>
+      </c>
+      <c r="H86" s="11" t="n">
+        <v>58.04</v>
+      </c>
+      <c r="I86" s="11" t="n">
+        <v>171.72</v>
+      </c>
+      <c r="J86" s="11" t="n">
+        <v>135.58</v>
+      </c>
+      <c r="K86" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="L86" s="13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="87" ht="20" customHeight="1">
+      <c r="A87" s="14" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="B87" s="14" t="inlineStr">
+        <is>
+          <t>500 conn (8 threads)</t>
+        </is>
+      </c>
+      <c r="C87" s="20" t="inlineStr">
+        <is>
+          <t>2table</t>
+        </is>
+      </c>
+      <c r="D87" s="16" t="n">
+        <v>4840.65</v>
+      </c>
+      <c r="E87" s="16" t="n">
+        <v>5458.07</v>
+      </c>
+      <c r="F87" s="17">
+        <f>IF(D87&gt;0, (E87-D87)/D87, 0)</f>
+        <v/>
+      </c>
+      <c r="G87" s="16" t="n">
+        <v>103.83</v>
+      </c>
+      <c r="H87" s="16" t="n">
+        <v>91.81</v>
+      </c>
+      <c r="I87" s="16" t="n">
+        <v>180.9</v>
+      </c>
+      <c r="J87" s="16" t="n">
+        <v>159.74</v>
+      </c>
+      <c r="K87" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="L87" s="18" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="88" ht="20" customHeight="1">
+      <c r="A88" s="9" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="B88" s="9" t="inlineStr">
+        <is>
+          <t>500 conn (8 threads)</t>
+        </is>
+      </c>
+      <c r="C88" s="19" t="inlineStr">
+        <is>
+          <t>3table</t>
+        </is>
+      </c>
+      <c r="D88" s="11" t="n">
+        <v>4290.63</v>
+      </c>
+      <c r="E88" s="11" t="n">
+        <v>4769.5</v>
+      </c>
+      <c r="F88" s="17">
+        <f>IF(D88&gt;0, (E88-D88)/D88, 0)</f>
+        <v/>
+      </c>
+      <c r="G88" s="11" t="n">
+        <v>116.35</v>
+      </c>
+      <c r="H88" s="11" t="n">
+        <v>104.36</v>
+      </c>
+      <c r="I88" s="11" t="n">
+        <v>195.84</v>
+      </c>
+      <c r="J88" s="11" t="n">
+        <v>174.98</v>
+      </c>
+      <c r="K88" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="L88" s="13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="89" ht="20" customHeight="1">
+      <c r="A89" s="14" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="B89" s="14" t="inlineStr">
+        <is>
+          <t>500 conn (8 threads)</t>
+        </is>
+      </c>
+      <c r="C89" s="20" t="inlineStr">
+        <is>
+          <t>4table</t>
+        </is>
+      </c>
+      <c r="D89" s="16" t="n">
+        <v>3101.37</v>
+      </c>
+      <c r="E89" s="16" t="n">
+        <v>3420.89</v>
+      </c>
+      <c r="F89" s="17">
+        <f>IF(D89&gt;0, (E89-D89)/D89, 0)</f>
+        <v/>
+      </c>
+      <c r="G89" s="16" t="n">
+        <v>160.71</v>
+      </c>
+      <c r="H89" s="16" t="n">
+        <v>144.94</v>
+      </c>
+      <c r="I89" s="16" t="n">
+        <v>260.69</v>
+      </c>
+      <c r="J89" s="16" t="n">
+        <v>231.08</v>
+      </c>
+      <c r="K89" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="L89" s="18" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="90" ht="20" customHeight="1">
+      <c r="A90" s="9" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="B90" s="9" t="inlineStr">
+        <is>
+          <t>2,000 conn (8 threads)</t>
+        </is>
+      </c>
+      <c r="C90" s="19" t="inlineStr">
+        <is>
+          <t>1table</t>
+        </is>
+      </c>
+      <c r="D90" s="11" t="n">
+        <v>7839.57</v>
+      </c>
+      <c r="E90" s="11" t="n">
+        <v>9396.459999999999</v>
+      </c>
+      <c r="F90" s="17">
+        <f>IF(D90&gt;0, (E90-D90)/D90, 0)</f>
+        <v/>
+      </c>
+      <c r="G90" s="11" t="n">
+        <v>255.58</v>
+      </c>
+      <c r="H90" s="11" t="n">
+        <v>212.51</v>
+      </c>
+      <c r="I90" s="11" t="n">
+        <v>333.5</v>
+      </c>
+      <c r="J90" s="11" t="n">
+        <v>281.77</v>
+      </c>
+      <c r="K90" s="23" t="n">
+        <v>66</v>
+      </c>
+      <c r="L90" s="23" t="n">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="91" ht="20" customHeight="1">
+      <c r="A91" s="14" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="B91" s="14" t="inlineStr">
+        <is>
+          <t>2,000 conn (8 threads)</t>
+        </is>
+      </c>
+      <c r="C91" s="20" t="inlineStr">
+        <is>
+          <t>2table</t>
+        </is>
+      </c>
+      <c r="D91" s="16" t="n">
+        <v>4845.02</v>
+      </c>
+      <c r="E91" s="16" t="n">
+        <v>5470.84</v>
+      </c>
+      <c r="F91" s="17">
+        <f>IF(D91&gt;0, (E91-D91)/D91, 0)</f>
+        <v/>
+      </c>
+      <c r="G91" s="16" t="n">
+        <v>411.98</v>
+      </c>
+      <c r="H91" s="16" t="n">
+        <v>363.34</v>
+      </c>
+      <c r="I91" s="16" t="n">
+        <v>513.11</v>
+      </c>
+      <c r="J91" s="16" t="n">
+        <v>447.27</v>
+      </c>
+      <c r="K91" s="23" t="n">
+        <v>225</v>
+      </c>
+      <c r="L91" s="23" t="n">
+        <v>874</v>
+      </c>
+    </row>
+    <row r="92" ht="20" customHeight="1">
+      <c r="A92" s="9" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="B92" s="9" t="inlineStr">
+        <is>
+          <t>2,000 conn (8 threads)</t>
+        </is>
+      </c>
+      <c r="C92" s="19" t="inlineStr">
+        <is>
+          <t>3table</t>
+        </is>
+      </c>
+      <c r="D92" s="11" t="n">
+        <v>4302.66</v>
+      </c>
+      <c r="E92" s="11" t="n">
+        <v>4786.73</v>
+      </c>
+      <c r="F92" s="17">
+        <f>IF(D92&gt;0, (E92-D92)/D92, 0)</f>
+        <v/>
+      </c>
+      <c r="G92" s="11" t="n">
+        <v>463.81</v>
+      </c>
+      <c r="H92" s="11" t="n">
+        <v>415.09</v>
+      </c>
+      <c r="I92" s="11" t="n">
+        <v>573.8200000000001</v>
+      </c>
+      <c r="J92" s="11" t="n">
+        <v>503.8</v>
+      </c>
+      <c r="K92" s="23" t="n">
+        <v>49</v>
+      </c>
+      <c r="L92" s="23" t="n">
+        <v>1106</v>
+      </c>
+    </row>
+    <row r="93" ht="20" customHeight="1">
+      <c r="A93" s="14" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="B93" s="14" t="inlineStr">
+        <is>
+          <t>2,000 conn (8 threads)</t>
+        </is>
+      </c>
+      <c r="C93" s="20" t="inlineStr">
+        <is>
+          <t>4table</t>
+        </is>
+      </c>
+      <c r="D93" s="16" t="n">
+        <v>3103.72</v>
+      </c>
+      <c r="E93" s="16" t="n">
+        <v>3410.87</v>
+      </c>
+      <c r="F93" s="17">
+        <f>IF(D93&gt;0, (E93-D93)/D93, 0)</f>
+        <v/>
+      </c>
+      <c r="G93" s="16" t="n">
+        <v>644.24</v>
+      </c>
+      <c r="H93" s="16" t="n">
+        <v>582.16</v>
+      </c>
+      <c r="I93" s="16" t="n">
+        <v>803.0599999999999</v>
+      </c>
+      <c r="J93" s="16" t="n">
+        <v>693.04</v>
+      </c>
+      <c r="K93" s="23" t="n">
+        <v>309</v>
+      </c>
+      <c r="L93" s="23" t="n">
+        <v>1116</v>
+      </c>
+    </row>
+    <row r="94" ht="20" customHeight="1">
+      <c r="A94" s="9" t="inlineStr">
+        <is>
+          <t>Stress</t>
+        </is>
+      </c>
+      <c r="B94" s="9" t="inlineStr">
+        <is>
+          <t>10,000 conn (16 threads)</t>
+        </is>
+      </c>
+      <c r="C94" s="19" t="inlineStr">
+        <is>
+          <t>1table</t>
+        </is>
+      </c>
+      <c r="D94" s="11" t="n">
+        <v>7720.57</v>
+      </c>
+      <c r="E94" s="11" t="n">
+        <v>9338.24</v>
+      </c>
+      <c r="F94" s="17">
+        <f>IF(D94&gt;0, (E94-D94)/D94, 0)</f>
+        <v/>
+      </c>
+      <c r="G94" s="11" t="n">
+        <v>1057.06</v>
+      </c>
+      <c r="H94" s="11" t="n">
+        <v>873.46</v>
+      </c>
+      <c r="I94" s="11" t="n">
+        <v>1215.95</v>
+      </c>
+      <c r="J94" s="11" t="n">
+        <v>991.66</v>
+      </c>
+      <c r="K94" s="23" t="n">
+        <v>143656</v>
+      </c>
+      <c r="L94" s="23" t="n">
+        <v>95393</v>
+      </c>
+    </row>
+    <row r="95" ht="20" customHeight="1">
+      <c r="A95" s="14" t="inlineStr">
+        <is>
+          <t>Stress</t>
+        </is>
+      </c>
+      <c r="B95" s="14" t="inlineStr">
+        <is>
+          <t>10,000 conn (16 threads)</t>
+        </is>
+      </c>
+      <c r="C95" s="20" t="inlineStr">
+        <is>
+          <t>2table</t>
+        </is>
+      </c>
+      <c r="D95" s="16" t="n">
+        <v>4783.26</v>
+      </c>
+      <c r="E95" s="16" t="n">
+        <v>5452.18</v>
+      </c>
+      <c r="F95" s="17">
+        <f>IF(D95&gt;0, (E95-D95)/D95, 0)</f>
+        <v/>
+      </c>
+      <c r="G95" s="16" t="n">
+        <v>1687.36</v>
+      </c>
+      <c r="H95" s="16" t="n">
+        <v>1493.61</v>
+      </c>
+      <c r="I95" s="16" t="n">
+        <v>1899.44</v>
+      </c>
+      <c r="J95" s="16" t="n">
+        <v>1648.81</v>
+      </c>
+      <c r="K95" s="23" t="n">
+        <v>1130283</v>
+      </c>
+      <c r="L95" s="23" t="n">
+        <v>131657</v>
+      </c>
+    </row>
+    <row r="96" ht="20" customHeight="1">
+      <c r="A96" s="9" t="inlineStr">
+        <is>
+          <t>Stress</t>
+        </is>
+      </c>
+      <c r="B96" s="9" t="inlineStr">
+        <is>
+          <t>10,000 conn (16 threads)</t>
+        </is>
+      </c>
+      <c r="C96" s="19" t="inlineStr">
+        <is>
+          <t>3table</t>
+        </is>
+      </c>
+      <c r="D96" s="11" t="n">
+        <v>4242.16</v>
+      </c>
+      <c r="E96" s="11" t="n">
+        <v>4792.04</v>
+      </c>
+      <c r="F96" s="17">
+        <f>IF(D96&gt;0, (E96-D96)/D96, 0)</f>
+        <v/>
+      </c>
+      <c r="G96" s="11" t="n">
+        <v>1475.37</v>
+      </c>
+      <c r="H96" s="11" t="n">
+        <v>1697.12</v>
+      </c>
+      <c r="I96" s="11" t="n">
+        <v>1997.85</v>
+      </c>
+      <c r="J96" s="11" t="n">
+        <v>1860.58</v>
+      </c>
+      <c r="K96" s="23" t="n">
+        <v>18450129</v>
+      </c>
+      <c r="L96" s="23" t="n">
+        <v>216273</v>
+      </c>
+    </row>
+    <row r="97" ht="20" customHeight="1">
+      <c r="A97" s="14" t="inlineStr">
+        <is>
+          <t>Stress</t>
+        </is>
+      </c>
+      <c r="B97" s="14" t="inlineStr">
+        <is>
+          <t>10,000 conn (16 threads)</t>
+        </is>
+      </c>
+      <c r="C97" s="20" t="inlineStr">
+        <is>
+          <t>4table</t>
+        </is>
+      </c>
+      <c r="D97" s="16" t="n">
+        <v>3129.07</v>
+      </c>
+      <c r="E97" s="16" t="n">
+        <v>3413.24</v>
+      </c>
+      <c r="F97" s="17">
+        <f>IF(D97&gt;0, (E97-D97)/D97, 0)</f>
+        <v/>
+      </c>
+      <c r="G97" s="16" t="n">
+        <v>72.65000000000001</v>
+      </c>
+      <c r="H97" s="16" t="n">
+        <v>333.99</v>
+      </c>
+      <c r="I97" s="16" t="n">
+        <v>190.23</v>
+      </c>
+      <c r="J97" s="16" t="n">
+        <v>1704.7</v>
+      </c>
+      <c r="K97" s="23" t="n">
+        <v>17612418</v>
+      </c>
+      <c r="L97" s="23" t="n">
+        <v>19690183</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
benchmarks: add Python (opt.) sheet to Excel, preserve baseline language sheets, and sync reports
</commit_message>
<xml_diff>
--- a/Programming_Benchmark_Report.xlsx
+++ b/Programming_Benchmark_Report.xlsx
@@ -13,6 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PHP" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Go" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Java" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Python (opt.)" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -4053,6 +4054,864 @@
 </chartSpace>
 </file>
 
+<file path=xl/charts/chart33.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="10"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Get No Index: Throughput (Req/sec)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Python (opt.)'!D5</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:srgbClr val="0284C7"/>
+            </a:solidFill>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Python (opt.)'!$C$6:$C$13</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Python (opt.)'!$D$6:$D$13</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'Python (opt.)'!E5</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:srgbClr val="10B981"/>
+            </a:solidFill>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Python (opt.)'!$C$6:$C$13</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Python (opt.)'!$E$6:$E$13</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Endpoint</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Req / Sec</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart34.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="10"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Get No Index: Tail Latency P95 (ms)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Python (opt.)'!I5</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:srgbClr val="0284C7"/>
+            </a:solidFill>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Python (opt.)'!$C$6:$C$13</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Python (opt.)'!$I$6:$I$13</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'Python (opt.)'!J5</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:srgbClr val="10B981"/>
+            </a:solidFill>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Python (opt.)'!$C$6:$C$13</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Python (opt.)'!$J$6:$J$13</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Endpoint</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>P95 (ms)</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart35.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="10"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Get With Index: Throughput (Req/sec)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Python (opt.)'!D41</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:srgbClr val="0284C7"/>
+            </a:solidFill>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Python (opt.)'!$C$42:$C$49</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Python (opt.)'!$D$42:$D$49</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'Python (opt.)'!E41</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:srgbClr val="10B981"/>
+            </a:solidFill>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Python (opt.)'!$C$42:$C$49</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Python (opt.)'!$E$42:$E$49</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Endpoint</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Req / Sec</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart36.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="10"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Get With Index: Tail Latency P95 (ms)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Python (opt.)'!I41</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:srgbClr val="0284C7"/>
+            </a:solidFill>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Python (opt.)'!$C$42:$C$49</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Python (opt.)'!$I$42:$I$49</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'Python (opt.)'!J41</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:srgbClr val="10B981"/>
+            </a:solidFill>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Python (opt.)'!$C$42:$C$49</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Python (opt.)'!$J$42:$J$49</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Endpoint</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>P95 (ms)</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart37.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="10"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Post: Throughput (Req/sec)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Python (opt.)'!D77</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:srgbClr val="0284C7"/>
+            </a:solidFill>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Python (opt.)'!$C$78:$C$85</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Python (opt.)'!$D$78:$D$85</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'Python (opt.)'!E77</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:srgbClr val="10B981"/>
+            </a:solidFill>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Python (opt.)'!$C$78:$C$85</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Python (opt.)'!$E$78:$E$85</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Endpoint</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Req / Sec</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart38.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="10"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Post: Tail Latency P95 (ms)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Python (opt.)'!I77</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:srgbClr val="0284C7"/>
+            </a:solidFill>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Python (opt.)'!$C$78:$C$85</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Python (opt.)'!$I$78:$I$85</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'Python (opt.)'!J77</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:srgbClr val="10B981"/>
+            </a:solidFill>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Python (opt.)'!$C$78:$C$85</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Python (opt.)'!$J$78:$J$85</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Endpoint</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>P95 (ms)</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
 <file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="10"/>
@@ -5645,6 +6504,143 @@
 </wsDr>
 </file>
 
+<file path=xl/drawings/drawing7.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>13</col>
+      <colOff>0</colOff>
+      <row>4</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5760000" cy="3600000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>13</col>
+      <colOff>0</colOff>
+      <row>21</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5760000" cy="3600000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="2" name="Chart 2"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>13</col>
+      <colOff>0</colOff>
+      <row>40</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5760000" cy="3600000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="3" name="Chart 3"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>13</col>
+      <colOff>0</colOff>
+      <row>57</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5760000" cy="3600000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="4" name="Chart 4"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>13</col>
+      <colOff>0</colOff>
+      <row>76</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5760000" cy="3600000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="5" name="Chart 5"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId5"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>13</col>
+      <colOff>0</colOff>
+      <row>93</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5760000" cy="3600000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="6" name="Chart 6"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId6"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -21821,4 +22817,2990 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L97"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="136" customWidth="1" min="1" max="1"/>
+    <col width="27" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="31" customWidth="1" min="6" max="6"/>
+    <col width="19" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="13" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>PYTHON (OPT.) (FASTAPI (OPT)) - DETAILED BENCHMARK SPECIFICATION</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="18" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Runtime: Python 3.12 (CustomORJSONResponse / uvloop / 16 workers) | Full Factorial Matrix: Docker Container (Dkr) vs Bare Metal (BME)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
+    <row r="4" ht="24" customHeight="1">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>1. GET (NO-INDEX) SUITE - FULL TABLE SCANS</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="22" customHeight="1">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>Tier</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>Concurrency</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="inlineStr">
+        <is>
+          <t>Endpoint</t>
+        </is>
+      </c>
+      <c r="D5" s="8" t="inlineStr">
+        <is>
+          <t>Docker Req/s</t>
+        </is>
+      </c>
+      <c r="E5" s="8" t="inlineStr">
+        <is>
+          <t>BME Req/s</t>
+        </is>
+      </c>
+      <c r="F5" s="8" t="inlineStr">
+        <is>
+          <t>BME Gain (%)</t>
+        </is>
+      </c>
+      <c r="G5" s="8" t="inlineStr">
+        <is>
+          <t>Docker Mean (ms)</t>
+        </is>
+      </c>
+      <c r="H5" s="8" t="inlineStr">
+        <is>
+          <t>BME Mean (ms)</t>
+        </is>
+      </c>
+      <c r="I5" s="8" t="inlineStr">
+        <is>
+          <t>Docker P95 (ms)</t>
+        </is>
+      </c>
+      <c r="J5" s="8" t="inlineStr">
+        <is>
+          <t>BME P95 (ms)</t>
+        </is>
+      </c>
+      <c r="K5" s="8" t="inlineStr">
+        <is>
+          <t>Docker Errors</t>
+        </is>
+      </c>
+      <c r="L5" s="8" t="inlineStr">
+        <is>
+          <t>BME Errors</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="20" customHeight="1">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>POC</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>20 conn (2 threads)</t>
+        </is>
+      </c>
+      <c r="C6" s="19" t="inlineStr">
+        <is>
+          <t>1table</t>
+        </is>
+      </c>
+      <c r="D6" s="11" t="n">
+        <v>2288.6</v>
+      </c>
+      <c r="E6" s="11" t="n">
+        <v>1384.43</v>
+      </c>
+      <c r="F6" s="12">
+        <f>IF(D6&gt;0, (E6-D6)/D6, 0)</f>
+        <v/>
+      </c>
+      <c r="G6" s="11" t="n">
+        <v>8.92</v>
+      </c>
+      <c r="H6" s="11" t="n">
+        <v>24.98</v>
+      </c>
+      <c r="I6" s="11" t="n">
+        <v>16.19</v>
+      </c>
+      <c r="J6" s="11" t="n">
+        <v>87.81999999999999</v>
+      </c>
+      <c r="K6" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" s="13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" ht="20" customHeight="1">
+      <c r="A7" s="14" t="inlineStr">
+        <is>
+          <t>POC</t>
+        </is>
+      </c>
+      <c r="B7" s="14" t="inlineStr">
+        <is>
+          <t>20 conn (2 threads)</t>
+        </is>
+      </c>
+      <c r="C7" s="20" t="inlineStr">
+        <is>
+          <t>2join</t>
+        </is>
+      </c>
+      <c r="D7" s="16" t="n">
+        <v>2583.93</v>
+      </c>
+      <c r="E7" s="16" t="n">
+        <v>2423.24</v>
+      </c>
+      <c r="F7" s="12">
+        <f>IF(D7&gt;0, (E7-D7)/D7, 0)</f>
+        <v/>
+      </c>
+      <c r="G7" s="16" t="n">
+        <v>7.78</v>
+      </c>
+      <c r="H7" s="16" t="n">
+        <v>8.32</v>
+      </c>
+      <c r="I7" s="16" t="n">
+        <v>12.31</v>
+      </c>
+      <c r="J7" s="16" t="n">
+        <v>14.55</v>
+      </c>
+      <c r="K7" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" s="18" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" ht="20" customHeight="1">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>POC</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>20 conn (2 threads)</t>
+        </is>
+      </c>
+      <c r="C8" s="19" t="inlineStr">
+        <is>
+          <t>3join</t>
+        </is>
+      </c>
+      <c r="D8" s="11" t="n">
+        <v>308.21</v>
+      </c>
+      <c r="E8" s="11" t="n">
+        <v>317.22</v>
+      </c>
+      <c r="F8" s="17">
+        <f>IF(D8&gt;0, (E8-D8)/D8, 0)</f>
+        <v/>
+      </c>
+      <c r="G8" s="11" t="n">
+        <v>64.81</v>
+      </c>
+      <c r="H8" s="11" t="n">
+        <v>62.55</v>
+      </c>
+      <c r="I8" s="11" t="n">
+        <v>92.84</v>
+      </c>
+      <c r="J8" s="11" t="n">
+        <v>89.88</v>
+      </c>
+      <c r="K8" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" s="13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" ht="20" customHeight="1">
+      <c r="A9" s="14" t="inlineStr">
+        <is>
+          <t>POC</t>
+        </is>
+      </c>
+      <c r="B9" s="14" t="inlineStr">
+        <is>
+          <t>20 conn (2 threads)</t>
+        </is>
+      </c>
+      <c r="C9" s="20" t="inlineStr">
+        <is>
+          <t>4join</t>
+        </is>
+      </c>
+      <c r="D9" s="16" t="n">
+        <v>71.84999999999999</v>
+      </c>
+      <c r="E9" s="16" t="n">
+        <v>722.62</v>
+      </c>
+      <c r="F9" s="17">
+        <f>IF(D9&gt;0, (E9-D9)/D9, 0)</f>
+        <v/>
+      </c>
+      <c r="G9" s="16" t="n">
+        <v>276.98</v>
+      </c>
+      <c r="H9" s="16" t="n">
+        <v>27.6</v>
+      </c>
+      <c r="I9" s="16" t="n">
+        <v>394.91</v>
+      </c>
+      <c r="J9" s="16" t="n">
+        <v>41.13</v>
+      </c>
+      <c r="K9" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="L9" s="18" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" ht="20" customHeight="1">
+      <c r="A10" s="9" t="inlineStr">
+        <is>
+          <t>Small</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>100 conn (4 threads)</t>
+        </is>
+      </c>
+      <c r="C10" s="19" t="inlineStr">
+        <is>
+          <t>1table</t>
+        </is>
+      </c>
+      <c r="D10" s="11" t="n">
+        <v>2442.05</v>
+      </c>
+      <c r="E10" s="11" t="n">
+        <v>4651.84</v>
+      </c>
+      <c r="F10" s="17">
+        <f>IF(D10&gt;0, (E10-D10)/D10, 0)</f>
+        <v/>
+      </c>
+      <c r="G10" s="11" t="n">
+        <v>41.1</v>
+      </c>
+      <c r="H10" s="11" t="n">
+        <v>23.18</v>
+      </c>
+      <c r="I10" s="11" t="n">
+        <v>64.19</v>
+      </c>
+      <c r="J10" s="11" t="n">
+        <v>59.82</v>
+      </c>
+      <c r="K10" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="L10" s="13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" ht="20" customHeight="1">
+      <c r="A11" s="14" t="inlineStr">
+        <is>
+          <t>Small</t>
+        </is>
+      </c>
+      <c r="B11" s="14" t="inlineStr">
+        <is>
+          <t>100 conn (4 threads)</t>
+        </is>
+      </c>
+      <c r="C11" s="20" t="inlineStr">
+        <is>
+          <t>2join</t>
+        </is>
+      </c>
+      <c r="D11" s="16" t="n">
+        <v>2845.01</v>
+      </c>
+      <c r="E11" s="16" t="n">
+        <v>4316.34</v>
+      </c>
+      <c r="F11" s="17">
+        <f>IF(D11&gt;0, (E11-D11)/D11, 0)</f>
+        <v/>
+      </c>
+      <c r="G11" s="16" t="n">
+        <v>35.14</v>
+      </c>
+      <c r="H11" s="16" t="n">
+        <v>23.54</v>
+      </c>
+      <c r="I11" s="16" t="n">
+        <v>53.02</v>
+      </c>
+      <c r="J11" s="16" t="n">
+        <v>49.84</v>
+      </c>
+      <c r="K11" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="L11" s="18" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" ht="20" customHeight="1">
+      <c r="A12" s="9" t="inlineStr">
+        <is>
+          <t>Small</t>
+        </is>
+      </c>
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>100 conn (4 threads)</t>
+        </is>
+      </c>
+      <c r="C12" s="19" t="inlineStr">
+        <is>
+          <t>3join</t>
+        </is>
+      </c>
+      <c r="D12" s="11" t="n">
+        <v>315.72</v>
+      </c>
+      <c r="E12" s="11" t="n">
+        <v>300.56</v>
+      </c>
+      <c r="F12" s="12">
+        <f>IF(D12&gt;0, (E12-D12)/D12, 0)</f>
+        <v/>
+      </c>
+      <c r="G12" s="11" t="n">
+        <v>315.65</v>
+      </c>
+      <c r="H12" s="11" t="n">
+        <v>319.87</v>
+      </c>
+      <c r="I12" s="11" t="n">
+        <v>498.56</v>
+      </c>
+      <c r="J12" s="11" t="n">
+        <v>481.04</v>
+      </c>
+      <c r="K12" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="L12" s="13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" ht="20" customHeight="1">
+      <c r="A13" s="14" t="inlineStr">
+        <is>
+          <t>Small</t>
+        </is>
+      </c>
+      <c r="B13" s="14" t="inlineStr">
+        <is>
+          <t>100 conn (4 threads)</t>
+        </is>
+      </c>
+      <c r="C13" s="20" t="inlineStr">
+        <is>
+          <t>4join</t>
+        </is>
+      </c>
+      <c r="D13" s="16" t="n">
+        <v>72.88</v>
+      </c>
+      <c r="E13" s="16" t="n">
+        <v>678.83</v>
+      </c>
+      <c r="F13" s="17">
+        <f>IF(D13&gt;0, (E13-D13)/D13, 0)</f>
+        <v/>
+      </c>
+      <c r="G13" s="16" t="n">
+        <v>1350.84</v>
+      </c>
+      <c r="H13" s="16" t="n">
+        <v>144.45</v>
+      </c>
+      <c r="I13" s="16" t="n">
+        <v>1773.07</v>
+      </c>
+      <c r="J13" s="16" t="n">
+        <v>241.39</v>
+      </c>
+      <c r="K13" s="23" t="n">
+        <v>515</v>
+      </c>
+      <c r="L13" s="18" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" ht="20" customHeight="1">
+      <c r="A14" s="9" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>500 conn (8 threads)</t>
+        </is>
+      </c>
+      <c r="C14" s="19" t="inlineStr">
+        <is>
+          <t>1table</t>
+        </is>
+      </c>
+      <c r="D14" s="11" t="n">
+        <v>2263.24</v>
+      </c>
+      <c r="E14" s="11" t="n">
+        <v>4598.21</v>
+      </c>
+      <c r="F14" s="17">
+        <f>IF(D14&gt;0, (E14-D14)/D14, 0)</f>
+        <v/>
+      </c>
+      <c r="G14" s="11" t="n">
+        <v>223.68</v>
+      </c>
+      <c r="H14" s="11" t="n">
+        <v>119.96</v>
+      </c>
+      <c r="I14" s="11" t="n">
+        <v>427.8</v>
+      </c>
+      <c r="J14" s="11" t="n">
+        <v>276.55</v>
+      </c>
+      <c r="K14" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="L14" s="23" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="15" ht="20" customHeight="1">
+      <c r="A15" s="14" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="B15" s="14" t="inlineStr">
+        <is>
+          <t>500 conn (8 threads)</t>
+        </is>
+      </c>
+      <c r="C15" s="20" t="inlineStr">
+        <is>
+          <t>2join</t>
+        </is>
+      </c>
+      <c r="D15" s="16" t="n">
+        <v>2536.46</v>
+      </c>
+      <c r="E15" s="16" t="n">
+        <v>4290.31</v>
+      </c>
+      <c r="F15" s="17">
+        <f>IF(D15&gt;0, (E15-D15)/D15, 0)</f>
+        <v/>
+      </c>
+      <c r="G15" s="16" t="n">
+        <v>203.19</v>
+      </c>
+      <c r="H15" s="16" t="n">
+        <v>140.01</v>
+      </c>
+      <c r="I15" s="16" t="n">
+        <v>413.12</v>
+      </c>
+      <c r="J15" s="16" t="n">
+        <v>420.98</v>
+      </c>
+      <c r="K15" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="L15" s="23" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="16" ht="20" customHeight="1">
+      <c r="A16" s="9" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>500 conn (8 threads)</t>
+        </is>
+      </c>
+      <c r="C16" s="19" t="inlineStr">
+        <is>
+          <t>3join</t>
+        </is>
+      </c>
+      <c r="D16" s="11" t="n">
+        <v>312.48</v>
+      </c>
+      <c r="E16" s="11" t="n">
+        <v>268.06</v>
+      </c>
+      <c r="F16" s="12">
+        <f>IF(D16&gt;0, (E16-D16)/D16, 0)</f>
+        <v/>
+      </c>
+      <c r="G16" s="11" t="n">
+        <v>1318.84</v>
+      </c>
+      <c r="H16" s="11" t="n">
+        <v>1122.48</v>
+      </c>
+      <c r="I16" s="11" t="n">
+        <v>1915.67</v>
+      </c>
+      <c r="J16" s="11" t="n">
+        <v>1877.45</v>
+      </c>
+      <c r="K16" s="23" t="n">
+        <v>81206</v>
+      </c>
+      <c r="L16" s="23" t="n">
+        <v>1001</v>
+      </c>
+    </row>
+    <row r="17" ht="20" customHeight="1">
+      <c r="A17" s="14" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="B17" s="14" t="inlineStr">
+        <is>
+          <t>500 conn (8 threads)</t>
+        </is>
+      </c>
+      <c r="C17" s="20" t="inlineStr">
+        <is>
+          <t>4join</t>
+        </is>
+      </c>
+      <c r="D17" s="16" t="n">
+        <v>66.38</v>
+      </c>
+      <c r="E17" s="16" t="n">
+        <v>646.46</v>
+      </c>
+      <c r="F17" s="17">
+        <f>IF(D17&gt;0, (E17-D17)/D17, 0)</f>
+        <v/>
+      </c>
+      <c r="G17" s="16" t="n">
+        <v>1208.08</v>
+      </c>
+      <c r="H17" s="16" t="n">
+        <v>667.42</v>
+      </c>
+      <c r="I17" s="16" t="n">
+        <v>1922.29</v>
+      </c>
+      <c r="J17" s="16" t="n">
+        <v>1381.23</v>
+      </c>
+      <c r="K17" s="23" t="n">
+        <v>78894</v>
+      </c>
+      <c r="L17" s="23" t="n">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="18" ht="20" customHeight="1">
+      <c r="A18" s="9" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="B18" s="9" t="inlineStr">
+        <is>
+          <t>2,000 conn (8 threads)</t>
+        </is>
+      </c>
+      <c r="C18" s="19" t="inlineStr">
+        <is>
+          <t>1table</t>
+        </is>
+      </c>
+      <c r="D18" s="11" t="n">
+        <v>2238.59</v>
+      </c>
+      <c r="E18" s="11" t="n">
+        <v>4357.49</v>
+      </c>
+      <c r="F18" s="17">
+        <f>IF(D18&gt;0, (E18-D18)/D18, 0)</f>
+        <v/>
+      </c>
+      <c r="G18" s="11" t="n">
+        <v>666.52</v>
+      </c>
+      <c r="H18" s="11" t="n">
+        <v>308.12</v>
+      </c>
+      <c r="I18" s="11" t="n">
+        <v>826.66</v>
+      </c>
+      <c r="J18" s="11" t="n">
+        <v>1235.2</v>
+      </c>
+      <c r="K18" s="23" t="n">
+        <v>180809</v>
+      </c>
+      <c r="L18" s="23" t="n">
+        <v>2341</v>
+      </c>
+    </row>
+    <row r="19" ht="20" customHeight="1">
+      <c r="A19" s="14" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="B19" s="14" t="inlineStr">
+        <is>
+          <t>2,000 conn (8 threads)</t>
+        </is>
+      </c>
+      <c r="C19" s="20" t="inlineStr">
+        <is>
+          <t>2join</t>
+        </is>
+      </c>
+      <c r="D19" s="16" t="n">
+        <v>2556.75</v>
+      </c>
+      <c r="E19" s="16" t="n">
+        <v>4047.56</v>
+      </c>
+      <c r="F19" s="17">
+        <f>IF(D19&gt;0, (E19-D19)/D19, 0)</f>
+        <v/>
+      </c>
+      <c r="G19" s="16" t="n">
+        <v>536.61</v>
+      </c>
+      <c r="H19" s="16" t="n">
+        <v>336.12</v>
+      </c>
+      <c r="I19" s="16" t="n">
+        <v>932.01</v>
+      </c>
+      <c r="J19" s="16" t="n">
+        <v>1289.28</v>
+      </c>
+      <c r="K19" s="23" t="n">
+        <v>372570</v>
+      </c>
+      <c r="L19" s="23" t="n">
+        <v>2191</v>
+      </c>
+    </row>
+    <row r="20" ht="20" customHeight="1">
+      <c r="A20" s="9" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="B20" s="9" t="inlineStr">
+        <is>
+          <t>2,000 conn (8 threads)</t>
+        </is>
+      </c>
+      <c r="C20" s="19" t="inlineStr">
+        <is>
+          <t>3join</t>
+        </is>
+      </c>
+      <c r="D20" s="11" t="n">
+        <v>301.12</v>
+      </c>
+      <c r="E20" s="11" t="n">
+        <v>108.65</v>
+      </c>
+      <c r="F20" s="12">
+        <f>IF(D20&gt;0, (E20-D20)/D20, 0)</f>
+        <v/>
+      </c>
+      <c r="G20" s="11" t="n">
+        <v>1239.21</v>
+      </c>
+      <c r="H20" s="11" t="n">
+        <v>865.89</v>
+      </c>
+      <c r="I20" s="11" t="n">
+        <v>1874.89</v>
+      </c>
+      <c r="J20" s="11" t="n">
+        <v>1317.67</v>
+      </c>
+      <c r="K20" s="23" t="n">
+        <v>619774</v>
+      </c>
+      <c r="L20" s="23" t="n">
+        <v>1026</v>
+      </c>
+    </row>
+    <row r="21" ht="20" customHeight="1">
+      <c r="A21" s="14" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="B21" s="14" t="inlineStr">
+        <is>
+          <t>2,000 conn (8 threads)</t>
+        </is>
+      </c>
+      <c r="C21" s="20" t="inlineStr">
+        <is>
+          <t>4join</t>
+        </is>
+      </c>
+      <c r="D21" s="16" t="n">
+        <v>57.79</v>
+      </c>
+      <c r="E21" s="16" t="n">
+        <v>254.33</v>
+      </c>
+      <c r="F21" s="17">
+        <f>IF(D21&gt;0, (E21-D21)/D21, 0)</f>
+        <v/>
+      </c>
+      <c r="G21" s="16" t="n">
+        <v>944.62</v>
+      </c>
+      <c r="H21" s="16" t="n">
+        <v>911.3</v>
+      </c>
+      <c r="I21" s="16" t="n">
+        <v>1657.53</v>
+      </c>
+      <c r="J21" s="16" t="n">
+        <v>1860.75</v>
+      </c>
+      <c r="K21" s="23" t="n">
+        <v>138661</v>
+      </c>
+      <c r="L21" s="23" t="n">
+        <v>2451</v>
+      </c>
+    </row>
+    <row r="22" ht="20" customHeight="1">
+      <c r="A22" s="9" t="inlineStr">
+        <is>
+          <t>Stress</t>
+        </is>
+      </c>
+      <c r="B22" s="9" t="inlineStr">
+        <is>
+          <t>10,000 conn (16 threads)</t>
+        </is>
+      </c>
+      <c r="C22" s="19" t="inlineStr">
+        <is>
+          <t>1table</t>
+        </is>
+      </c>
+      <c r="D22" s="11" t="n">
+        <v>2043.66</v>
+      </c>
+      <c r="E22" s="11" t="n">
+        <v>3837.87</v>
+      </c>
+      <c r="F22" s="17">
+        <f>IF(D22&gt;0, (E22-D22)/D22, 0)</f>
+        <v/>
+      </c>
+      <c r="G22" s="11" t="n">
+        <v>697.37</v>
+      </c>
+      <c r="H22" s="11" t="n">
+        <v>219.26</v>
+      </c>
+      <c r="I22" s="11" t="n">
+        <v>877.52</v>
+      </c>
+      <c r="J22" s="11" t="n">
+        <v>984.24</v>
+      </c>
+      <c r="K22" s="23" t="n">
+        <v>871432</v>
+      </c>
+      <c r="L22" s="23" t="n">
+        <v>5336</v>
+      </c>
+    </row>
+    <row r="23" ht="20" customHeight="1">
+      <c r="A23" s="14" t="inlineStr">
+        <is>
+          <t>Stress</t>
+        </is>
+      </c>
+      <c r="B23" s="14" t="inlineStr">
+        <is>
+          <t>10,000 conn (16 threads)</t>
+        </is>
+      </c>
+      <c r="C23" s="20" t="inlineStr">
+        <is>
+          <t>2join</t>
+        </is>
+      </c>
+      <c r="D23" s="16" t="n">
+        <v>2273.36</v>
+      </c>
+      <c r="E23" s="16" t="n">
+        <v>3560.28</v>
+      </c>
+      <c r="F23" s="17">
+        <f>IF(D23&gt;0, (E23-D23)/D23, 0)</f>
+        <v/>
+      </c>
+      <c r="G23" s="16" t="n">
+        <v>539.49</v>
+      </c>
+      <c r="H23" s="16" t="n">
+        <v>259.31</v>
+      </c>
+      <c r="I23" s="16" t="n">
+        <v>735.16</v>
+      </c>
+      <c r="J23" s="16" t="n">
+        <v>1332.79</v>
+      </c>
+      <c r="K23" s="23" t="n">
+        <v>1611777</v>
+      </c>
+      <c r="L23" s="23" t="n">
+        <v>5846</v>
+      </c>
+    </row>
+    <row r="24" ht="20" customHeight="1">
+      <c r="A24" s="9" t="inlineStr">
+        <is>
+          <t>Stress</t>
+        </is>
+      </c>
+      <c r="B24" s="9" t="inlineStr">
+        <is>
+          <t>10,000 conn (16 threads)</t>
+        </is>
+      </c>
+      <c r="C24" s="19" t="inlineStr">
+        <is>
+          <t>3join</t>
+        </is>
+      </c>
+      <c r="D24" s="11" t="n">
+        <v>275.29</v>
+      </c>
+      <c r="E24" s="11" t="n">
+        <v>117.14</v>
+      </c>
+      <c r="F24" s="12">
+        <f>IF(D24&gt;0, (E24-D24)/D24, 0)</f>
+        <v/>
+      </c>
+      <c r="G24" s="11" t="n">
+        <v>1247.32</v>
+      </c>
+      <c r="H24" s="11" t="n">
+        <v>968.28</v>
+      </c>
+      <c r="I24" s="11" t="n">
+        <v>1880.77</v>
+      </c>
+      <c r="J24" s="11" t="n">
+        <v>1607.21</v>
+      </c>
+      <c r="K24" s="23" t="n">
+        <v>1430364</v>
+      </c>
+      <c r="L24" s="23" t="n">
+        <v>842</v>
+      </c>
+    </row>
+    <row r="25" ht="20" customHeight="1">
+      <c r="A25" s="14" t="inlineStr">
+        <is>
+          <t>Stress</t>
+        </is>
+      </c>
+      <c r="B25" s="14" t="inlineStr">
+        <is>
+          <t>10,000 conn (16 threads)</t>
+        </is>
+      </c>
+      <c r="C25" s="20" t="inlineStr">
+        <is>
+          <t>4join</t>
+        </is>
+      </c>
+      <c r="D25" s="16" t="n">
+        <v>40.45</v>
+      </c>
+      <c r="E25" s="16" t="n">
+        <v>61.09</v>
+      </c>
+      <c r="F25" s="17">
+        <f>IF(D25&gt;0, (E25-D25)/D25, 0)</f>
+        <v/>
+      </c>
+      <c r="G25" s="16" t="n">
+        <v>744.15</v>
+      </c>
+      <c r="H25" s="16" t="n">
+        <v>634.0700000000001</v>
+      </c>
+      <c r="I25" s="16" t="n">
+        <v>1701.78</v>
+      </c>
+      <c r="J25" s="16" t="n">
+        <v>1201.3</v>
+      </c>
+      <c r="K25" s="23" t="n">
+        <v>243356</v>
+      </c>
+      <c r="L25" s="18" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26"/>
+    <row r="27"/>
+    <row r="28"/>
+    <row r="29"/>
+    <row r="30"/>
+    <row r="31"/>
+    <row r="32"/>
+    <row r="33"/>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
+    <row r="40" ht="24" customHeight="1">
+      <c r="A40" s="7" t="inlineStr">
+        <is>
+          <t>2. GET (WITH-INDEX) SUITE - INDEXED B-TREE POINT LOOKUPS</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="22" customHeight="1">
+      <c r="A41" s="8" t="inlineStr">
+        <is>
+          <t>Tier</t>
+        </is>
+      </c>
+      <c r="B41" s="8" t="inlineStr">
+        <is>
+          <t>Concurrency</t>
+        </is>
+      </c>
+      <c r="C41" s="8" t="inlineStr">
+        <is>
+          <t>Endpoint</t>
+        </is>
+      </c>
+      <c r="D41" s="8" t="inlineStr">
+        <is>
+          <t>Docker Req/s</t>
+        </is>
+      </c>
+      <c r="E41" s="8" t="inlineStr">
+        <is>
+          <t>BME Req/s</t>
+        </is>
+      </c>
+      <c r="F41" s="8" t="inlineStr">
+        <is>
+          <t>BME Gain (%)</t>
+        </is>
+      </c>
+      <c r="G41" s="8" t="inlineStr">
+        <is>
+          <t>Docker Mean (ms)</t>
+        </is>
+      </c>
+      <c r="H41" s="8" t="inlineStr">
+        <is>
+          <t>BME Mean (ms)</t>
+        </is>
+      </c>
+      <c r="I41" s="8" t="inlineStr">
+        <is>
+          <t>Docker P95 (ms)</t>
+        </is>
+      </c>
+      <c r="J41" s="8" t="inlineStr">
+        <is>
+          <t>BME P95 (ms)</t>
+        </is>
+      </c>
+      <c r="K41" s="8" t="inlineStr">
+        <is>
+          <t>Docker Errors</t>
+        </is>
+      </c>
+      <c r="L41" s="8" t="inlineStr">
+        <is>
+          <t>BME Errors</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="20" customHeight="1">
+      <c r="A42" s="9" t="inlineStr">
+        <is>
+          <t>POC</t>
+        </is>
+      </c>
+      <c r="B42" s="9" t="inlineStr">
+        <is>
+          <t>20 conn (2 threads)</t>
+        </is>
+      </c>
+      <c r="C42" s="19" t="inlineStr">
+        <is>
+          <t>1table</t>
+        </is>
+      </c>
+      <c r="D42" s="11" t="n">
+        <v>2279.05</v>
+      </c>
+      <c r="E42" s="11" t="n">
+        <v>3023.71</v>
+      </c>
+      <c r="F42" s="17">
+        <f>IF(D42&gt;0, (E42-D42)/D42, 0)</f>
+        <v/>
+      </c>
+      <c r="G42" s="11" t="n">
+        <v>8.92</v>
+      </c>
+      <c r="H42" s="11" t="n">
+        <v>6.71</v>
+      </c>
+      <c r="I42" s="11" t="n">
+        <v>15.6</v>
+      </c>
+      <c r="J42" s="11" t="n">
+        <v>12.16</v>
+      </c>
+      <c r="K42" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="L42" s="13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43" ht="20" customHeight="1">
+      <c r="A43" s="14" t="inlineStr">
+        <is>
+          <t>POC</t>
+        </is>
+      </c>
+      <c r="B43" s="14" t="inlineStr">
+        <is>
+          <t>20 conn (2 threads)</t>
+        </is>
+      </c>
+      <c r="C43" s="20" t="inlineStr">
+        <is>
+          <t>2join</t>
+        </is>
+      </c>
+      <c r="D43" s="16" t="n">
+        <v>2575.84</v>
+      </c>
+      <c r="E43" s="16" t="n">
+        <v>2454.7</v>
+      </c>
+      <c r="F43" s="12">
+        <f>IF(D43&gt;0, (E43-D43)/D43, 0)</f>
+        <v/>
+      </c>
+      <c r="G43" s="16" t="n">
+        <v>7.82</v>
+      </c>
+      <c r="H43" s="16" t="n">
+        <v>8.460000000000001</v>
+      </c>
+      <c r="I43" s="16" t="n">
+        <v>12.15</v>
+      </c>
+      <c r="J43" s="16" t="n">
+        <v>17.33</v>
+      </c>
+      <c r="K43" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="L43" s="18" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44" ht="20" customHeight="1">
+      <c r="A44" s="9" t="inlineStr">
+        <is>
+          <t>POC</t>
+        </is>
+      </c>
+      <c r="B44" s="9" t="inlineStr">
+        <is>
+          <t>20 conn (2 threads)</t>
+        </is>
+      </c>
+      <c r="C44" s="19" t="inlineStr">
+        <is>
+          <t>3join</t>
+        </is>
+      </c>
+      <c r="D44" s="11" t="n">
+        <v>1723.85</v>
+      </c>
+      <c r="E44" s="11" t="n">
+        <v>1607.55</v>
+      </c>
+      <c r="F44" s="12">
+        <f>IF(D44&gt;0, (E44-D44)/D44, 0)</f>
+        <v/>
+      </c>
+      <c r="G44" s="11" t="n">
+        <v>11.63</v>
+      </c>
+      <c r="H44" s="11" t="n">
+        <v>12.63</v>
+      </c>
+      <c r="I44" s="11" t="n">
+        <v>18.04</v>
+      </c>
+      <c r="J44" s="11" t="n">
+        <v>24.07</v>
+      </c>
+      <c r="K44" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="L44" s="13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45" ht="20" customHeight="1">
+      <c r="A45" s="14" t="inlineStr">
+        <is>
+          <t>POC</t>
+        </is>
+      </c>
+      <c r="B45" s="14" t="inlineStr">
+        <is>
+          <t>20 conn (2 threads)</t>
+        </is>
+      </c>
+      <c r="C45" s="20" t="inlineStr">
+        <is>
+          <t>4join</t>
+        </is>
+      </c>
+      <c r="D45" s="16" t="n">
+        <v>1369.93</v>
+      </c>
+      <c r="E45" s="16" t="n">
+        <v>1540.36</v>
+      </c>
+      <c r="F45" s="17">
+        <f>IF(D45&gt;0, (E45-D45)/D45, 0)</f>
+        <v/>
+      </c>
+      <c r="G45" s="16" t="n">
+        <v>14.66</v>
+      </c>
+      <c r="H45" s="16" t="n">
+        <v>13.08</v>
+      </c>
+      <c r="I45" s="16" t="n">
+        <v>23.59</v>
+      </c>
+      <c r="J45" s="16" t="n">
+        <v>25.1</v>
+      </c>
+      <c r="K45" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="L45" s="18" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46" ht="20" customHeight="1">
+      <c r="A46" s="9" t="inlineStr">
+        <is>
+          <t>Small</t>
+        </is>
+      </c>
+      <c r="B46" s="9" t="inlineStr">
+        <is>
+          <t>100 conn (4 threads)</t>
+        </is>
+      </c>
+      <c r="C46" s="19" t="inlineStr">
+        <is>
+          <t>1table</t>
+        </is>
+      </c>
+      <c r="D46" s="11" t="n">
+        <v>2394.42</v>
+      </c>
+      <c r="E46" s="11" t="n">
+        <v>4660.62</v>
+      </c>
+      <c r="F46" s="17">
+        <f>IF(D46&gt;0, (E46-D46)/D46, 0)</f>
+        <v/>
+      </c>
+      <c r="G46" s="11" t="n">
+        <v>41.76</v>
+      </c>
+      <c r="H46" s="11" t="n">
+        <v>22.23</v>
+      </c>
+      <c r="I46" s="11" t="n">
+        <v>65.51000000000001</v>
+      </c>
+      <c r="J46" s="11" t="n">
+        <v>49.02</v>
+      </c>
+      <c r="K46" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="L46" s="13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47" ht="20" customHeight="1">
+      <c r="A47" s="14" t="inlineStr">
+        <is>
+          <t>Small</t>
+        </is>
+      </c>
+      <c r="B47" s="14" t="inlineStr">
+        <is>
+          <t>100 conn (4 threads)</t>
+        </is>
+      </c>
+      <c r="C47" s="20" t="inlineStr">
+        <is>
+          <t>2join</t>
+        </is>
+      </c>
+      <c r="D47" s="16" t="n">
+        <v>2770.45</v>
+      </c>
+      <c r="E47" s="16" t="n">
+        <v>4314.84</v>
+      </c>
+      <c r="F47" s="17">
+        <f>IF(D47&gt;0, (E47-D47)/D47, 0)</f>
+        <v/>
+      </c>
+      <c r="G47" s="16" t="n">
+        <v>36.09</v>
+      </c>
+      <c r="H47" s="16" t="n">
+        <v>23.95</v>
+      </c>
+      <c r="I47" s="16" t="n">
+        <v>55.82</v>
+      </c>
+      <c r="J47" s="16" t="n">
+        <v>51.83</v>
+      </c>
+      <c r="K47" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="L47" s="18" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48" ht="20" customHeight="1">
+      <c r="A48" s="9" t="inlineStr">
+        <is>
+          <t>Small</t>
+        </is>
+      </c>
+      <c r="B48" s="9" t="inlineStr">
+        <is>
+          <t>100 conn (4 threads)</t>
+        </is>
+      </c>
+      <c r="C48" s="19" t="inlineStr">
+        <is>
+          <t>3join</t>
+        </is>
+      </c>
+      <c r="D48" s="11" t="n">
+        <v>1978.06</v>
+      </c>
+      <c r="E48" s="11" t="n">
+        <v>1767.4</v>
+      </c>
+      <c r="F48" s="12">
+        <f>IF(D48&gt;0, (E48-D48)/D48, 0)</f>
+        <v/>
+      </c>
+      <c r="G48" s="11" t="n">
+        <v>51.18</v>
+      </c>
+      <c r="H48" s="11" t="n">
+        <v>58.41</v>
+      </c>
+      <c r="I48" s="11" t="n">
+        <v>94.48</v>
+      </c>
+      <c r="J48" s="11" t="n">
+        <v>130.52</v>
+      </c>
+      <c r="K48" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="L48" s="13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49" ht="20" customHeight="1">
+      <c r="A49" s="14" t="inlineStr">
+        <is>
+          <t>Small</t>
+        </is>
+      </c>
+      <c r="B49" s="14" t="inlineStr">
+        <is>
+          <t>100 conn (4 threads)</t>
+        </is>
+      </c>
+      <c r="C49" s="20" t="inlineStr">
+        <is>
+          <t>4join</t>
+        </is>
+      </c>
+      <c r="D49" s="16" t="n">
+        <v>1663.88</v>
+      </c>
+      <c r="E49" s="16" t="n">
+        <v>1759.4</v>
+      </c>
+      <c r="F49" s="17">
+        <f>IF(D49&gt;0, (E49-D49)/D49, 0)</f>
+        <v/>
+      </c>
+      <c r="G49" s="16" t="n">
+        <v>60.73</v>
+      </c>
+      <c r="H49" s="16" t="n">
+        <v>58.15</v>
+      </c>
+      <c r="I49" s="16" t="n">
+        <v>110.48</v>
+      </c>
+      <c r="J49" s="16" t="n">
+        <v>124.6</v>
+      </c>
+      <c r="K49" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="L49" s="18" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50" ht="20" customHeight="1">
+      <c r="A50" s="9" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="B50" s="9" t="inlineStr">
+        <is>
+          <t>500 conn (8 threads)</t>
+        </is>
+      </c>
+      <c r="C50" s="19" t="inlineStr">
+        <is>
+          <t>1table</t>
+        </is>
+      </c>
+      <c r="D50" s="11" t="n">
+        <v>2221.51</v>
+      </c>
+      <c r="E50" s="11" t="n">
+        <v>4496.02</v>
+      </c>
+      <c r="F50" s="17">
+        <f>IF(D50&gt;0, (E50-D50)/D50, 0)</f>
+        <v/>
+      </c>
+      <c r="G50" s="11" t="n">
+        <v>229.8</v>
+      </c>
+      <c r="H50" s="11" t="n">
+        <v>114.78</v>
+      </c>
+      <c r="I50" s="11" t="n">
+        <v>471.67</v>
+      </c>
+      <c r="J50" s="11" t="n">
+        <v>202.05</v>
+      </c>
+      <c r="K50" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="L50" s="23" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="51" ht="20" customHeight="1">
+      <c r="A51" s="14" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="B51" s="14" t="inlineStr">
+        <is>
+          <t>500 conn (8 threads)</t>
+        </is>
+      </c>
+      <c r="C51" s="20" t="inlineStr">
+        <is>
+          <t>2join</t>
+        </is>
+      </c>
+      <c r="D51" s="16" t="n">
+        <v>2494.54</v>
+      </c>
+      <c r="E51" s="16" t="n">
+        <v>4243.25</v>
+      </c>
+      <c r="F51" s="17">
+        <f>IF(D51&gt;0, (E51-D51)/D51, 0)</f>
+        <v/>
+      </c>
+      <c r="G51" s="16" t="n">
+        <v>209.93</v>
+      </c>
+      <c r="H51" s="16" t="n">
+        <v>132.43</v>
+      </c>
+      <c r="I51" s="16" t="n">
+        <v>435.76</v>
+      </c>
+      <c r="J51" s="16" t="n">
+        <v>355.11</v>
+      </c>
+      <c r="K51" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="L51" s="23" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="52" ht="20" customHeight="1">
+      <c r="A52" s="9" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="B52" s="9" t="inlineStr">
+        <is>
+          <t>500 conn (8 threads)</t>
+        </is>
+      </c>
+      <c r="C52" s="19" t="inlineStr">
+        <is>
+          <t>3join</t>
+        </is>
+      </c>
+      <c r="D52" s="11" t="n">
+        <v>1783.44</v>
+      </c>
+      <c r="E52" s="11" t="n">
+        <v>1679.34</v>
+      </c>
+      <c r="F52" s="12">
+        <f>IF(D52&gt;0, (E52-D52)/D52, 0)</f>
+        <v/>
+      </c>
+      <c r="G52" s="11" t="n">
+        <v>308.25</v>
+      </c>
+      <c r="H52" s="11" t="n">
+        <v>309.43</v>
+      </c>
+      <c r="I52" s="11" t="n">
+        <v>795.98</v>
+      </c>
+      <c r="J52" s="11" t="n">
+        <v>844.86</v>
+      </c>
+      <c r="K52" s="23" t="n">
+        <v>314</v>
+      </c>
+      <c r="L52" s="23" t="n">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="53" ht="20" customHeight="1">
+      <c r="A53" s="14" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="B53" s="14" t="inlineStr">
+        <is>
+          <t>500 conn (8 threads)</t>
+        </is>
+      </c>
+      <c r="C53" s="20" t="inlineStr">
+        <is>
+          <t>4join</t>
+        </is>
+      </c>
+      <c r="D53" s="16" t="n">
+        <v>1445.35</v>
+      </c>
+      <c r="E53" s="16" t="n">
+        <v>1665.81</v>
+      </c>
+      <c r="F53" s="17">
+        <f>IF(D53&gt;0, (E53-D53)/D53, 0)</f>
+        <v/>
+      </c>
+      <c r="G53" s="16" t="n">
+        <v>367.92</v>
+      </c>
+      <c r="H53" s="16" t="n">
+        <v>306.52</v>
+      </c>
+      <c r="I53" s="16" t="n">
+        <v>896.09</v>
+      </c>
+      <c r="J53" s="16" t="n">
+        <v>801.27</v>
+      </c>
+      <c r="K53" s="23" t="n">
+        <v>967</v>
+      </c>
+      <c r="L53" s="23" t="n">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="54" ht="20" customHeight="1">
+      <c r="A54" s="9" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="B54" s="9" t="inlineStr">
+        <is>
+          <t>2,000 conn (8 threads)</t>
+        </is>
+      </c>
+      <c r="C54" s="19" t="inlineStr">
+        <is>
+          <t>1table</t>
+        </is>
+      </c>
+      <c r="D54" s="11" t="n">
+        <v>2205.47</v>
+      </c>
+      <c r="E54" s="11" t="n">
+        <v>4407.93</v>
+      </c>
+      <c r="F54" s="17">
+        <f>IF(D54&gt;0, (E54-D54)/D54, 0)</f>
+        <v/>
+      </c>
+      <c r="G54" s="11" t="n">
+        <v>674.4400000000001</v>
+      </c>
+      <c r="H54" s="11" t="n">
+        <v>298.59</v>
+      </c>
+      <c r="I54" s="11" t="n">
+        <v>833.92</v>
+      </c>
+      <c r="J54" s="11" t="n">
+        <v>1201.26</v>
+      </c>
+      <c r="K54" s="23" t="n">
+        <v>180877</v>
+      </c>
+      <c r="L54" s="23" t="n">
+        <v>2381</v>
+      </c>
+    </row>
+    <row r="55" ht="20" customHeight="1">
+      <c r="A55" s="14" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="B55" s="14" t="inlineStr">
+        <is>
+          <t>2,000 conn (8 threads)</t>
+        </is>
+      </c>
+      <c r="C55" s="20" t="inlineStr">
+        <is>
+          <t>2join</t>
+        </is>
+      </c>
+      <c r="D55" s="16" t="n">
+        <v>2515.07</v>
+      </c>
+      <c r="E55" s="16" t="n">
+        <v>4075.42</v>
+      </c>
+      <c r="F55" s="17">
+        <f>IF(D55&gt;0, (E55-D55)/D55, 0)</f>
+        <v/>
+      </c>
+      <c r="G55" s="16" t="n">
+        <v>542.66</v>
+      </c>
+      <c r="H55" s="16" t="n">
+        <v>339.03</v>
+      </c>
+      <c r="I55" s="16" t="n">
+        <v>923.6900000000001</v>
+      </c>
+      <c r="J55" s="16" t="n">
+        <v>1301.62</v>
+      </c>
+      <c r="K55" s="23" t="n">
+        <v>372072</v>
+      </c>
+      <c r="L55" s="23" t="n">
+        <v>2293</v>
+      </c>
+    </row>
+    <row r="56" ht="20" customHeight="1">
+      <c r="A56" s="9" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="B56" s="9" t="inlineStr">
+        <is>
+          <t>2,000 conn (8 threads)</t>
+        </is>
+      </c>
+      <c r="C56" s="19" t="inlineStr">
+        <is>
+          <t>3join</t>
+        </is>
+      </c>
+      <c r="D56" s="11" t="n">
+        <v>1772.15</v>
+      </c>
+      <c r="E56" s="11" t="n">
+        <v>1588.2</v>
+      </c>
+      <c r="F56" s="12">
+        <f>IF(D56&gt;0, (E56-D56)/D56, 0)</f>
+        <v/>
+      </c>
+      <c r="G56" s="11" t="n">
+        <v>699.66</v>
+      </c>
+      <c r="H56" s="11" t="n">
+        <v>679.27</v>
+      </c>
+      <c r="I56" s="11" t="n">
+        <v>1745.81</v>
+      </c>
+      <c r="J56" s="11" t="n">
+        <v>1717.38</v>
+      </c>
+      <c r="K56" s="23" t="n">
+        <v>668997</v>
+      </c>
+      <c r="L56" s="23" t="n">
+        <v>2787</v>
+      </c>
+    </row>
+    <row r="57" ht="20" customHeight="1">
+      <c r="A57" s="14" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="B57" s="14" t="inlineStr">
+        <is>
+          <t>2,000 conn (8 threads)</t>
+        </is>
+      </c>
+      <c r="C57" s="20" t="inlineStr">
+        <is>
+          <t>4join</t>
+        </is>
+      </c>
+      <c r="D57" s="16" t="n">
+        <v>1427.28</v>
+      </c>
+      <c r="E57" s="16" t="n">
+        <v>1593.35</v>
+      </c>
+      <c r="F57" s="17">
+        <f>IF(D57&gt;0, (E57-D57)/D57, 0)</f>
+        <v/>
+      </c>
+      <c r="G57" s="16" t="n">
+        <v>748.92</v>
+      </c>
+      <c r="H57" s="16" t="n">
+        <v>637.35</v>
+      </c>
+      <c r="I57" s="16" t="n">
+        <v>1800.43</v>
+      </c>
+      <c r="J57" s="16" t="n">
+        <v>1742.55</v>
+      </c>
+      <c r="K57" s="23" t="n">
+        <v>788107</v>
+      </c>
+      <c r="L57" s="23" t="n">
+        <v>2843</v>
+      </c>
+    </row>
+    <row r="58" ht="20" customHeight="1">
+      <c r="A58" s="9" t="inlineStr">
+        <is>
+          <t>Stress</t>
+        </is>
+      </c>
+      <c r="B58" s="9" t="inlineStr">
+        <is>
+          <t>10,000 conn (16 threads)</t>
+        </is>
+      </c>
+      <c r="C58" s="19" t="inlineStr">
+        <is>
+          <t>1table</t>
+        </is>
+      </c>
+      <c r="D58" s="11" t="n">
+        <v>2029.15</v>
+      </c>
+      <c r="E58" s="11" t="n">
+        <v>3908.34</v>
+      </c>
+      <c r="F58" s="17">
+        <f>IF(D58&gt;0, (E58-D58)/D58, 0)</f>
+        <v/>
+      </c>
+      <c r="G58" s="11" t="n">
+        <v>704.3</v>
+      </c>
+      <c r="H58" s="11" t="n">
+        <v>233.79</v>
+      </c>
+      <c r="I58" s="11" t="n">
+        <v>884.4</v>
+      </c>
+      <c r="J58" s="11" t="n">
+        <v>1079.05</v>
+      </c>
+      <c r="K58" s="23" t="n">
+        <v>852420</v>
+      </c>
+      <c r="L58" s="23" t="n">
+        <v>5003</v>
+      </c>
+    </row>
+    <row r="59" ht="20" customHeight="1">
+      <c r="A59" s="14" t="inlineStr">
+        <is>
+          <t>Stress</t>
+        </is>
+      </c>
+      <c r="B59" s="14" t="inlineStr">
+        <is>
+          <t>10,000 conn (16 threads)</t>
+        </is>
+      </c>
+      <c r="C59" s="20" t="inlineStr">
+        <is>
+          <t>2join</t>
+        </is>
+      </c>
+      <c r="D59" s="16" t="n">
+        <v>2252.1</v>
+      </c>
+      <c r="E59" s="16" t="n">
+        <v>3597.59</v>
+      </c>
+      <c r="F59" s="17">
+        <f>IF(D59&gt;0, (E59-D59)/D59, 0)</f>
+        <v/>
+      </c>
+      <c r="G59" s="16" t="n">
+        <v>539.9299999999999</v>
+      </c>
+      <c r="H59" s="16" t="n">
+        <v>259.18</v>
+      </c>
+      <c r="I59" s="16" t="n">
+        <v>739.1799999999999</v>
+      </c>
+      <c r="J59" s="16" t="n">
+        <v>1283.08</v>
+      </c>
+      <c r="K59" s="23" t="n">
+        <v>1618242</v>
+      </c>
+      <c r="L59" s="23" t="n">
+        <v>6547</v>
+      </c>
+    </row>
+    <row r="60" ht="20" customHeight="1">
+      <c r="A60" s="9" t="inlineStr">
+        <is>
+          <t>Stress</t>
+        </is>
+      </c>
+      <c r="B60" s="9" t="inlineStr">
+        <is>
+          <t>10,000 conn (16 threads)</t>
+        </is>
+      </c>
+      <c r="C60" s="19" t="inlineStr">
+        <is>
+          <t>3join</t>
+        </is>
+      </c>
+      <c r="D60" s="11" t="n">
+        <v>1739.5</v>
+      </c>
+      <c r="E60" s="11" t="n">
+        <v>1109.4</v>
+      </c>
+      <c r="F60" s="12">
+        <f>IF(D60&gt;0, (E60-D60)/D60, 0)</f>
+        <v/>
+      </c>
+      <c r="G60" s="11" t="n">
+        <v>435.79</v>
+      </c>
+      <c r="H60" s="11" t="n">
+        <v>411.09</v>
+      </c>
+      <c r="I60" s="11" t="n">
+        <v>670.3</v>
+      </c>
+      <c r="J60" s="11" t="n">
+        <v>1322.52</v>
+      </c>
+      <c r="K60" s="23" t="n">
+        <v>3497581</v>
+      </c>
+      <c r="L60" s="23" t="n">
+        <v>5445</v>
+      </c>
+    </row>
+    <row r="61" ht="20" customHeight="1">
+      <c r="A61" s="14" t="inlineStr">
+        <is>
+          <t>Stress</t>
+        </is>
+      </c>
+      <c r="B61" s="14" t="inlineStr">
+        <is>
+          <t>10,000 conn (16 threads)</t>
+        </is>
+      </c>
+      <c r="C61" s="20" t="inlineStr">
+        <is>
+          <t>4join</t>
+        </is>
+      </c>
+      <c r="D61" s="16" t="n">
+        <v>1433.16</v>
+      </c>
+      <c r="E61" s="16" t="n">
+        <v>868.96</v>
+      </c>
+      <c r="F61" s="12">
+        <f>IF(D61&gt;0, (E61-D61)/D61, 0)</f>
+        <v/>
+      </c>
+      <c r="G61" s="16" t="n">
+        <v>384.15</v>
+      </c>
+      <c r="H61" s="16" t="n">
+        <v>560.41</v>
+      </c>
+      <c r="I61" s="16" t="n">
+        <v>782</v>
+      </c>
+      <c r="J61" s="16" t="n">
+        <v>1583.21</v>
+      </c>
+      <c r="K61" s="23" t="n">
+        <v>4355905</v>
+      </c>
+      <c r="L61" s="23" t="n">
+        <v>1326</v>
+      </c>
+    </row>
+    <row r="62"/>
+    <row r="63"/>
+    <row r="64"/>
+    <row r="65"/>
+    <row r="66"/>
+    <row r="67"/>
+    <row r="68"/>
+    <row r="69"/>
+    <row r="70"/>
+    <row r="71"/>
+    <row r="72"/>
+    <row r="73"/>
+    <row r="74"/>
+    <row r="75"/>
+    <row r="76" ht="24" customHeight="1">
+      <c r="A76" s="7" t="inlineStr">
+        <is>
+          <t>3. POST SUITE - WRITE &amp; MULTI-TABLE TRANSACTIONS</t>
+        </is>
+      </c>
+    </row>
+    <row r="77" ht="22" customHeight="1">
+      <c r="A77" s="8" t="inlineStr">
+        <is>
+          <t>Tier</t>
+        </is>
+      </c>
+      <c r="B77" s="8" t="inlineStr">
+        <is>
+          <t>Concurrency</t>
+        </is>
+      </c>
+      <c r="C77" s="8" t="inlineStr">
+        <is>
+          <t>Endpoint</t>
+        </is>
+      </c>
+      <c r="D77" s="8" t="inlineStr">
+        <is>
+          <t>Docker Req/s</t>
+        </is>
+      </c>
+      <c r="E77" s="8" t="inlineStr">
+        <is>
+          <t>BME Req/s</t>
+        </is>
+      </c>
+      <c r="F77" s="8" t="inlineStr">
+        <is>
+          <t>BME Gain (%)</t>
+        </is>
+      </c>
+      <c r="G77" s="8" t="inlineStr">
+        <is>
+          <t>Docker Mean (ms)</t>
+        </is>
+      </c>
+      <c r="H77" s="8" t="inlineStr">
+        <is>
+          <t>BME Mean (ms)</t>
+        </is>
+      </c>
+      <c r="I77" s="8" t="inlineStr">
+        <is>
+          <t>Docker P95 (ms)</t>
+        </is>
+      </c>
+      <c r="J77" s="8" t="inlineStr">
+        <is>
+          <t>BME P95 (ms)</t>
+        </is>
+      </c>
+      <c r="K77" s="8" t="inlineStr">
+        <is>
+          <t>Docker Errors</t>
+        </is>
+      </c>
+      <c r="L77" s="8" t="inlineStr">
+        <is>
+          <t>BME Errors</t>
+        </is>
+      </c>
+    </row>
+    <row r="78" ht="20" customHeight="1">
+      <c r="A78" s="9" t="inlineStr">
+        <is>
+          <t>POC</t>
+        </is>
+      </c>
+      <c r="B78" s="9" t="inlineStr">
+        <is>
+          <t>20 conn (2 threads)</t>
+        </is>
+      </c>
+      <c r="C78" s="19" t="inlineStr">
+        <is>
+          <t>1table</t>
+        </is>
+      </c>
+      <c r="D78" s="11" t="n">
+        <v>9324.9</v>
+      </c>
+      <c r="E78" s="11" t="n">
+        <v>10087.07</v>
+      </c>
+      <c r="F78" s="17">
+        <f>IF(D78&gt;0, (E78-D78)/D78, 0)</f>
+        <v/>
+      </c>
+      <c r="G78" s="11" t="n">
+        <v>2.31</v>
+      </c>
+      <c r="H78" s="11" t="n">
+        <v>2.42</v>
+      </c>
+      <c r="I78" s="11" t="n">
+        <v>4.11</v>
+      </c>
+      <c r="J78" s="11" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="K78" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="L78" s="13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="79" ht="20" customHeight="1">
+      <c r="A79" s="14" t="inlineStr">
+        <is>
+          <t>POC</t>
+        </is>
+      </c>
+      <c r="B79" s="14" t="inlineStr">
+        <is>
+          <t>20 conn (2 threads)</t>
+        </is>
+      </c>
+      <c r="C79" s="20" t="inlineStr">
+        <is>
+          <t>2table</t>
+        </is>
+      </c>
+      <c r="D79" s="16" t="n">
+        <v>5274.29</v>
+      </c>
+      <c r="E79" s="16" t="n">
+        <v>5556.55</v>
+      </c>
+      <c r="F79" s="17">
+        <f>IF(D79&gt;0, (E79-D79)/D79, 0)</f>
+        <v/>
+      </c>
+      <c r="G79" s="16" t="n">
+        <v>3.97</v>
+      </c>
+      <c r="H79" s="16" t="n">
+        <v>3.85</v>
+      </c>
+      <c r="I79" s="16" t="n">
+        <v>6.42</v>
+      </c>
+      <c r="J79" s="16" t="n">
+        <v>5.75</v>
+      </c>
+      <c r="K79" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="L79" s="18" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="80" ht="20" customHeight="1">
+      <c r="A80" s="9" t="inlineStr">
+        <is>
+          <t>POC</t>
+        </is>
+      </c>
+      <c r="B80" s="9" t="inlineStr">
+        <is>
+          <t>20 conn (2 threads)</t>
+        </is>
+      </c>
+      <c r="C80" s="19" t="inlineStr">
+        <is>
+          <t>3table</t>
+        </is>
+      </c>
+      <c r="D80" s="11" t="n">
+        <v>4457.83</v>
+      </c>
+      <c r="E80" s="11" t="n">
+        <v>4852.79</v>
+      </c>
+      <c r="F80" s="17">
+        <f>IF(D80&gt;0, (E80-D80)/D80, 0)</f>
+        <v/>
+      </c>
+      <c r="G80" s="11" t="n">
+        <v>4.66</v>
+      </c>
+      <c r="H80" s="11" t="n">
+        <v>4.31</v>
+      </c>
+      <c r="I80" s="11" t="n">
+        <v>7.44</v>
+      </c>
+      <c r="J80" s="11" t="n">
+        <v>6.31</v>
+      </c>
+      <c r="K80" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="L80" s="13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="81" ht="20" customHeight="1">
+      <c r="A81" s="14" t="inlineStr">
+        <is>
+          <t>POC</t>
+        </is>
+      </c>
+      <c r="B81" s="14" t="inlineStr">
+        <is>
+          <t>20 conn (2 threads)</t>
+        </is>
+      </c>
+      <c r="C81" s="20" t="inlineStr">
+        <is>
+          <t>4table</t>
+        </is>
+      </c>
+      <c r="D81" s="16" t="n">
+        <v>3360.52</v>
+      </c>
+      <c r="E81" s="16" t="n">
+        <v>3651.39</v>
+      </c>
+      <c r="F81" s="17">
+        <f>IF(D81&gt;0, (E81-D81)/D81, 0)</f>
+        <v/>
+      </c>
+      <c r="G81" s="16" t="n">
+        <v>6.45</v>
+      </c>
+      <c r="H81" s="16" t="n">
+        <v>5.65</v>
+      </c>
+      <c r="I81" s="16" t="n">
+        <v>9.93</v>
+      </c>
+      <c r="J81" s="16" t="n">
+        <v>8.33</v>
+      </c>
+      <c r="K81" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="L81" s="18" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="82" ht="20" customHeight="1">
+      <c r="A82" s="9" t="inlineStr">
+        <is>
+          <t>Small</t>
+        </is>
+      </c>
+      <c r="B82" s="9" t="inlineStr">
+        <is>
+          <t>100 conn (4 threads)</t>
+        </is>
+      </c>
+      <c r="C82" s="19" t="inlineStr">
+        <is>
+          <t>1table</t>
+        </is>
+      </c>
+      <c r="D82" s="11" t="n">
+        <v>8698.629999999999</v>
+      </c>
+      <c r="E82" s="11" t="n">
+        <v>13839.32</v>
+      </c>
+      <c r="F82" s="17">
+        <f>IF(D82&gt;0, (E82-D82)/D82, 0)</f>
+        <v/>
+      </c>
+      <c r="G82" s="11" t="n">
+        <v>22.51</v>
+      </c>
+      <c r="H82" s="11" t="n">
+        <v>8.800000000000001</v>
+      </c>
+      <c r="I82" s="11" t="n">
+        <v>96.52</v>
+      </c>
+      <c r="J82" s="11" t="n">
+        <v>20.59</v>
+      </c>
+      <c r="K82" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="L82" s="13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="83" ht="20" customHeight="1">
+      <c r="A83" s="14" t="inlineStr">
+        <is>
+          <t>Small</t>
+        </is>
+      </c>
+      <c r="B83" s="14" t="inlineStr">
+        <is>
+          <t>100 conn (4 threads)</t>
+        </is>
+      </c>
+      <c r="C83" s="20" t="inlineStr">
+        <is>
+          <t>2table</t>
+        </is>
+      </c>
+      <c r="D83" s="16" t="n">
+        <v>6258.85</v>
+      </c>
+      <c r="E83" s="16" t="n">
+        <v>7563.67</v>
+      </c>
+      <c r="F83" s="17">
+        <f>IF(D83&gt;0, (E83-D83)/D83, 0)</f>
+        <v/>
+      </c>
+      <c r="G83" s="16" t="n">
+        <v>18.06</v>
+      </c>
+      <c r="H83" s="16" t="n">
+        <v>14.51</v>
+      </c>
+      <c r="I83" s="16" t="n">
+        <v>44.39</v>
+      </c>
+      <c r="J83" s="16" t="n">
+        <v>32.41</v>
+      </c>
+      <c r="K83" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="L83" s="18" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="84" ht="20" customHeight="1">
+      <c r="A84" s="9" t="inlineStr">
+        <is>
+          <t>Small</t>
+        </is>
+      </c>
+      <c r="B84" s="9" t="inlineStr">
+        <is>
+          <t>100 conn (4 threads)</t>
+        </is>
+      </c>
+      <c r="C84" s="19" t="inlineStr">
+        <is>
+          <t>3table</t>
+        </is>
+      </c>
+      <c r="D84" s="11" t="n">
+        <v>5410.04</v>
+      </c>
+      <c r="E84" s="11" t="n">
+        <v>6236.25</v>
+      </c>
+      <c r="F84" s="17">
+        <f>IF(D84&gt;0, (E84-D84)/D84, 0)</f>
+        <v/>
+      </c>
+      <c r="G84" s="11" t="n">
+        <v>20.07</v>
+      </c>
+      <c r="H84" s="11" t="n">
+        <v>17.41</v>
+      </c>
+      <c r="I84" s="11" t="n">
+        <v>44.97</v>
+      </c>
+      <c r="J84" s="11" t="n">
+        <v>38.3</v>
+      </c>
+      <c r="K84" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="L84" s="13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="85" ht="20" customHeight="1">
+      <c r="A85" s="14" t="inlineStr">
+        <is>
+          <t>Small</t>
+        </is>
+      </c>
+      <c r="B85" s="14" t="inlineStr">
+        <is>
+          <t>100 conn (4 threads)</t>
+        </is>
+      </c>
+      <c r="C85" s="20" t="inlineStr">
+        <is>
+          <t>4table</t>
+        </is>
+      </c>
+      <c r="D85" s="16" t="n">
+        <v>3927</v>
+      </c>
+      <c r="E85" s="16" t="n">
+        <v>4299.57</v>
+      </c>
+      <c r="F85" s="17">
+        <f>IF(D85&gt;0, (E85-D85)/D85, 0)</f>
+        <v/>
+      </c>
+      <c r="G85" s="16" t="n">
+        <v>27.07</v>
+      </c>
+      <c r="H85" s="16" t="n">
+        <v>24.83</v>
+      </c>
+      <c r="I85" s="16" t="n">
+        <v>58.67</v>
+      </c>
+      <c r="J85" s="16" t="n">
+        <v>54.7</v>
+      </c>
+      <c r="K85" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="L85" s="18" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="86" ht="20" customHeight="1">
+      <c r="A86" s="9" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="B86" s="9" t="inlineStr">
+        <is>
+          <t>500 conn (8 threads)</t>
+        </is>
+      </c>
+      <c r="C86" s="19" t="inlineStr">
+        <is>
+          <t>1table</t>
+        </is>
+      </c>
+      <c r="D86" s="11" t="n">
+        <v>7384.74</v>
+      </c>
+      <c r="E86" s="11" t="n">
+        <v>8950.27</v>
+      </c>
+      <c r="F86" s="17">
+        <f>IF(D86&gt;0, (E86-D86)/D86, 0)</f>
+        <v/>
+      </c>
+      <c r="G86" s="11" t="n">
+        <v>202.47</v>
+      </c>
+      <c r="H86" s="11" t="n">
+        <v>171.07</v>
+      </c>
+      <c r="I86" s="11" t="n">
+        <v>925.89</v>
+      </c>
+      <c r="J86" s="11" t="n">
+        <v>771.48</v>
+      </c>
+      <c r="K86" s="23" t="n">
+        <v>14776</v>
+      </c>
+      <c r="L86" s="23" t="n">
+        <v>4819</v>
+      </c>
+    </row>
+    <row r="87" ht="20" customHeight="1">
+      <c r="A87" s="14" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="B87" s="14" t="inlineStr">
+        <is>
+          <t>500 conn (8 threads)</t>
+        </is>
+      </c>
+      <c r="C87" s="20" t="inlineStr">
+        <is>
+          <t>2table</t>
+        </is>
+      </c>
+      <c r="D87" s="16" t="n">
+        <v>4952.12</v>
+      </c>
+      <c r="E87" s="16" t="n">
+        <v>5612.02</v>
+      </c>
+      <c r="F87" s="17">
+        <f>IF(D87&gt;0, (E87-D87)/D87, 0)</f>
+        <v/>
+      </c>
+      <c r="G87" s="16" t="n">
+        <v>196.89</v>
+      </c>
+      <c r="H87" s="16" t="n">
+        <v>164.66</v>
+      </c>
+      <c r="I87" s="16" t="n">
+        <v>837.21</v>
+      </c>
+      <c r="J87" s="16" t="n">
+        <v>676.5599999999999</v>
+      </c>
+      <c r="K87" s="23" t="n">
+        <v>7519</v>
+      </c>
+      <c r="L87" s="23" t="n">
+        <v>2012</v>
+      </c>
+    </row>
+    <row r="88" ht="20" customHeight="1">
+      <c r="A88" s="9" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="B88" s="9" t="inlineStr">
+        <is>
+          <t>500 conn (8 threads)</t>
+        </is>
+      </c>
+      <c r="C88" s="19" t="inlineStr">
+        <is>
+          <t>3table</t>
+        </is>
+      </c>
+      <c r="D88" s="11" t="n">
+        <v>4263.4</v>
+      </c>
+      <c r="E88" s="11" t="n">
+        <v>4655.97</v>
+      </c>
+      <c r="F88" s="17">
+        <f>IF(D88&gt;0, (E88-D88)/D88, 0)</f>
+        <v/>
+      </c>
+      <c r="G88" s="11" t="n">
+        <v>194</v>
+      </c>
+      <c r="H88" s="11" t="n">
+        <v>163.46</v>
+      </c>
+      <c r="I88" s="11" t="n">
+        <v>774.13</v>
+      </c>
+      <c r="J88" s="11" t="n">
+        <v>607.6799999999999</v>
+      </c>
+      <c r="K88" s="23" t="n">
+        <v>5172</v>
+      </c>
+      <c r="L88" s="23" t="n">
+        <v>1203</v>
+      </c>
+    </row>
+    <row r="89" ht="20" customHeight="1">
+      <c r="A89" s="14" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="B89" s="14" t="inlineStr">
+        <is>
+          <t>500 conn (8 threads)</t>
+        </is>
+      </c>
+      <c r="C89" s="20" t="inlineStr">
+        <is>
+          <t>4table</t>
+        </is>
+      </c>
+      <c r="D89" s="16" t="n">
+        <v>2932.88</v>
+      </c>
+      <c r="E89" s="16" t="n">
+        <v>3155.03</v>
+      </c>
+      <c r="F89" s="17">
+        <f>IF(D89&gt;0, (E89-D89)/D89, 0)</f>
+        <v/>
+      </c>
+      <c r="G89" s="16" t="n">
+        <v>255.98</v>
+      </c>
+      <c r="H89" s="16" t="n">
+        <v>239.71</v>
+      </c>
+      <c r="I89" s="16" t="n">
+        <v>1035.98</v>
+      </c>
+      <c r="J89" s="16" t="n">
+        <v>935.54</v>
+      </c>
+      <c r="K89" s="23" t="n">
+        <v>23500</v>
+      </c>
+      <c r="L89" s="23" t="n">
+        <v>12612</v>
+      </c>
+    </row>
+    <row r="90" ht="20" customHeight="1">
+      <c r="A90" s="9" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="B90" s="9" t="inlineStr">
+        <is>
+          <t>2,000 conn (8 threads)</t>
+        </is>
+      </c>
+      <c r="C90" s="19" t="inlineStr">
+        <is>
+          <t>1table</t>
+        </is>
+      </c>
+      <c r="D90" s="11" t="n">
+        <v>7091.58</v>
+      </c>
+      <c r="E90" s="11" t="n">
+        <v>8728.6</v>
+      </c>
+      <c r="F90" s="17">
+        <f>IF(D90&gt;0, (E90-D90)/D90, 0)</f>
+        <v/>
+      </c>
+      <c r="G90" s="11" t="n">
+        <v>325.16</v>
+      </c>
+      <c r="H90" s="11" t="n">
+        <v>277.94</v>
+      </c>
+      <c r="I90" s="11" t="n">
+        <v>945.62</v>
+      </c>
+      <c r="J90" s="11" t="n">
+        <v>821.12</v>
+      </c>
+      <c r="K90" s="23" t="n">
+        <v>65027</v>
+      </c>
+      <c r="L90" s="23" t="n">
+        <v>21979</v>
+      </c>
+    </row>
+    <row r="91" ht="20" customHeight="1">
+      <c r="A91" s="14" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="B91" s="14" t="inlineStr">
+        <is>
+          <t>2,000 conn (8 threads)</t>
+        </is>
+      </c>
+      <c r="C91" s="20" t="inlineStr">
+        <is>
+          <t>2table</t>
+        </is>
+      </c>
+      <c r="D91" s="16" t="n">
+        <v>4826.72</v>
+      </c>
+      <c r="E91" s="16" t="n">
+        <v>5453.79</v>
+      </c>
+      <c r="F91" s="17">
+        <f>IF(D91&gt;0, (E91-D91)/D91, 0)</f>
+        <v/>
+      </c>
+      <c r="G91" s="16" t="n">
+        <v>440.95</v>
+      </c>
+      <c r="H91" s="16" t="n">
+        <v>399.35</v>
+      </c>
+      <c r="I91" s="16" t="n">
+        <v>1122.96</v>
+      </c>
+      <c r="J91" s="16" t="n">
+        <v>1022.8</v>
+      </c>
+      <c r="K91" s="23" t="n">
+        <v>64129</v>
+      </c>
+      <c r="L91" s="23" t="n">
+        <v>28847</v>
+      </c>
+    </row>
+    <row r="92" ht="20" customHeight="1">
+      <c r="A92" s="9" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="B92" s="9" t="inlineStr">
+        <is>
+          <t>2,000 conn (8 threads)</t>
+        </is>
+      </c>
+      <c r="C92" s="19" t="inlineStr">
+        <is>
+          <t>3table</t>
+        </is>
+      </c>
+      <c r="D92" s="11" t="n">
+        <v>4170.34</v>
+      </c>
+      <c r="E92" s="11" t="n">
+        <v>4548.17</v>
+      </c>
+      <c r="F92" s="17">
+        <f>IF(D92&gt;0, (E92-D92)/D92, 0)</f>
+        <v/>
+      </c>
+      <c r="G92" s="11" t="n">
+        <v>496.05</v>
+      </c>
+      <c r="H92" s="11" t="n">
+        <v>463.02</v>
+      </c>
+      <c r="I92" s="11" t="n">
+        <v>1211.24</v>
+      </c>
+      <c r="J92" s="11" t="n">
+        <v>1122.53</v>
+      </c>
+      <c r="K92" s="23" t="n">
+        <v>76588</v>
+      </c>
+      <c r="L92" s="23" t="n">
+        <v>39318</v>
+      </c>
+    </row>
+    <row r="93" ht="20" customHeight="1">
+      <c r="A93" s="14" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="B93" s="14" t="inlineStr">
+        <is>
+          <t>2,000 conn (8 threads)</t>
+        </is>
+      </c>
+      <c r="C93" s="20" t="inlineStr">
+        <is>
+          <t>4table</t>
+        </is>
+      </c>
+      <c r="D93" s="16" t="n">
+        <v>2896.76</v>
+      </c>
+      <c r="E93" s="16" t="n">
+        <v>3068.06</v>
+      </c>
+      <c r="F93" s="17">
+        <f>IF(D93&gt;0, (E93-D93)/D93, 0)</f>
+        <v/>
+      </c>
+      <c r="G93" s="16" t="n">
+        <v>646.6</v>
+      </c>
+      <c r="H93" s="16" t="n">
+        <v>628</v>
+      </c>
+      <c r="I93" s="16" t="n">
+        <v>1451.61</v>
+      </c>
+      <c r="J93" s="16" t="n">
+        <v>1389.48</v>
+      </c>
+      <c r="K93" s="23" t="n">
+        <v>207120</v>
+      </c>
+      <c r="L93" s="23" t="n">
+        <v>157846</v>
+      </c>
+    </row>
+    <row r="94" ht="20" customHeight="1">
+      <c r="A94" s="9" t="inlineStr">
+        <is>
+          <t>Stress</t>
+        </is>
+      </c>
+      <c r="B94" s="9" t="inlineStr">
+        <is>
+          <t>10,000 conn (16 threads)</t>
+        </is>
+      </c>
+      <c r="C94" s="19" t="inlineStr">
+        <is>
+          <t>1table</t>
+        </is>
+      </c>
+      <c r="D94" s="11" t="n">
+        <v>6759.35</v>
+      </c>
+      <c r="E94" s="11" t="n">
+        <v>8641.09</v>
+      </c>
+      <c r="F94" s="17">
+        <f>IF(D94&gt;0, (E94-D94)/D94, 0)</f>
+        <v/>
+      </c>
+      <c r="G94" s="11" t="n">
+        <v>812.0700000000001</v>
+      </c>
+      <c r="H94" s="11" t="n">
+        <v>540.45</v>
+      </c>
+      <c r="I94" s="11" t="n">
+        <v>1777.54</v>
+      </c>
+      <c r="J94" s="11" t="n">
+        <v>1544.14</v>
+      </c>
+      <c r="K94" s="23" t="n">
+        <v>9930089</v>
+      </c>
+      <c r="L94" s="23" t="n">
+        <v>11396035</v>
+      </c>
+    </row>
+    <row r="95" ht="20" customHeight="1">
+      <c r="A95" s="14" t="inlineStr">
+        <is>
+          <t>Stress</t>
+        </is>
+      </c>
+      <c r="B95" s="14" t="inlineStr">
+        <is>
+          <t>10,000 conn (16 threads)</t>
+        </is>
+      </c>
+      <c r="C95" s="20" t="inlineStr">
+        <is>
+          <t>2table</t>
+        </is>
+      </c>
+      <c r="D95" s="16" t="n">
+        <v>4730.62</v>
+      </c>
+      <c r="E95" s="16" t="n">
+        <v>5488.15</v>
+      </c>
+      <c r="F95" s="17">
+        <f>IF(D95&gt;0, (E95-D95)/D95, 0)</f>
+        <v/>
+      </c>
+      <c r="G95" s="16" t="n">
+        <v>667.74</v>
+      </c>
+      <c r="H95" s="16" t="n">
+        <v>768.85</v>
+      </c>
+      <c r="I95" s="16" t="n">
+        <v>1940.59</v>
+      </c>
+      <c r="J95" s="16" t="n">
+        <v>1915.8</v>
+      </c>
+      <c r="K95" s="23" t="n">
+        <v>13844249</v>
+      </c>
+      <c r="L95" s="23" t="n">
+        <v>11436935</v>
+      </c>
+    </row>
+    <row r="96" ht="20" customHeight="1">
+      <c r="A96" s="9" t="inlineStr">
+        <is>
+          <t>Stress</t>
+        </is>
+      </c>
+      <c r="B96" s="9" t="inlineStr">
+        <is>
+          <t>10,000 conn (16 threads)</t>
+        </is>
+      </c>
+      <c r="C96" s="19" t="inlineStr">
+        <is>
+          <t>3table</t>
+        </is>
+      </c>
+      <c r="D96" s="11" t="n">
+        <v>4106.6</v>
+      </c>
+      <c r="E96" s="11" t="n">
+        <v>4571.22</v>
+      </c>
+      <c r="F96" s="17">
+        <f>IF(D96&gt;0, (E96-D96)/D96, 0)</f>
+        <v/>
+      </c>
+      <c r="G96" s="11" t="n">
+        <v>402.45</v>
+      </c>
+      <c r="H96" s="11" t="n">
+        <v>534.55</v>
+      </c>
+      <c r="I96" s="11" t="n">
+        <v>1895.41</v>
+      </c>
+      <c r="J96" s="11" t="n">
+        <v>1956.34</v>
+      </c>
+      <c r="K96" s="23" t="n">
+        <v>15235684</v>
+      </c>
+      <c r="L96" s="23" t="n">
+        <v>15212131</v>
+      </c>
+    </row>
+    <row r="97" ht="20" customHeight="1">
+      <c r="A97" s="14" t="inlineStr">
+        <is>
+          <t>Stress</t>
+        </is>
+      </c>
+      <c r="B97" s="14" t="inlineStr">
+        <is>
+          <t>10,000 conn (16 threads)</t>
+        </is>
+      </c>
+      <c r="C97" s="20" t="inlineStr">
+        <is>
+          <t>4table</t>
+        </is>
+      </c>
+      <c r="D97" s="16" t="n">
+        <v>2874.17</v>
+      </c>
+      <c r="E97" s="16" t="n">
+        <v>3053.83</v>
+      </c>
+      <c r="F97" s="17">
+        <f>IF(D97&gt;0, (E97-D97)/D97, 0)</f>
+        <v/>
+      </c>
+      <c r="G97" s="16" t="n">
+        <v>150.05</v>
+      </c>
+      <c r="H97" s="16" t="n">
+        <v>142.18</v>
+      </c>
+      <c r="I97" s="16" t="n">
+        <v>716.75</v>
+      </c>
+      <c r="J97" s="16" t="n">
+        <v>633</v>
+      </c>
+      <c r="K97" s="23" t="n">
+        <v>13106737</v>
+      </c>
+      <c r="L97" s="23" t="n">
+        <v>13761138</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="A2:L2"/>
+    <mergeCell ref="A76:L76"/>
+    <mergeCell ref="A1:L1"/>
+    <mergeCell ref="A40:L40"/>
+    <mergeCell ref="A4:L4"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
benchmarks: Python (opt.) get_with_index tier POC completed (20 runs DKR & BME)
</commit_message>
<xml_diff>
--- a/Programming_Benchmark_Report.xlsx
+++ b/Programming_Benchmark_Report.xlsx
@@ -23926,26 +23926,26 @@
         </is>
       </c>
       <c r="D42" s="11" t="n">
-        <v>2279.05</v>
+        <v>3202.93</v>
       </c>
       <c r="E42" s="11" t="n">
-        <v>3023.71</v>
-      </c>
-      <c r="F42" s="17">
+        <v>2913.31</v>
+      </c>
+      <c r="F42" s="12">
         <f>IF(D42&gt;0, (E42-D42)/D42, 0)</f>
         <v/>
       </c>
       <c r="G42" s="11" t="n">
-        <v>8.92</v>
+        <v>6.4</v>
       </c>
       <c r="H42" s="11" t="n">
-        <v>6.71</v>
+        <v>7.31</v>
       </c>
       <c r="I42" s="11" t="n">
-        <v>15.6</v>
+        <v>11.54</v>
       </c>
       <c r="J42" s="11" t="n">
-        <v>12.16</v>
+        <v>14.43</v>
       </c>
       <c r="K42" s="13" t="n">
         <v>0</v>
@@ -23971,26 +23971,26 @@
         </is>
       </c>
       <c r="D43" s="16" t="n">
-        <v>2575.84</v>
+        <v>3075.25</v>
       </c>
       <c r="E43" s="16" t="n">
-        <v>2454.7</v>
+        <v>2825.46</v>
       </c>
       <c r="F43" s="12">
         <f>IF(D43&gt;0, (E43-D43)/D43, 0)</f>
         <v/>
       </c>
       <c r="G43" s="16" t="n">
-        <v>7.82</v>
+        <v>6.58</v>
       </c>
       <c r="H43" s="16" t="n">
-        <v>8.460000000000001</v>
+        <v>7.3</v>
       </c>
       <c r="I43" s="16" t="n">
-        <v>12.15</v>
+        <v>10.99</v>
       </c>
       <c r="J43" s="16" t="n">
-        <v>17.33</v>
+        <v>14.39</v>
       </c>
       <c r="K43" s="18" t="n">
         <v>0</v>
@@ -24016,26 +24016,26 @@
         </is>
       </c>
       <c r="D44" s="11" t="n">
-        <v>1723.85</v>
+        <v>1762.95</v>
       </c>
       <c r="E44" s="11" t="n">
-        <v>1607.55</v>
+        <v>1705.34</v>
       </c>
       <c r="F44" s="12">
         <f>IF(D44&gt;0, (E44-D44)/D44, 0)</f>
         <v/>
       </c>
       <c r="G44" s="11" t="n">
-        <v>11.63</v>
+        <v>11.4</v>
       </c>
       <c r="H44" s="11" t="n">
-        <v>12.63</v>
+        <v>12.01</v>
       </c>
       <c r="I44" s="11" t="n">
-        <v>18.04</v>
+        <v>18.79</v>
       </c>
       <c r="J44" s="11" t="n">
-        <v>24.07</v>
+        <v>21.81</v>
       </c>
       <c r="K44" s="13" t="n">
         <v>0</v>
@@ -24061,26 +24061,26 @@
         </is>
       </c>
       <c r="D45" s="16" t="n">
-        <v>1369.93</v>
+        <v>1697.24</v>
       </c>
       <c r="E45" s="16" t="n">
-        <v>1540.36</v>
-      </c>
-      <c r="F45" s="17">
+        <v>1606.63</v>
+      </c>
+      <c r="F45" s="12">
         <f>IF(D45&gt;0, (E45-D45)/D45, 0)</f>
         <v/>
       </c>
       <c r="G45" s="16" t="n">
-        <v>14.66</v>
+        <v>11.86</v>
       </c>
       <c r="H45" s="16" t="n">
-        <v>13.08</v>
+        <v>12.74</v>
       </c>
       <c r="I45" s="16" t="n">
-        <v>23.59</v>
+        <v>19.65</v>
       </c>
       <c r="J45" s="16" t="n">
-        <v>25.1</v>
+        <v>23.01</v>
       </c>
       <c r="K45" s="18" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
benchmarks: Python (opt.) get_with_index tier SMALL completed (20 runs DKR & BME)
</commit_message>
<xml_diff>
--- a/Programming_Benchmark_Report.xlsx
+++ b/Programming_Benchmark_Report.xlsx
@@ -24106,26 +24106,26 @@
         </is>
       </c>
       <c r="D46" s="11" t="n">
-        <v>2394.42</v>
+        <v>4225.05</v>
       </c>
       <c r="E46" s="11" t="n">
-        <v>4660.62</v>
+        <v>4754.7</v>
       </c>
       <c r="F46" s="17">
         <f>IF(D46&gt;0, (E46-D46)/D46, 0)</f>
         <v/>
       </c>
       <c r="G46" s="11" t="n">
-        <v>41.76</v>
+        <v>24.48</v>
       </c>
       <c r="H46" s="11" t="n">
-        <v>22.23</v>
+        <v>22.34</v>
       </c>
       <c r="I46" s="11" t="n">
-        <v>65.51000000000001</v>
+        <v>50.69</v>
       </c>
       <c r="J46" s="11" t="n">
-        <v>49.02</v>
+        <v>53.03</v>
       </c>
       <c r="K46" s="13" t="n">
         <v>0</v>
@@ -24151,26 +24151,26 @@
         </is>
       </c>
       <c r="D47" s="16" t="n">
-        <v>2770.45</v>
+        <v>3954.94</v>
       </c>
       <c r="E47" s="16" t="n">
-        <v>4314.84</v>
+        <v>4381.76</v>
       </c>
       <c r="F47" s="17">
         <f>IF(D47&gt;0, (E47-D47)/D47, 0)</f>
         <v/>
       </c>
       <c r="G47" s="16" t="n">
-        <v>36.09</v>
+        <v>26.11</v>
       </c>
       <c r="H47" s="16" t="n">
-        <v>23.95</v>
+        <v>23.91</v>
       </c>
       <c r="I47" s="16" t="n">
-        <v>55.82</v>
+        <v>54.48</v>
       </c>
       <c r="J47" s="16" t="n">
-        <v>51.83</v>
+        <v>52.62</v>
       </c>
       <c r="K47" s="18" t="n">
         <v>0</v>
@@ -24196,26 +24196,26 @@
         </is>
       </c>
       <c r="D48" s="11" t="n">
-        <v>1978.06</v>
+        <v>1759.79</v>
       </c>
       <c r="E48" s="11" t="n">
-        <v>1767.4</v>
-      </c>
-      <c r="F48" s="12">
+        <v>1793.58</v>
+      </c>
+      <c r="F48" s="17">
         <f>IF(D48&gt;0, (E48-D48)/D48, 0)</f>
         <v/>
       </c>
       <c r="G48" s="11" t="n">
-        <v>51.18</v>
+        <v>60.14</v>
       </c>
       <c r="H48" s="11" t="n">
-        <v>58.41</v>
+        <v>59.2</v>
       </c>
       <c r="I48" s="11" t="n">
-        <v>94.48</v>
+        <v>137.34</v>
       </c>
       <c r="J48" s="11" t="n">
-        <v>130.52</v>
+        <v>136.26</v>
       </c>
       <c r="K48" s="13" t="n">
         <v>0</v>
@@ -24241,26 +24241,26 @@
         </is>
       </c>
       <c r="D49" s="16" t="n">
-        <v>1663.88</v>
+        <v>1753.26</v>
       </c>
       <c r="E49" s="16" t="n">
-        <v>1759.4</v>
+        <v>1783.16</v>
       </c>
       <c r="F49" s="17">
         <f>IF(D49&gt;0, (E49-D49)/D49, 0)</f>
         <v/>
       </c>
       <c r="G49" s="16" t="n">
-        <v>60.73</v>
+        <v>59.17</v>
       </c>
       <c r="H49" s="16" t="n">
-        <v>58.15</v>
+        <v>58.59</v>
       </c>
       <c r="I49" s="16" t="n">
-        <v>110.48</v>
+        <v>126.35</v>
       </c>
       <c r="J49" s="16" t="n">
-        <v>124.6</v>
+        <v>128.3</v>
       </c>
       <c r="K49" s="18" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
benchmarks: Python (opt.) get_with_index tier GENERAL completed (20 runs DKR & BME)
</commit_message>
<xml_diff>
--- a/Programming_Benchmark_Report.xlsx
+++ b/Programming_Benchmark_Report.xlsx
@@ -24286,32 +24286,32 @@
         </is>
       </c>
       <c r="D50" s="11" t="n">
-        <v>2221.51</v>
+        <v>4100.48</v>
       </c>
       <c r="E50" s="11" t="n">
-        <v>4496.02</v>
+        <v>4646.94</v>
       </c>
       <c r="F50" s="17">
         <f>IF(D50&gt;0, (E50-D50)/D50, 0)</f>
         <v/>
       </c>
       <c r="G50" s="11" t="n">
-        <v>229.8</v>
+        <v>123.88</v>
       </c>
       <c r="H50" s="11" t="n">
-        <v>114.78</v>
+        <v>118.14</v>
       </c>
       <c r="I50" s="11" t="n">
-        <v>471.67</v>
+        <v>225.88</v>
       </c>
       <c r="J50" s="11" t="n">
-        <v>202.05</v>
-      </c>
-      <c r="K50" s="13" t="n">
-        <v>0</v>
+        <v>263.55</v>
+      </c>
+      <c r="K50" s="23" t="n">
+        <v>6</v>
       </c>
       <c r="L50" s="23" t="n">
-        <v>2</v>
+        <v>205</v>
       </c>
     </row>
     <row r="51" ht="20" customHeight="1">
@@ -24331,32 +24331,32 @@
         </is>
       </c>
       <c r="D51" s="16" t="n">
-        <v>2494.54</v>
+        <v>3897.57</v>
       </c>
       <c r="E51" s="16" t="n">
-        <v>4243.25</v>
+        <v>4319.43</v>
       </c>
       <c r="F51" s="17">
         <f>IF(D51&gt;0, (E51-D51)/D51, 0)</f>
         <v/>
       </c>
       <c r="G51" s="16" t="n">
-        <v>209.93</v>
+        <v>134.41</v>
       </c>
       <c r="H51" s="16" t="n">
-        <v>132.43</v>
+        <v>142.45</v>
       </c>
       <c r="I51" s="16" t="n">
-        <v>435.76</v>
+        <v>284.87</v>
       </c>
       <c r="J51" s="16" t="n">
-        <v>355.11</v>
-      </c>
-      <c r="K51" s="18" t="n">
-        <v>0</v>
+        <v>424.99</v>
+      </c>
+      <c r="K51" s="23" t="n">
+        <v>3</v>
       </c>
       <c r="L51" s="23" t="n">
-        <v>1</v>
+        <v>255</v>
       </c>
     </row>
     <row r="52" ht="20" customHeight="1">
@@ -24376,32 +24376,32 @@
         </is>
       </c>
       <c r="D52" s="11" t="n">
-        <v>1783.44</v>
+        <v>1657.1</v>
       </c>
       <c r="E52" s="11" t="n">
-        <v>1679.34</v>
-      </c>
-      <c r="F52" s="12">
+        <v>1700.94</v>
+      </c>
+      <c r="F52" s="17">
         <f>IF(D52&gt;0, (E52-D52)/D52, 0)</f>
         <v/>
       </c>
       <c r="G52" s="11" t="n">
-        <v>308.25</v>
+        <v>328.9</v>
       </c>
       <c r="H52" s="11" t="n">
-        <v>309.43</v>
+        <v>321.89</v>
       </c>
       <c r="I52" s="11" t="n">
-        <v>795.98</v>
+        <v>850.4</v>
       </c>
       <c r="J52" s="11" t="n">
-        <v>844.86</v>
+        <v>828.98</v>
       </c>
       <c r="K52" s="23" t="n">
-        <v>314</v>
+        <v>3020</v>
       </c>
       <c r="L52" s="23" t="n">
-        <v>21</v>
+        <v>1437</v>
       </c>
     </row>
     <row r="53" ht="20" customHeight="1">
@@ -24421,32 +24421,32 @@
         </is>
       </c>
       <c r="D53" s="16" t="n">
-        <v>1445.35</v>
+        <v>1634.28</v>
       </c>
       <c r="E53" s="16" t="n">
-        <v>1665.81</v>
+        <v>1681.42</v>
       </c>
       <c r="F53" s="17">
         <f>IF(D53&gt;0, (E53-D53)/D53, 0)</f>
         <v/>
       </c>
       <c r="G53" s="16" t="n">
-        <v>367.92</v>
+        <v>333.3</v>
       </c>
       <c r="H53" s="16" t="n">
-        <v>306.52</v>
+        <v>325.69</v>
       </c>
       <c r="I53" s="16" t="n">
-        <v>896.09</v>
+        <v>868.42</v>
       </c>
       <c r="J53" s="16" t="n">
-        <v>801.27</v>
+        <v>845.6</v>
       </c>
       <c r="K53" s="23" t="n">
-        <v>967</v>
+        <v>3775</v>
       </c>
       <c r="L53" s="23" t="n">
-        <v>19</v>
+        <v>2214</v>
       </c>
     </row>
     <row r="54" ht="20" customHeight="1">

</xml_diff>

<commit_message>
benchmarks: Python (opt.) get_with_index tier HIGH completed (20 runs DKR & BME)
</commit_message>
<xml_diff>
--- a/Programming_Benchmark_Report.xlsx
+++ b/Programming_Benchmark_Report.xlsx
@@ -24466,32 +24466,32 @@
         </is>
       </c>
       <c r="D54" s="11" t="n">
-        <v>2205.47</v>
+        <v>3963.58</v>
       </c>
       <c r="E54" s="11" t="n">
-        <v>4407.93</v>
+        <v>4508.28</v>
       </c>
       <c r="F54" s="17">
         <f>IF(D54&gt;0, (E54-D54)/D54, 0)</f>
         <v/>
       </c>
       <c r="G54" s="11" t="n">
-        <v>674.4400000000001</v>
+        <v>411.44</v>
       </c>
       <c r="H54" s="11" t="n">
-        <v>298.59</v>
+        <v>347.55</v>
       </c>
       <c r="I54" s="11" t="n">
-        <v>833.92</v>
+        <v>1310.72</v>
       </c>
       <c r="J54" s="11" t="n">
-        <v>1201.26</v>
+        <v>1086.04</v>
       </c>
       <c r="K54" s="23" t="n">
-        <v>180877</v>
+        <v>570362</v>
       </c>
       <c r="L54" s="23" t="n">
-        <v>2381</v>
+        <v>429991</v>
       </c>
     </row>
     <row r="55" ht="20" customHeight="1">
@@ -24511,32 +24511,32 @@
         </is>
       </c>
       <c r="D55" s="16" t="n">
-        <v>2515.07</v>
+        <v>3819.51</v>
       </c>
       <c r="E55" s="16" t="n">
-        <v>4075.42</v>
+        <v>4222.39</v>
       </c>
       <c r="F55" s="17">
         <f>IF(D55&gt;0, (E55-D55)/D55, 0)</f>
         <v/>
       </c>
       <c r="G55" s="16" t="n">
-        <v>542.66</v>
+        <v>472.45</v>
       </c>
       <c r="H55" s="16" t="n">
-        <v>339.03</v>
+        <v>353.99</v>
       </c>
       <c r="I55" s="16" t="n">
-        <v>923.6900000000001</v>
+        <v>1395.81</v>
       </c>
       <c r="J55" s="16" t="n">
-        <v>1301.62</v>
+        <v>1332.75</v>
       </c>
       <c r="K55" s="23" t="n">
-        <v>372072</v>
+        <v>384944</v>
       </c>
       <c r="L55" s="23" t="n">
-        <v>2293</v>
+        <v>597517</v>
       </c>
     </row>
     <row r="56" ht="20" customHeight="1">
@@ -24556,32 +24556,32 @@
         </is>
       </c>
       <c r="D56" s="11" t="n">
-        <v>1772.15</v>
+        <v>1673.33</v>
       </c>
       <c r="E56" s="11" t="n">
-        <v>1588.2</v>
-      </c>
-      <c r="F56" s="12">
+        <v>1746.64</v>
+      </c>
+      <c r="F56" s="17">
         <f>IF(D56&gt;0, (E56-D56)/D56, 0)</f>
         <v/>
       </c>
       <c r="G56" s="11" t="n">
-        <v>699.66</v>
+        <v>645.03</v>
       </c>
       <c r="H56" s="11" t="n">
-        <v>679.27</v>
+        <v>658.37</v>
       </c>
       <c r="I56" s="11" t="n">
-        <v>1745.81</v>
+        <v>1788.81</v>
       </c>
       <c r="J56" s="11" t="n">
-        <v>1717.38</v>
+        <v>1771.03</v>
       </c>
       <c r="K56" s="23" t="n">
-        <v>668997</v>
+        <v>757807</v>
       </c>
       <c r="L56" s="23" t="n">
-        <v>2787</v>
+        <v>733611</v>
       </c>
     </row>
     <row r="57" ht="20" customHeight="1">
@@ -24601,32 +24601,32 @@
         </is>
       </c>
       <c r="D57" s="16" t="n">
-        <v>1427.28</v>
+        <v>1683.77</v>
       </c>
       <c r="E57" s="16" t="n">
-        <v>1593.35</v>
+        <v>1721.7</v>
       </c>
       <c r="F57" s="17">
         <f>IF(D57&gt;0, (E57-D57)/D57, 0)</f>
         <v/>
       </c>
       <c r="G57" s="16" t="n">
-        <v>748.92</v>
+        <v>583.15</v>
       </c>
       <c r="H57" s="16" t="n">
-        <v>637.35</v>
+        <v>632.51</v>
       </c>
       <c r="I57" s="16" t="n">
-        <v>1800.43</v>
+        <v>1713.88</v>
       </c>
       <c r="J57" s="16" t="n">
-        <v>1742.55</v>
+        <v>1758.53</v>
       </c>
       <c r="K57" s="23" t="n">
-        <v>788107</v>
+        <v>752569</v>
       </c>
       <c r="L57" s="23" t="n">
-        <v>2843</v>
+        <v>744769</v>
       </c>
     </row>
     <row r="58" ht="20" customHeight="1">

</xml_diff>

<commit_message>
benchmarks: Python (opt.) get_with_index tier STRESS completed (20 runs DKR & BME)
</commit_message>
<xml_diff>
--- a/Programming_Benchmark_Report.xlsx
+++ b/Programming_Benchmark_Report.xlsx
@@ -24646,32 +24646,32 @@
         </is>
       </c>
       <c r="D58" s="11" t="n">
-        <v>2029.15</v>
+        <v>3561.39</v>
       </c>
       <c r="E58" s="11" t="n">
-        <v>3908.34</v>
+        <v>4117.97</v>
       </c>
       <c r="F58" s="17">
         <f>IF(D58&gt;0, (E58-D58)/D58, 0)</f>
         <v/>
       </c>
       <c r="G58" s="11" t="n">
-        <v>704.3</v>
+        <v>1178.2</v>
       </c>
       <c r="H58" s="11" t="n">
-        <v>233.79</v>
+        <v>1074.02</v>
       </c>
       <c r="I58" s="11" t="n">
-        <v>884.4</v>
+        <v>1962</v>
       </c>
       <c r="J58" s="11" t="n">
-        <v>1079.05</v>
+        <v>1477.21</v>
       </c>
       <c r="K58" s="23" t="n">
-        <v>852420</v>
+        <v>19687612</v>
       </c>
       <c r="L58" s="23" t="n">
-        <v>5003</v>
+        <v>18232247</v>
       </c>
     </row>
     <row r="59" ht="20" customHeight="1">
@@ -24691,32 +24691,32 @@
         </is>
       </c>
       <c r="D59" s="16" t="n">
-        <v>2252.1</v>
+        <v>3564.67</v>
       </c>
       <c r="E59" s="16" t="n">
-        <v>3597.59</v>
+        <v>3962.04</v>
       </c>
       <c r="F59" s="17">
         <f>IF(D59&gt;0, (E59-D59)/D59, 0)</f>
         <v/>
       </c>
       <c r="G59" s="16" t="n">
-        <v>539.9299999999999</v>
+        <v>205.92</v>
       </c>
       <c r="H59" s="16" t="n">
-        <v>259.18</v>
+        <v>245.95</v>
       </c>
       <c r="I59" s="16" t="n">
-        <v>739.1799999999999</v>
+        <v>1169.41</v>
       </c>
       <c r="J59" s="16" t="n">
-        <v>1283.08</v>
+        <v>1279.37</v>
       </c>
       <c r="K59" s="23" t="n">
-        <v>1618242</v>
+        <v>9198074</v>
       </c>
       <c r="L59" s="23" t="n">
-        <v>6547</v>
+        <v>10914743</v>
       </c>
     </row>
     <row r="60" ht="20" customHeight="1">
@@ -24736,32 +24736,32 @@
         </is>
       </c>
       <c r="D60" s="11" t="n">
-        <v>1739.5</v>
+        <v>1651.09</v>
       </c>
       <c r="E60" s="11" t="n">
-        <v>1109.4</v>
-      </c>
-      <c r="F60" s="12">
+        <v>1667.1</v>
+      </c>
+      <c r="F60" s="21">
         <f>IF(D60&gt;0, (E60-D60)/D60, 0)</f>
         <v/>
       </c>
       <c r="G60" s="11" t="n">
-        <v>435.79</v>
+        <v>171.61</v>
       </c>
       <c r="H60" s="11" t="n">
-        <v>411.09</v>
+        <v>156.04</v>
       </c>
       <c r="I60" s="11" t="n">
-        <v>670.3</v>
+        <v>579.59</v>
       </c>
       <c r="J60" s="11" t="n">
-        <v>1322.52</v>
+        <v>584.72</v>
       </c>
       <c r="K60" s="23" t="n">
-        <v>3497581</v>
+        <v>6366276</v>
       </c>
       <c r="L60" s="23" t="n">
-        <v>5445</v>
+        <v>6766645</v>
       </c>
     </row>
     <row r="61" ht="20" customHeight="1">
@@ -24781,32 +24781,32 @@
         </is>
       </c>
       <c r="D61" s="16" t="n">
-        <v>1433.16</v>
+        <v>1641.29</v>
       </c>
       <c r="E61" s="16" t="n">
-        <v>868.96</v>
-      </c>
-      <c r="F61" s="12">
+        <v>1643.54</v>
+      </c>
+      <c r="F61" s="22">
         <f>IF(D61&gt;0, (E61-D61)/D61, 0)</f>
         <v/>
       </c>
       <c r="G61" s="16" t="n">
-        <v>384.15</v>
+        <v>184.24</v>
       </c>
       <c r="H61" s="16" t="n">
-        <v>560.41</v>
+        <v>176.01</v>
       </c>
       <c r="I61" s="16" t="n">
-        <v>782</v>
+        <v>371.02</v>
       </c>
       <c r="J61" s="16" t="n">
-        <v>1583.21</v>
+        <v>651.54</v>
       </c>
       <c r="K61" s="23" t="n">
-        <v>4355905</v>
+        <v>5730393</v>
       </c>
       <c r="L61" s="23" t="n">
-        <v>1326</v>
+        <v>6235002</v>
       </c>
     </row>
     <row r="62"/>

</xml_diff>

<commit_message>
benchmarks: Python (opt.) get_no_index tier POC completed (20 runs DKR & BME)
</commit_message>
<xml_diff>
--- a/Programming_Benchmark_Report.xlsx
+++ b/Programming_Benchmark_Report.xlsx
@@ -22943,26 +22943,26 @@
         </is>
       </c>
       <c r="D6" s="11" t="n">
-        <v>2288.6</v>
+        <v>3228.25</v>
       </c>
       <c r="E6" s="11" t="n">
-        <v>1384.43</v>
+        <v>2814.82</v>
       </c>
       <c r="F6" s="12">
         <f>IF(D6&gt;0, (E6-D6)/D6, 0)</f>
         <v/>
       </c>
       <c r="G6" s="11" t="n">
-        <v>8.92</v>
+        <v>6.28</v>
       </c>
       <c r="H6" s="11" t="n">
-        <v>24.98</v>
+        <v>7.71</v>
       </c>
       <c r="I6" s="11" t="n">
-        <v>16.19</v>
+        <v>11.14</v>
       </c>
       <c r="J6" s="11" t="n">
-        <v>87.81999999999999</v>
+        <v>17.14</v>
       </c>
       <c r="K6" s="13" t="n">
         <v>0</v>
@@ -22988,26 +22988,26 @@
         </is>
       </c>
       <c r="D7" s="16" t="n">
-        <v>2583.93</v>
+        <v>2925.46</v>
       </c>
       <c r="E7" s="16" t="n">
-        <v>2423.24</v>
+        <v>2704.72</v>
       </c>
       <c r="F7" s="12">
         <f>IF(D7&gt;0, (E7-D7)/D7, 0)</f>
         <v/>
       </c>
       <c r="G7" s="16" t="n">
-        <v>7.78</v>
+        <v>6.96</v>
       </c>
       <c r="H7" s="16" t="n">
-        <v>8.32</v>
+        <v>7.64</v>
       </c>
       <c r="I7" s="16" t="n">
-        <v>12.31</v>
+        <v>11.6</v>
       </c>
       <c r="J7" s="16" t="n">
-        <v>14.55</v>
+        <v>13.91</v>
       </c>
       <c r="K7" s="18" t="n">
         <v>0</v>
@@ -23033,26 +23033,26 @@
         </is>
       </c>
       <c r="D8" s="11" t="n">
-        <v>308.21</v>
+        <v>311.47</v>
       </c>
       <c r="E8" s="11" t="n">
-        <v>317.22</v>
-      </c>
-      <c r="F8" s="17">
+        <v>309.51</v>
+      </c>
+      <c r="F8" s="21">
         <f>IF(D8&gt;0, (E8-D8)/D8, 0)</f>
         <v/>
       </c>
       <c r="G8" s="11" t="n">
-        <v>64.81</v>
+        <v>64.13</v>
       </c>
       <c r="H8" s="11" t="n">
-        <v>62.55</v>
+        <v>64.51000000000001</v>
       </c>
       <c r="I8" s="11" t="n">
-        <v>92.84</v>
+        <v>95.05</v>
       </c>
       <c r="J8" s="11" t="n">
-        <v>89.88</v>
+        <v>93.31999999999999</v>
       </c>
       <c r="K8" s="13" t="n">
         <v>0</v>
@@ -23078,26 +23078,26 @@
         </is>
       </c>
       <c r="D9" s="16" t="n">
-        <v>71.84999999999999</v>
+        <v>705.24</v>
       </c>
       <c r="E9" s="16" t="n">
-        <v>722.62</v>
+        <v>716.13</v>
       </c>
       <c r="F9" s="17">
         <f>IF(D9&gt;0, (E9-D9)/D9, 0)</f>
         <v/>
       </c>
       <c r="G9" s="16" t="n">
-        <v>276.98</v>
+        <v>28.35</v>
       </c>
       <c r="H9" s="16" t="n">
-        <v>27.6</v>
+        <v>27.93</v>
       </c>
       <c r="I9" s="16" t="n">
-        <v>394.91</v>
+        <v>42.67</v>
       </c>
       <c r="J9" s="16" t="n">
-        <v>41.13</v>
+        <v>42.91</v>
       </c>
       <c r="K9" s="18" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
benchmarks: Python (opt.) get_no_index tier SMALL completed (20 runs DKR & BME)
</commit_message>
<xml_diff>
--- a/Programming_Benchmark_Report.xlsx
+++ b/Programming_Benchmark_Report.xlsx
@@ -23123,26 +23123,26 @@
         </is>
       </c>
       <c r="D10" s="11" t="n">
-        <v>2442.05</v>
+        <v>4212.22</v>
       </c>
       <c r="E10" s="11" t="n">
-        <v>4651.84</v>
+        <v>4688.18</v>
       </c>
       <c r="F10" s="17">
         <f>IF(D10&gt;0, (E10-D10)/D10, 0)</f>
         <v/>
       </c>
       <c r="G10" s="11" t="n">
-        <v>41.1</v>
+        <v>24.51</v>
       </c>
       <c r="H10" s="11" t="n">
-        <v>23.18</v>
+        <v>22.49</v>
       </c>
       <c r="I10" s="11" t="n">
-        <v>64.19</v>
+        <v>49.94</v>
       </c>
       <c r="J10" s="11" t="n">
-        <v>59.82</v>
+        <v>51.49</v>
       </c>
       <c r="K10" s="13" t="n">
         <v>0</v>
@@ -23168,26 +23168,26 @@
         </is>
       </c>
       <c r="D11" s="16" t="n">
-        <v>2845.01</v>
+        <v>3943.07</v>
       </c>
       <c r="E11" s="16" t="n">
-        <v>4316.34</v>
+        <v>4380.43</v>
       </c>
       <c r="F11" s="17">
         <f>IF(D11&gt;0, (E11-D11)/D11, 0)</f>
         <v/>
       </c>
       <c r="G11" s="16" t="n">
-        <v>35.14</v>
+        <v>26.42</v>
       </c>
       <c r="H11" s="16" t="n">
-        <v>23.54</v>
+        <v>23.67</v>
       </c>
       <c r="I11" s="16" t="n">
-        <v>53.02</v>
+        <v>57.77</v>
       </c>
       <c r="J11" s="16" t="n">
-        <v>49.84</v>
+        <v>50.13</v>
       </c>
       <c r="K11" s="18" t="n">
         <v>0</v>
@@ -23213,26 +23213,26 @@
         </is>
       </c>
       <c r="D12" s="11" t="n">
-        <v>315.72</v>
+        <v>300.41</v>
       </c>
       <c r="E12" s="11" t="n">
-        <v>300.56</v>
-      </c>
-      <c r="F12" s="12">
+        <v>305.14</v>
+      </c>
+      <c r="F12" s="17">
         <f>IF(D12&gt;0, (E12-D12)/D12, 0)</f>
         <v/>
       </c>
       <c r="G12" s="11" t="n">
-        <v>315.65</v>
+        <v>331.72</v>
       </c>
       <c r="H12" s="11" t="n">
-        <v>319.87</v>
+        <v>326.78</v>
       </c>
       <c r="I12" s="11" t="n">
-        <v>498.56</v>
+        <v>571.1</v>
       </c>
       <c r="J12" s="11" t="n">
-        <v>481.04</v>
+        <v>505.14</v>
       </c>
       <c r="K12" s="13" t="n">
         <v>0</v>
@@ -23258,29 +23258,29 @@
         </is>
       </c>
       <c r="D13" s="16" t="n">
-        <v>72.88</v>
+        <v>662.1900000000001</v>
       </c>
       <c r="E13" s="16" t="n">
-        <v>678.83</v>
+        <v>686.16</v>
       </c>
       <c r="F13" s="17">
         <f>IF(D13&gt;0, (E13-D13)/D13, 0)</f>
         <v/>
       </c>
       <c r="G13" s="16" t="n">
-        <v>1350.84</v>
+        <v>152</v>
       </c>
       <c r="H13" s="16" t="n">
-        <v>144.45</v>
+        <v>146.11</v>
       </c>
       <c r="I13" s="16" t="n">
-        <v>1773.07</v>
+        <v>295.19</v>
       </c>
       <c r="J13" s="16" t="n">
-        <v>241.39</v>
-      </c>
-      <c r="K13" s="23" t="n">
-        <v>515</v>
+        <v>248.02</v>
+      </c>
+      <c r="K13" s="18" t="n">
+        <v>0</v>
       </c>
       <c r="L13" s="18" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
benchmarks: Python (opt.) get_no_index tier GENERAL completed (20 runs DKR & BME)
</commit_message>
<xml_diff>
--- a/Programming_Benchmark_Report.xlsx
+++ b/Programming_Benchmark_Report.xlsx
@@ -23303,32 +23303,32 @@
         </is>
       </c>
       <c r="D14" s="11" t="n">
-        <v>2263.24</v>
+        <v>4106.33</v>
       </c>
       <c r="E14" s="11" t="n">
-        <v>4598.21</v>
+        <v>4635.03</v>
       </c>
       <c r="F14" s="17">
         <f>IF(D14&gt;0, (E14-D14)/D14, 0)</f>
         <v/>
       </c>
       <c r="G14" s="11" t="n">
-        <v>223.68</v>
+        <v>123.46</v>
       </c>
       <c r="H14" s="11" t="n">
-        <v>119.96</v>
+        <v>118.54</v>
       </c>
       <c r="I14" s="11" t="n">
-        <v>427.8</v>
+        <v>224.75</v>
       </c>
       <c r="J14" s="11" t="n">
-        <v>276.55</v>
-      </c>
-      <c r="K14" s="13" t="n">
-        <v>0</v>
+        <v>255.81</v>
+      </c>
+      <c r="K14" s="23" t="n">
+        <v>12</v>
       </c>
       <c r="L14" s="23" t="n">
-        <v>2</v>
+        <v>244</v>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
@@ -23348,32 +23348,32 @@
         </is>
       </c>
       <c r="D15" s="16" t="n">
-        <v>2536.46</v>
+        <v>3913.44</v>
       </c>
       <c r="E15" s="16" t="n">
-        <v>4290.31</v>
+        <v>4323.16</v>
       </c>
       <c r="F15" s="17">
         <f>IF(D15&gt;0, (E15-D15)/D15, 0)</f>
         <v/>
       </c>
       <c r="G15" s="16" t="n">
-        <v>203.19</v>
+        <v>135.5</v>
       </c>
       <c r="H15" s="16" t="n">
-        <v>140.01</v>
+        <v>143.49</v>
       </c>
       <c r="I15" s="16" t="n">
-        <v>413.12</v>
+        <v>293.62</v>
       </c>
       <c r="J15" s="16" t="n">
-        <v>420.98</v>
-      </c>
-      <c r="K15" s="18" t="n">
-        <v>0</v>
+        <v>436.28</v>
+      </c>
+      <c r="K15" s="23" t="n">
+        <v>12</v>
       </c>
       <c r="L15" s="23" t="n">
-        <v>4</v>
+        <v>434</v>
       </c>
     </row>
     <row r="16" ht="20" customHeight="1">
@@ -23393,32 +23393,32 @@
         </is>
       </c>
       <c r="D16" s="11" t="n">
-        <v>312.48</v>
+        <v>296.84</v>
       </c>
       <c r="E16" s="11" t="n">
-        <v>268.06</v>
-      </c>
-      <c r="F16" s="12">
+        <v>299.99</v>
+      </c>
+      <c r="F16" s="17">
         <f>IF(D16&gt;0, (E16-D16)/D16, 0)</f>
         <v/>
       </c>
       <c r="G16" s="11" t="n">
-        <v>1318.84</v>
+        <v>1034.73</v>
       </c>
       <c r="H16" s="11" t="n">
-        <v>1122.48</v>
+        <v>1166.03</v>
       </c>
       <c r="I16" s="11" t="n">
-        <v>1915.67</v>
+        <v>1847.14</v>
       </c>
       <c r="J16" s="11" t="n">
-        <v>1877.45</v>
+        <v>1875.85</v>
       </c>
       <c r="K16" s="23" t="n">
-        <v>81206</v>
+        <v>104345</v>
       </c>
       <c r="L16" s="23" t="n">
-        <v>1001</v>
+        <v>101995</v>
       </c>
     </row>
     <row r="17" ht="20" customHeight="1">
@@ -23438,32 +23438,32 @@
         </is>
       </c>
       <c r="D17" s="16" t="n">
-        <v>66.38</v>
+        <v>651.41</v>
       </c>
       <c r="E17" s="16" t="n">
-        <v>646.46</v>
+        <v>668.4299999999999</v>
       </c>
       <c r="F17" s="17">
         <f>IF(D17&gt;0, (E17-D17)/D17, 0)</f>
         <v/>
       </c>
       <c r="G17" s="16" t="n">
-        <v>1208.08</v>
+        <v>728.72</v>
       </c>
       <c r="H17" s="16" t="n">
-        <v>667.42</v>
+        <v>710.97</v>
       </c>
       <c r="I17" s="16" t="n">
-        <v>1922.29</v>
+        <v>1446.62</v>
       </c>
       <c r="J17" s="16" t="n">
-        <v>1381.23</v>
+        <v>1391.47</v>
       </c>
       <c r="K17" s="23" t="n">
-        <v>78894</v>
+        <v>14646</v>
       </c>
       <c r="L17" s="23" t="n">
-        <v>115</v>
+        <v>14758</v>
       </c>
     </row>
     <row r="18" ht="20" customHeight="1">

</xml_diff>

<commit_message>
benchmarks: Python (opt.) get_no_index tier HIGH completed (20 runs DKR & BME)
</commit_message>
<xml_diff>
--- a/Programming_Benchmark_Report.xlsx
+++ b/Programming_Benchmark_Report.xlsx
@@ -23483,32 +23483,32 @@
         </is>
       </c>
       <c r="D18" s="11" t="n">
-        <v>2238.59</v>
+        <v>3962.61</v>
       </c>
       <c r="E18" s="11" t="n">
-        <v>4357.49</v>
+        <v>4498.12</v>
       </c>
       <c r="F18" s="17">
         <f>IF(D18&gt;0, (E18-D18)/D18, 0)</f>
         <v/>
       </c>
       <c r="G18" s="11" t="n">
-        <v>666.52</v>
+        <v>442.89</v>
       </c>
       <c r="H18" s="11" t="n">
-        <v>308.12</v>
+        <v>348.25</v>
       </c>
       <c r="I18" s="11" t="n">
-        <v>826.66</v>
+        <v>1370.61</v>
       </c>
       <c r="J18" s="11" t="n">
-        <v>1235.2</v>
+        <v>1073.61</v>
       </c>
       <c r="K18" s="23" t="n">
-        <v>180809</v>
+        <v>463033</v>
       </c>
       <c r="L18" s="23" t="n">
-        <v>2341</v>
+        <v>421600</v>
       </c>
     </row>
     <row r="19" ht="20" customHeight="1">
@@ -23528,32 +23528,32 @@
         </is>
       </c>
       <c r="D19" s="16" t="n">
-        <v>2556.75</v>
+        <v>3805.89</v>
       </c>
       <c r="E19" s="16" t="n">
-        <v>4047.56</v>
+        <v>4209.92</v>
       </c>
       <c r="F19" s="17">
         <f>IF(D19&gt;0, (E19-D19)/D19, 0)</f>
         <v/>
       </c>
       <c r="G19" s="16" t="n">
-        <v>536.61</v>
+        <v>473.23</v>
       </c>
       <c r="H19" s="16" t="n">
-        <v>336.12</v>
+        <v>356.09</v>
       </c>
       <c r="I19" s="16" t="n">
-        <v>932.01</v>
+        <v>1394.36</v>
       </c>
       <c r="J19" s="16" t="n">
-        <v>1289.28</v>
+        <v>1341.95</v>
       </c>
       <c r="K19" s="23" t="n">
-        <v>372570</v>
+        <v>380817</v>
       </c>
       <c r="L19" s="23" t="n">
-        <v>2191</v>
+        <v>601770</v>
       </c>
     </row>
     <row r="20" ht="20" customHeight="1">
@@ -23573,32 +23573,32 @@
         </is>
       </c>
       <c r="D20" s="11" t="n">
-        <v>301.12</v>
+        <v>291.63</v>
       </c>
       <c r="E20" s="11" t="n">
-        <v>108.65</v>
-      </c>
-      <c r="F20" s="12">
+        <v>294.94</v>
+      </c>
+      <c r="F20" s="17">
         <f>IF(D20&gt;0, (E20-D20)/D20, 0)</f>
         <v/>
       </c>
       <c r="G20" s="11" t="n">
-        <v>1239.21</v>
+        <v>796.85</v>
       </c>
       <c r="H20" s="11" t="n">
-        <v>865.89</v>
+        <v>717.38</v>
       </c>
       <c r="I20" s="11" t="n">
-        <v>1874.89</v>
+        <v>1557.62</v>
       </c>
       <c r="J20" s="11" t="n">
-        <v>1317.67</v>
+        <v>1311.04</v>
       </c>
       <c r="K20" s="23" t="n">
-        <v>619774</v>
+        <v>645669</v>
       </c>
       <c r="L20" s="23" t="n">
-        <v>1026</v>
+        <v>660679</v>
       </c>
     </row>
     <row r="21" ht="20" customHeight="1">
@@ -23618,32 +23618,32 @@
         </is>
       </c>
       <c r="D21" s="16" t="n">
-        <v>57.79</v>
+        <v>637.26</v>
       </c>
       <c r="E21" s="16" t="n">
-        <v>254.33</v>
+        <v>656.25</v>
       </c>
       <c r="F21" s="17">
         <f>IF(D21&gt;0, (E21-D21)/D21, 0)</f>
         <v/>
       </c>
       <c r="G21" s="16" t="n">
-        <v>944.62</v>
+        <v>872.92</v>
       </c>
       <c r="H21" s="16" t="n">
-        <v>911.3</v>
+        <v>915.4400000000001</v>
       </c>
       <c r="I21" s="16" t="n">
-        <v>1657.53</v>
+        <v>1908.6</v>
       </c>
       <c r="J21" s="16" t="n">
-        <v>1860.75</v>
+        <v>1935.11</v>
       </c>
       <c r="K21" s="23" t="n">
-        <v>138661</v>
+        <v>1045258</v>
       </c>
       <c r="L21" s="23" t="n">
-        <v>2451</v>
+        <v>1138679</v>
       </c>
     </row>
     <row r="22" ht="20" customHeight="1">

</xml_diff>

<commit_message>
benchmarks: Python (opt.) get_no_index tier STRESS completed (20 runs DKR & BME)
</commit_message>
<xml_diff>
--- a/Programming_Benchmark_Report.xlsx
+++ b/Programming_Benchmark_Report.xlsx
@@ -23663,32 +23663,32 @@
         </is>
       </c>
       <c r="D22" s="11" t="n">
-        <v>2043.66</v>
+        <v>3542.72</v>
       </c>
       <c r="E22" s="11" t="n">
-        <v>3837.87</v>
+        <v>4131.32</v>
       </c>
       <c r="F22" s="17">
         <f>IF(D22&gt;0, (E22-D22)/D22, 0)</f>
         <v/>
       </c>
       <c r="G22" s="11" t="n">
-        <v>697.37</v>
+        <v>1535.96</v>
       </c>
       <c r="H22" s="11" t="n">
-        <v>219.26</v>
+        <v>1332.5</v>
       </c>
       <c r="I22" s="11" t="n">
-        <v>877.52</v>
+        <v>1962.11</v>
       </c>
       <c r="J22" s="11" t="n">
-        <v>984.24</v>
+        <v>1713.01</v>
       </c>
       <c r="K22" s="23" t="n">
-        <v>871432</v>
+        <v>19808467</v>
       </c>
       <c r="L22" s="23" t="n">
-        <v>5336</v>
+        <v>17241200</v>
       </c>
     </row>
     <row r="23" ht="20" customHeight="1">
@@ -23708,32 +23708,32 @@
         </is>
       </c>
       <c r="D23" s="16" t="n">
-        <v>2273.36</v>
+        <v>3561.88</v>
       </c>
       <c r="E23" s="16" t="n">
-        <v>3560.28</v>
+        <v>3993.72</v>
       </c>
       <c r="F23" s="17">
         <f>IF(D23&gt;0, (E23-D23)/D23, 0)</f>
         <v/>
       </c>
       <c r="G23" s="16" t="n">
-        <v>539.49</v>
+        <v>210.02</v>
       </c>
       <c r="H23" s="16" t="n">
-        <v>259.31</v>
+        <v>234.02</v>
       </c>
       <c r="I23" s="16" t="n">
-        <v>735.16</v>
+        <v>1372.78</v>
       </c>
       <c r="J23" s="16" t="n">
-        <v>1332.79</v>
+        <v>1296.67</v>
       </c>
       <c r="K23" s="23" t="n">
-        <v>1611777</v>
+        <v>9118692</v>
       </c>
       <c r="L23" s="23" t="n">
-        <v>5846</v>
+        <v>7940192</v>
       </c>
     </row>
     <row r="24" ht="20" customHeight="1">
@@ -23753,32 +23753,32 @@
         </is>
       </c>
       <c r="D24" s="11" t="n">
-        <v>275.29</v>
+        <v>274.5</v>
       </c>
       <c r="E24" s="11" t="n">
-        <v>117.14</v>
-      </c>
-      <c r="F24" s="12">
+        <v>275.36</v>
+      </c>
+      <c r="F24" s="21">
         <f>IF(D24&gt;0, (E24-D24)/D24, 0)</f>
         <v/>
       </c>
       <c r="G24" s="11" t="n">
-        <v>1247.32</v>
+        <v>671.6900000000001</v>
       </c>
       <c r="H24" s="11" t="n">
-        <v>968.28</v>
+        <v>662.23</v>
       </c>
       <c r="I24" s="11" t="n">
-        <v>1880.77</v>
+        <v>1106.35</v>
       </c>
       <c r="J24" s="11" t="n">
-        <v>1607.21</v>
+        <v>942.5</v>
       </c>
       <c r="K24" s="23" t="n">
-        <v>1430364</v>
+        <v>1540211</v>
       </c>
       <c r="L24" s="23" t="n">
-        <v>842</v>
+        <v>1547893</v>
       </c>
     </row>
     <row r="25" ht="20" customHeight="1">
@@ -23798,32 +23798,32 @@
         </is>
       </c>
       <c r="D25" s="16" t="n">
-        <v>40.45</v>
+        <v>616.79</v>
       </c>
       <c r="E25" s="16" t="n">
-        <v>61.09</v>
+        <v>632.65</v>
       </c>
       <c r="F25" s="17">
         <f>IF(D25&gt;0, (E25-D25)/D25, 0)</f>
         <v/>
       </c>
       <c r="G25" s="16" t="n">
-        <v>744.15</v>
+        <v>314.6</v>
       </c>
       <c r="H25" s="16" t="n">
-        <v>634.0700000000001</v>
+        <v>303.65</v>
       </c>
       <c r="I25" s="16" t="n">
-        <v>1701.78</v>
+        <v>580.1</v>
       </c>
       <c r="J25" s="16" t="n">
-        <v>1201.3</v>
+        <v>532.5599999999999</v>
       </c>
       <c r="K25" s="23" t="n">
-        <v>243356</v>
-      </c>
-      <c r="L25" s="18" t="n">
-        <v>0</v>
+        <v>3079136</v>
+      </c>
+      <c r="L25" s="23" t="n">
+        <v>3231051</v>
       </c>
     </row>
     <row r="26"/>

</xml_diff>

<commit_message>
benchmarks: Python (opt.) get_with_index tier POC completed (20 runs DKR)
</commit_message>
<xml_diff>
--- a/Programming_Benchmark_Report.xlsx
+++ b/Programming_Benchmark_Report.xlsx
@@ -23926,7 +23926,7 @@
         </is>
       </c>
       <c r="D42" s="11" t="n">
-        <v>3202.93</v>
+        <v>3220.85</v>
       </c>
       <c r="E42" s="11" t="n">
         <v>2913.31</v>
@@ -23936,13 +23936,13 @@
         <v/>
       </c>
       <c r="G42" s="11" t="n">
-        <v>6.4</v>
+        <v>6.35</v>
       </c>
       <c r="H42" s="11" t="n">
         <v>7.31</v>
       </c>
       <c r="I42" s="11" t="n">
-        <v>11.54</v>
+        <v>11.52</v>
       </c>
       <c r="J42" s="11" t="n">
         <v>14.43</v>
@@ -23971,7 +23971,7 @@
         </is>
       </c>
       <c r="D43" s="16" t="n">
-        <v>3075.25</v>
+        <v>2951.16</v>
       </c>
       <c r="E43" s="16" t="n">
         <v>2825.46</v>
@@ -23981,13 +23981,13 @@
         <v/>
       </c>
       <c r="G43" s="16" t="n">
-        <v>6.58</v>
+        <v>6.86</v>
       </c>
       <c r="H43" s="16" t="n">
         <v>7.3</v>
       </c>
       <c r="I43" s="16" t="n">
-        <v>10.99</v>
+        <v>11.28</v>
       </c>
       <c r="J43" s="16" t="n">
         <v>14.39</v>
@@ -24016,7 +24016,7 @@
         </is>
       </c>
       <c r="D44" s="11" t="n">
-        <v>1762.95</v>
+        <v>1754.3</v>
       </c>
       <c r="E44" s="11" t="n">
         <v>1705.34</v>
@@ -24026,13 +24026,13 @@
         <v/>
       </c>
       <c r="G44" s="11" t="n">
-        <v>11.4</v>
+        <v>11.46</v>
       </c>
       <c r="H44" s="11" t="n">
         <v>12.01</v>
       </c>
       <c r="I44" s="11" t="n">
-        <v>18.79</v>
+        <v>18.85</v>
       </c>
       <c r="J44" s="11" t="n">
         <v>21.81</v>
@@ -24061,7 +24061,7 @@
         </is>
       </c>
       <c r="D45" s="16" t="n">
-        <v>1697.24</v>
+        <v>1691.82</v>
       </c>
       <c r="E45" s="16" t="n">
         <v>1606.63</v>
@@ -24071,13 +24071,13 @@
         <v/>
       </c>
       <c r="G45" s="16" t="n">
-        <v>11.86</v>
+        <v>11.88</v>
       </c>
       <c r="H45" s="16" t="n">
         <v>12.74</v>
       </c>
       <c r="I45" s="16" t="n">
-        <v>19.65</v>
+        <v>19.44</v>
       </c>
       <c r="J45" s="16" t="n">
         <v>23.01</v>

</xml_diff>

<commit_message>
benchmarks: Python (opt.) get_with_index tier SMALL completed (20 runs DKR)
</commit_message>
<xml_diff>
--- a/Programming_Benchmark_Report.xlsx
+++ b/Programming_Benchmark_Report.xlsx
@@ -24106,7 +24106,7 @@
         </is>
       </c>
       <c r="D46" s="11" t="n">
-        <v>4225.05</v>
+        <v>4131.64</v>
       </c>
       <c r="E46" s="11" t="n">
         <v>4754.7</v>
@@ -24116,13 +24116,13 @@
         <v/>
       </c>
       <c r="G46" s="11" t="n">
-        <v>24.48</v>
+        <v>25.14</v>
       </c>
       <c r="H46" s="11" t="n">
         <v>22.34</v>
       </c>
       <c r="I46" s="11" t="n">
-        <v>50.69</v>
+        <v>52.49</v>
       </c>
       <c r="J46" s="11" t="n">
         <v>53.03</v>
@@ -24151,7 +24151,7 @@
         </is>
       </c>
       <c r="D47" s="16" t="n">
-        <v>3954.94</v>
+        <v>3831.79</v>
       </c>
       <c r="E47" s="16" t="n">
         <v>4381.76</v>
@@ -24161,13 +24161,13 @@
         <v/>
       </c>
       <c r="G47" s="16" t="n">
-        <v>26.11</v>
+        <v>27.1</v>
       </c>
       <c r="H47" s="16" t="n">
         <v>23.91</v>
       </c>
       <c r="I47" s="16" t="n">
-        <v>54.48</v>
+        <v>57.98</v>
       </c>
       <c r="J47" s="16" t="n">
         <v>52.62</v>
@@ -24196,7 +24196,7 @@
         </is>
       </c>
       <c r="D48" s="11" t="n">
-        <v>1759.79</v>
+        <v>1774.47</v>
       </c>
       <c r="E48" s="11" t="n">
         <v>1793.58</v>
@@ -24206,13 +24206,13 @@
         <v/>
       </c>
       <c r="G48" s="11" t="n">
-        <v>60.14</v>
+        <v>58.92</v>
       </c>
       <c r="H48" s="11" t="n">
         <v>59.2</v>
       </c>
       <c r="I48" s="11" t="n">
-        <v>137.34</v>
+        <v>129.24</v>
       </c>
       <c r="J48" s="11" t="n">
         <v>136.26</v>
@@ -24241,23 +24241,23 @@
         </is>
       </c>
       <c r="D49" s="16" t="n">
-        <v>1753.26</v>
+        <v>1806.93</v>
       </c>
       <c r="E49" s="16" t="n">
         <v>1783.16</v>
       </c>
-      <c r="F49" s="17">
+      <c r="F49" s="12">
         <f>IF(D49&gt;0, (E49-D49)/D49, 0)</f>
         <v/>
       </c>
       <c r="G49" s="16" t="n">
-        <v>59.17</v>
+        <v>57.08</v>
       </c>
       <c r="H49" s="16" t="n">
         <v>58.59</v>
       </c>
       <c r="I49" s="16" t="n">
-        <v>126.35</v>
+        <v>119.53</v>
       </c>
       <c r="J49" s="16" t="n">
         <v>128.3</v>

</xml_diff>

<commit_message>
benchmarks: Python (opt.) get_with_index tier GENERAL completed (20 runs DKR)
</commit_message>
<xml_diff>
--- a/Programming_Benchmark_Report.xlsx
+++ b/Programming_Benchmark_Report.xlsx
@@ -24286,7 +24286,7 @@
         </is>
       </c>
       <c r="D50" s="11" t="n">
-        <v>4100.48</v>
+        <v>4041.54</v>
       </c>
       <c r="E50" s="11" t="n">
         <v>4646.94</v>
@@ -24296,19 +24296,19 @@
         <v/>
       </c>
       <c r="G50" s="11" t="n">
-        <v>123.88</v>
+        <v>127.27</v>
       </c>
       <c r="H50" s="11" t="n">
         <v>118.14</v>
       </c>
       <c r="I50" s="11" t="n">
-        <v>225.88</v>
+        <v>235.07</v>
       </c>
       <c r="J50" s="11" t="n">
         <v>263.55</v>
       </c>
       <c r="K50" s="23" t="n">
-        <v>6</v>
+        <v>149</v>
       </c>
       <c r="L50" s="23" t="n">
         <v>205</v>
@@ -24331,7 +24331,7 @@
         </is>
       </c>
       <c r="D51" s="16" t="n">
-        <v>3897.57</v>
+        <v>3804.68</v>
       </c>
       <c r="E51" s="16" t="n">
         <v>4319.43</v>
@@ -24341,19 +24341,19 @@
         <v/>
       </c>
       <c r="G51" s="16" t="n">
-        <v>134.41</v>
+        <v>137.41</v>
       </c>
       <c r="H51" s="16" t="n">
         <v>142.45</v>
       </c>
       <c r="I51" s="16" t="n">
-        <v>284.87</v>
+        <v>287.67</v>
       </c>
       <c r="J51" s="16" t="n">
         <v>424.99</v>
       </c>
       <c r="K51" s="23" t="n">
-        <v>3</v>
+        <v>13</v>
       </c>
       <c r="L51" s="23" t="n">
         <v>255</v>
@@ -24376,29 +24376,29 @@
         </is>
       </c>
       <c r="D52" s="11" t="n">
-        <v>1657.1</v>
+        <v>1686.4</v>
       </c>
       <c r="E52" s="11" t="n">
         <v>1700.94</v>
       </c>
-      <c r="F52" s="17">
+      <c r="F52" s="21">
         <f>IF(D52&gt;0, (E52-D52)/D52, 0)</f>
         <v/>
       </c>
       <c r="G52" s="11" t="n">
-        <v>328.9</v>
+        <v>322.16</v>
       </c>
       <c r="H52" s="11" t="n">
         <v>321.89</v>
       </c>
       <c r="I52" s="11" t="n">
-        <v>850.4</v>
+        <v>820.8200000000001</v>
       </c>
       <c r="J52" s="11" t="n">
         <v>828.98</v>
       </c>
       <c r="K52" s="23" t="n">
-        <v>3020</v>
+        <v>2170</v>
       </c>
       <c r="L52" s="23" t="n">
         <v>1437</v>
@@ -24421,29 +24421,29 @@
         </is>
       </c>
       <c r="D53" s="16" t="n">
-        <v>1634.28</v>
+        <v>1687.39</v>
       </c>
       <c r="E53" s="16" t="n">
         <v>1681.42</v>
       </c>
-      <c r="F53" s="17">
+      <c r="F53" s="22">
         <f>IF(D53&gt;0, (E53-D53)/D53, 0)</f>
         <v/>
       </c>
       <c r="G53" s="16" t="n">
-        <v>333.3</v>
+        <v>323.35</v>
       </c>
       <c r="H53" s="16" t="n">
         <v>325.69</v>
       </c>
       <c r="I53" s="16" t="n">
-        <v>868.42</v>
+        <v>843.9299999999999</v>
       </c>
       <c r="J53" s="16" t="n">
         <v>845.6</v>
       </c>
       <c r="K53" s="23" t="n">
-        <v>3775</v>
+        <v>4006</v>
       </c>
       <c r="L53" s="23" t="n">
         <v>2214</v>

</xml_diff>

<commit_message>
benchmarks: Python (opt.) get_with_index tier HIGH completed (20 runs DKR)
</commit_message>
<xml_diff>
--- a/Programming_Benchmark_Report.xlsx
+++ b/Programming_Benchmark_Report.xlsx
@@ -24466,7 +24466,7 @@
         </is>
       </c>
       <c r="D54" s="11" t="n">
-        <v>3963.58</v>
+        <v>3912.72</v>
       </c>
       <c r="E54" s="11" t="n">
         <v>4508.28</v>
@@ -24476,19 +24476,19 @@
         <v/>
       </c>
       <c r="G54" s="11" t="n">
-        <v>411.44</v>
+        <v>393.54</v>
       </c>
       <c r="H54" s="11" t="n">
         <v>347.55</v>
       </c>
       <c r="I54" s="11" t="n">
-        <v>1310.72</v>
+        <v>1256.94</v>
       </c>
       <c r="J54" s="11" t="n">
         <v>1086.04</v>
       </c>
       <c r="K54" s="23" t="n">
-        <v>570362</v>
+        <v>489562</v>
       </c>
       <c r="L54" s="23" t="n">
         <v>429991</v>
@@ -24511,7 +24511,7 @@
         </is>
       </c>
       <c r="D55" s="16" t="n">
-        <v>3819.51</v>
+        <v>3708.12</v>
       </c>
       <c r="E55" s="16" t="n">
         <v>4222.39</v>
@@ -24521,19 +24521,19 @@
         <v/>
       </c>
       <c r="G55" s="16" t="n">
-        <v>472.45</v>
+        <v>475.31</v>
       </c>
       <c r="H55" s="16" t="n">
         <v>353.99</v>
       </c>
       <c r="I55" s="16" t="n">
-        <v>1395.81</v>
+        <v>1399.13</v>
       </c>
       <c r="J55" s="16" t="n">
         <v>1332.75</v>
       </c>
       <c r="K55" s="23" t="n">
-        <v>384944</v>
+        <v>404354</v>
       </c>
       <c r="L55" s="23" t="n">
         <v>597517</v>
@@ -24556,7 +24556,7 @@
         </is>
       </c>
       <c r="D56" s="11" t="n">
-        <v>1673.33</v>
+        <v>1680.61</v>
       </c>
       <c r="E56" s="11" t="n">
         <v>1746.64</v>
@@ -24566,19 +24566,19 @@
         <v/>
       </c>
       <c r="G56" s="11" t="n">
-        <v>645.03</v>
+        <v>641.96</v>
       </c>
       <c r="H56" s="11" t="n">
         <v>658.37</v>
       </c>
       <c r="I56" s="11" t="n">
-        <v>1788.81</v>
+        <v>1744.5</v>
       </c>
       <c r="J56" s="11" t="n">
         <v>1771.03</v>
       </c>
       <c r="K56" s="23" t="n">
-        <v>757807</v>
+        <v>776802</v>
       </c>
       <c r="L56" s="23" t="n">
         <v>733611</v>
@@ -24601,7 +24601,7 @@
         </is>
       </c>
       <c r="D57" s="16" t="n">
-        <v>1683.77</v>
+        <v>1697.24</v>
       </c>
       <c r="E57" s="16" t="n">
         <v>1721.7</v>
@@ -24611,19 +24611,19 @@
         <v/>
       </c>
       <c r="G57" s="16" t="n">
-        <v>583.15</v>
+        <v>580.22</v>
       </c>
       <c r="H57" s="16" t="n">
         <v>632.51</v>
       </c>
       <c r="I57" s="16" t="n">
-        <v>1713.88</v>
+        <v>1712.41</v>
       </c>
       <c r="J57" s="16" t="n">
         <v>1758.53</v>
       </c>
       <c r="K57" s="23" t="n">
-        <v>752569</v>
+        <v>768510</v>
       </c>
       <c r="L57" s="23" t="n">
         <v>744769</v>

</xml_diff>

<commit_message>
benchmarks: Python (opt.) get_with_index tier STRESS completed (20 runs DKR)
</commit_message>
<xml_diff>
--- a/Programming_Benchmark_Report.xlsx
+++ b/Programming_Benchmark_Report.xlsx
@@ -24646,7 +24646,7 @@
         </is>
       </c>
       <c r="D58" s="11" t="n">
-        <v>3561.39</v>
+        <v>3515.26</v>
       </c>
       <c r="E58" s="11" t="n">
         <v>4117.97</v>
@@ -24656,19 +24656,19 @@
         <v/>
       </c>
       <c r="G58" s="11" t="n">
-        <v>1178.2</v>
+        <v>1892.94</v>
       </c>
       <c r="H58" s="11" t="n">
         <v>1074.02</v>
       </c>
       <c r="I58" s="11" t="n">
-        <v>1962</v>
+        <v>1992.83</v>
       </c>
       <c r="J58" s="11" t="n">
         <v>1477.21</v>
       </c>
       <c r="K58" s="23" t="n">
-        <v>19687612</v>
+        <v>20247546</v>
       </c>
       <c r="L58" s="23" t="n">
         <v>18232247</v>
@@ -24691,7 +24691,7 @@
         </is>
       </c>
       <c r="D59" s="16" t="n">
-        <v>3564.67</v>
+        <v>3507.57</v>
       </c>
       <c r="E59" s="16" t="n">
         <v>3962.04</v>
@@ -24701,19 +24701,19 @@
         <v/>
       </c>
       <c r="G59" s="16" t="n">
-        <v>205.92</v>
+        <v>197.43</v>
       </c>
       <c r="H59" s="16" t="n">
         <v>245.95</v>
       </c>
       <c r="I59" s="16" t="n">
-        <v>1169.41</v>
+        <v>792.6900000000001</v>
       </c>
       <c r="J59" s="16" t="n">
         <v>1279.37</v>
       </c>
       <c r="K59" s="23" t="n">
-        <v>9198074</v>
+        <v>9114768</v>
       </c>
       <c r="L59" s="23" t="n">
         <v>10914743</v>
@@ -24736,7 +24736,7 @@
         </is>
       </c>
       <c r="D60" s="11" t="n">
-        <v>1651.09</v>
+        <v>1676.31</v>
       </c>
       <c r="E60" s="11" t="n">
         <v>1667.1</v>
@@ -24746,19 +24746,19 @@
         <v/>
       </c>
       <c r="G60" s="11" t="n">
-        <v>171.61</v>
+        <v>173.42</v>
       </c>
       <c r="H60" s="11" t="n">
         <v>156.04</v>
       </c>
       <c r="I60" s="11" t="n">
-        <v>579.59</v>
+        <v>555.12</v>
       </c>
       <c r="J60" s="11" t="n">
         <v>584.72</v>
       </c>
       <c r="K60" s="23" t="n">
-        <v>6366276</v>
+        <v>6463441</v>
       </c>
       <c r="L60" s="23" t="n">
         <v>6766645</v>
@@ -24781,29 +24781,29 @@
         </is>
       </c>
       <c r="D61" s="16" t="n">
-        <v>1641.29</v>
+        <v>1677.93</v>
       </c>
       <c r="E61" s="16" t="n">
         <v>1643.54</v>
       </c>
-      <c r="F61" s="22">
+      <c r="F61" s="12">
         <f>IF(D61&gt;0, (E61-D61)/D61, 0)</f>
         <v/>
       </c>
       <c r="G61" s="16" t="n">
-        <v>184.24</v>
+        <v>188</v>
       </c>
       <c r="H61" s="16" t="n">
         <v>176.01</v>
       </c>
       <c r="I61" s="16" t="n">
-        <v>371.02</v>
+        <v>343.55</v>
       </c>
       <c r="J61" s="16" t="n">
         <v>651.54</v>
       </c>
       <c r="K61" s="23" t="n">
-        <v>5730393</v>
+        <v>5778982</v>
       </c>
       <c r="L61" s="23" t="n">
         <v>6235002</v>

</xml_diff>

<commit_message>
benchmarks: Python (opt.) get_no_index tier POC completed (20 runs DKR)
</commit_message>
<xml_diff>
--- a/Programming_Benchmark_Report.xlsx
+++ b/Programming_Benchmark_Report.xlsx
@@ -22943,7 +22943,7 @@
         </is>
       </c>
       <c r="D6" s="11" t="n">
-        <v>3228.25</v>
+        <v>3216.02</v>
       </c>
       <c r="E6" s="11" t="n">
         <v>2814.82</v>
@@ -22953,13 +22953,13 @@
         <v/>
       </c>
       <c r="G6" s="11" t="n">
-        <v>6.28</v>
+        <v>6.33</v>
       </c>
       <c r="H6" s="11" t="n">
         <v>7.71</v>
       </c>
       <c r="I6" s="11" t="n">
-        <v>11.14</v>
+        <v>11.25</v>
       </c>
       <c r="J6" s="11" t="n">
         <v>17.14</v>
@@ -22988,7 +22988,7 @@
         </is>
       </c>
       <c r="D7" s="16" t="n">
-        <v>2925.46</v>
+        <v>2867.09</v>
       </c>
       <c r="E7" s="16" t="n">
         <v>2704.72</v>
@@ -22998,13 +22998,13 @@
         <v/>
       </c>
       <c r="G7" s="16" t="n">
-        <v>6.96</v>
+        <v>7.08</v>
       </c>
       <c r="H7" s="16" t="n">
         <v>7.64</v>
       </c>
       <c r="I7" s="16" t="n">
-        <v>11.6</v>
+        <v>11.94</v>
       </c>
       <c r="J7" s="16" t="n">
         <v>13.91</v>
@@ -23033,23 +23033,23 @@
         </is>
       </c>
       <c r="D8" s="11" t="n">
-        <v>311.47</v>
+        <v>300.57</v>
       </c>
       <c r="E8" s="11" t="n">
         <v>309.51</v>
       </c>
-      <c r="F8" s="21">
+      <c r="F8" s="17">
         <f>IF(D8&gt;0, (E8-D8)/D8, 0)</f>
         <v/>
       </c>
       <c r="G8" s="11" t="n">
-        <v>64.13</v>
+        <v>66.45</v>
       </c>
       <c r="H8" s="11" t="n">
         <v>64.51000000000001</v>
       </c>
       <c r="I8" s="11" t="n">
-        <v>95.05</v>
+        <v>98.18000000000001</v>
       </c>
       <c r="J8" s="11" t="n">
         <v>93.31999999999999</v>
@@ -23078,7 +23078,7 @@
         </is>
       </c>
       <c r="D9" s="16" t="n">
-        <v>705.24</v>
+        <v>701.38</v>
       </c>
       <c r="E9" s="16" t="n">
         <v>716.13</v>
@@ -23088,13 +23088,13 @@
         <v/>
       </c>
       <c r="G9" s="16" t="n">
-        <v>28.35</v>
+        <v>28.51</v>
       </c>
       <c r="H9" s="16" t="n">
         <v>27.93</v>
       </c>
       <c r="I9" s="16" t="n">
-        <v>42.67</v>
+        <v>42.92</v>
       </c>
       <c r="J9" s="16" t="n">
         <v>42.91</v>

</xml_diff>

<commit_message>
benchmarks: Python (opt.) get_no_index tier SMALL completed (20 runs DKR)
</commit_message>
<xml_diff>
--- a/Programming_Benchmark_Report.xlsx
+++ b/Programming_Benchmark_Report.xlsx
@@ -23123,7 +23123,7 @@
         </is>
       </c>
       <c r="D10" s="11" t="n">
-        <v>4212.22</v>
+        <v>4120.04</v>
       </c>
       <c r="E10" s="11" t="n">
         <v>4688.18</v>
@@ -23133,13 +23133,13 @@
         <v/>
       </c>
       <c r="G10" s="11" t="n">
-        <v>24.51</v>
+        <v>25.34</v>
       </c>
       <c r="H10" s="11" t="n">
         <v>22.49</v>
       </c>
       <c r="I10" s="11" t="n">
-        <v>49.94</v>
+        <v>53.53</v>
       </c>
       <c r="J10" s="11" t="n">
         <v>51.49</v>
@@ -23168,7 +23168,7 @@
         </is>
       </c>
       <c r="D11" s="16" t="n">
-        <v>3943.07</v>
+        <v>3820.01</v>
       </c>
       <c r="E11" s="16" t="n">
         <v>4380.43</v>
@@ -23178,13 +23178,13 @@
         <v/>
       </c>
       <c r="G11" s="16" t="n">
-        <v>26.42</v>
+        <v>27.16</v>
       </c>
       <c r="H11" s="16" t="n">
         <v>23.67</v>
       </c>
       <c r="I11" s="16" t="n">
-        <v>57.77</v>
+        <v>58.09</v>
       </c>
       <c r="J11" s="16" t="n">
         <v>50.13</v>
@@ -23213,7 +23213,7 @@
         </is>
       </c>
       <c r="D12" s="11" t="n">
-        <v>300.41</v>
+        <v>296</v>
       </c>
       <c r="E12" s="11" t="n">
         <v>305.14</v>
@@ -23223,13 +23223,13 @@
         <v/>
       </c>
       <c r="G12" s="11" t="n">
-        <v>331.72</v>
+        <v>336.84</v>
       </c>
       <c r="H12" s="11" t="n">
         <v>326.78</v>
       </c>
       <c r="I12" s="11" t="n">
-        <v>571.1</v>
+        <v>584.01</v>
       </c>
       <c r="J12" s="11" t="n">
         <v>505.14</v>
@@ -23258,7 +23258,7 @@
         </is>
       </c>
       <c r="D13" s="16" t="n">
-        <v>662.1900000000001</v>
+        <v>663.11</v>
       </c>
       <c r="E13" s="16" t="n">
         <v>686.16</v>
@@ -23268,13 +23268,13 @@
         <v/>
       </c>
       <c r="G13" s="16" t="n">
-        <v>152</v>
+        <v>151.77</v>
       </c>
       <c r="H13" s="16" t="n">
         <v>146.11</v>
       </c>
       <c r="I13" s="16" t="n">
-        <v>295.19</v>
+        <v>294.22</v>
       </c>
       <c r="J13" s="16" t="n">
         <v>248.02</v>

</xml_diff>

<commit_message>
benchmarks: Python (opt.) get_no_index tier GENERAL completed (20 runs DKR)
</commit_message>
<xml_diff>
--- a/Programming_Benchmark_Report.xlsx
+++ b/Programming_Benchmark_Report.xlsx
@@ -23303,7 +23303,7 @@
         </is>
       </c>
       <c r="D14" s="11" t="n">
-        <v>4106.33</v>
+        <v>4018.1</v>
       </c>
       <c r="E14" s="11" t="n">
         <v>4635.03</v>
@@ -23313,19 +23313,19 @@
         <v/>
       </c>
       <c r="G14" s="11" t="n">
-        <v>123.46</v>
+        <v>125.65</v>
       </c>
       <c r="H14" s="11" t="n">
         <v>118.54</v>
       </c>
       <c r="I14" s="11" t="n">
-        <v>224.75</v>
+        <v>226.89</v>
       </c>
       <c r="J14" s="11" t="n">
         <v>255.81</v>
       </c>
       <c r="K14" s="23" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="L14" s="23" t="n">
         <v>244</v>
@@ -23348,7 +23348,7 @@
         </is>
       </c>
       <c r="D15" s="16" t="n">
-        <v>3913.44</v>
+        <v>3797.28</v>
       </c>
       <c r="E15" s="16" t="n">
         <v>4323.16</v>
@@ -23358,19 +23358,19 @@
         <v/>
       </c>
       <c r="G15" s="16" t="n">
-        <v>135.5</v>
+        <v>139.35</v>
       </c>
       <c r="H15" s="16" t="n">
         <v>143.49</v>
       </c>
       <c r="I15" s="16" t="n">
-        <v>293.62</v>
+        <v>301.83</v>
       </c>
       <c r="J15" s="16" t="n">
         <v>436.28</v>
       </c>
       <c r="K15" s="23" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="L15" s="23" t="n">
         <v>434</v>
@@ -23393,7 +23393,7 @@
         </is>
       </c>
       <c r="D16" s="11" t="n">
-        <v>296.84</v>
+        <v>292.21</v>
       </c>
       <c r="E16" s="11" t="n">
         <v>299.99</v>
@@ -23403,19 +23403,19 @@
         <v/>
       </c>
       <c r="G16" s="11" t="n">
-        <v>1034.73</v>
+        <v>1069.6</v>
       </c>
       <c r="H16" s="11" t="n">
         <v>1166.03</v>
       </c>
       <c r="I16" s="11" t="n">
-        <v>1847.14</v>
+        <v>1846.86</v>
       </c>
       <c r="J16" s="11" t="n">
         <v>1875.85</v>
       </c>
       <c r="K16" s="23" t="n">
-        <v>104345</v>
+        <v>108957</v>
       </c>
       <c r="L16" s="23" t="n">
         <v>101995</v>
@@ -23438,7 +23438,7 @@
         </is>
       </c>
       <c r="D17" s="16" t="n">
-        <v>651.41</v>
+        <v>649.09</v>
       </c>
       <c r="E17" s="16" t="n">
         <v>668.4299999999999</v>
@@ -23448,19 +23448,19 @@
         <v/>
       </c>
       <c r="G17" s="16" t="n">
-        <v>728.72</v>
+        <v>724.9299999999999</v>
       </c>
       <c r="H17" s="16" t="n">
         <v>710.97</v>
       </c>
       <c r="I17" s="16" t="n">
-        <v>1446.62</v>
+        <v>1461.32</v>
       </c>
       <c r="J17" s="16" t="n">
         <v>1391.47</v>
       </c>
       <c r="K17" s="23" t="n">
-        <v>14646</v>
+        <v>17126</v>
       </c>
       <c r="L17" s="23" t="n">
         <v>14758</v>

</xml_diff>

<commit_message>
benchmarks: Python (opt.) get_no_index tier HIGH completed (20 runs DKR)
</commit_message>
<xml_diff>
--- a/Programming_Benchmark_Report.xlsx
+++ b/Programming_Benchmark_Report.xlsx
@@ -23483,7 +23483,7 @@
         </is>
       </c>
       <c r="D18" s="11" t="n">
-        <v>3962.61</v>
+        <v>3907.05</v>
       </c>
       <c r="E18" s="11" t="n">
         <v>4498.12</v>
@@ -23493,19 +23493,19 @@
         <v/>
       </c>
       <c r="G18" s="11" t="n">
-        <v>442.89</v>
+        <v>413.46</v>
       </c>
       <c r="H18" s="11" t="n">
         <v>348.25</v>
       </c>
       <c r="I18" s="11" t="n">
-        <v>1370.61</v>
+        <v>1266.57</v>
       </c>
       <c r="J18" s="11" t="n">
         <v>1073.61</v>
       </c>
       <c r="K18" s="23" t="n">
-        <v>463033</v>
+        <v>443375</v>
       </c>
       <c r="L18" s="23" t="n">
         <v>421600</v>
@@ -23528,7 +23528,7 @@
         </is>
       </c>
       <c r="D19" s="16" t="n">
-        <v>3805.89</v>
+        <v>3712.62</v>
       </c>
       <c r="E19" s="16" t="n">
         <v>4209.92</v>
@@ -23538,19 +23538,19 @@
         <v/>
       </c>
       <c r="G19" s="16" t="n">
-        <v>473.23</v>
+        <v>476.89</v>
       </c>
       <c r="H19" s="16" t="n">
         <v>356.09</v>
       </c>
       <c r="I19" s="16" t="n">
-        <v>1394.36</v>
+        <v>1402.89</v>
       </c>
       <c r="J19" s="16" t="n">
         <v>1341.95</v>
       </c>
       <c r="K19" s="23" t="n">
-        <v>380817</v>
+        <v>402701</v>
       </c>
       <c r="L19" s="23" t="n">
         <v>601770</v>
@@ -23573,7 +23573,7 @@
         </is>
       </c>
       <c r="D20" s="11" t="n">
-        <v>291.63</v>
+        <v>283.41</v>
       </c>
       <c r="E20" s="11" t="n">
         <v>294.94</v>
@@ -23583,19 +23583,19 @@
         <v/>
       </c>
       <c r="G20" s="11" t="n">
-        <v>796.85</v>
+        <v>821.79</v>
       </c>
       <c r="H20" s="11" t="n">
         <v>717.38</v>
       </c>
       <c r="I20" s="11" t="n">
-        <v>1557.62</v>
+        <v>1566.22</v>
       </c>
       <c r="J20" s="11" t="n">
         <v>1311.04</v>
       </c>
       <c r="K20" s="23" t="n">
-        <v>645669</v>
+        <v>626338</v>
       </c>
       <c r="L20" s="23" t="n">
         <v>660679</v>
@@ -23618,7 +23618,7 @@
         </is>
       </c>
       <c r="D21" s="16" t="n">
-        <v>637.26</v>
+        <v>636.13</v>
       </c>
       <c r="E21" s="16" t="n">
         <v>656.25</v>
@@ -23628,19 +23628,19 @@
         <v/>
       </c>
       <c r="G21" s="16" t="n">
-        <v>872.92</v>
+        <v>861.1900000000001</v>
       </c>
       <c r="H21" s="16" t="n">
         <v>915.4400000000001</v>
       </c>
       <c r="I21" s="16" t="n">
-        <v>1908.6</v>
+        <v>1888.45</v>
       </c>
       <c r="J21" s="16" t="n">
         <v>1935.11</v>
       </c>
       <c r="K21" s="23" t="n">
-        <v>1045258</v>
+        <v>1060380</v>
       </c>
       <c r="L21" s="23" t="n">
         <v>1138679</v>

</xml_diff>

<commit_message>
benchmarks: Python (opt.) get_no_index tier STRESS completed (20 runs DKR)
</commit_message>
<xml_diff>
--- a/Programming_Benchmark_Report.xlsx
+++ b/Programming_Benchmark_Report.xlsx
@@ -23663,7 +23663,7 @@
         </is>
       </c>
       <c r="D22" s="11" t="n">
-        <v>3542.72</v>
+        <v>3539.25</v>
       </c>
       <c r="E22" s="11" t="n">
         <v>4131.32</v>
@@ -23673,19 +23673,19 @@
         <v/>
       </c>
       <c r="G22" s="11" t="n">
-        <v>1535.96</v>
+        <v>582.17</v>
       </c>
       <c r="H22" s="11" t="n">
         <v>1332.5</v>
       </c>
       <c r="I22" s="11" t="n">
-        <v>1962.11</v>
+        <v>1503.57</v>
       </c>
       <c r="J22" s="11" t="n">
         <v>1713.01</v>
       </c>
       <c r="K22" s="23" t="n">
-        <v>19808467</v>
+        <v>18873183</v>
       </c>
       <c r="L22" s="23" t="n">
         <v>17241200</v>
@@ -23708,7 +23708,7 @@
         </is>
       </c>
       <c r="D23" s="16" t="n">
-        <v>3561.88</v>
+        <v>3502.16</v>
       </c>
       <c r="E23" s="16" t="n">
         <v>3993.72</v>
@@ -23718,19 +23718,19 @@
         <v/>
       </c>
       <c r="G23" s="16" t="n">
-        <v>210.02</v>
+        <v>194.34</v>
       </c>
       <c r="H23" s="16" t="n">
         <v>234.02</v>
       </c>
       <c r="I23" s="16" t="n">
-        <v>1372.78</v>
+        <v>619.62</v>
       </c>
       <c r="J23" s="16" t="n">
         <v>1296.67</v>
       </c>
       <c r="K23" s="23" t="n">
-        <v>9118692</v>
+        <v>9119823</v>
       </c>
       <c r="L23" s="23" t="n">
         <v>7940192</v>
@@ -23753,29 +23753,29 @@
         </is>
       </c>
       <c r="D24" s="11" t="n">
-        <v>274.5</v>
+        <v>270.47</v>
       </c>
       <c r="E24" s="11" t="n">
         <v>275.36</v>
       </c>
-      <c r="F24" s="21">
+      <c r="F24" s="17">
         <f>IF(D24&gt;0, (E24-D24)/D24, 0)</f>
         <v/>
       </c>
       <c r="G24" s="11" t="n">
-        <v>671.6900000000001</v>
+        <v>681.1</v>
       </c>
       <c r="H24" s="11" t="n">
         <v>662.23</v>
       </c>
       <c r="I24" s="11" t="n">
-        <v>1106.35</v>
+        <v>1123.55</v>
       </c>
       <c r="J24" s="11" t="n">
         <v>942.5</v>
       </c>
       <c r="K24" s="23" t="n">
-        <v>1540211</v>
+        <v>1521417</v>
       </c>
       <c r="L24" s="23" t="n">
         <v>1547893</v>
@@ -23798,7 +23798,7 @@
         </is>
       </c>
       <c r="D25" s="16" t="n">
-        <v>616.79</v>
+        <v>615.76</v>
       </c>
       <c r="E25" s="16" t="n">
         <v>632.65</v>
@@ -23808,19 +23808,19 @@
         <v/>
       </c>
       <c r="G25" s="16" t="n">
-        <v>314.6</v>
+        <v>316.4</v>
       </c>
       <c r="H25" s="16" t="n">
         <v>303.65</v>
       </c>
       <c r="I25" s="16" t="n">
-        <v>580.1</v>
+        <v>583.02</v>
       </c>
       <c r="J25" s="16" t="n">
         <v>532.5599999999999</v>
       </c>
       <c r="K25" s="23" t="n">
-        <v>3079136</v>
+        <v>3107341</v>
       </c>
       <c r="L25" s="23" t="n">
         <v>3231051</v>

</xml_diff>